<commit_message>
Added chance of attacks missing and item sorting
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9447D3BB-8ED7-4159-8651-368EFB61CA08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAC1C04-F1AD-4181-A80F-FE4153CB4315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-25905" yWindow="990" windowWidth="21585" windowHeight="12690" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -117,9 +117,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,17 +481,17 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="1">
         <v>140</v>
       </c>
-      <c r="C3" s="4">
-        <v>62</v>
-      </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
+      <c r="C3" s="1">
+        <v>52</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
@@ -504,12 +501,12 @@
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <f>(B3+6)</f>
-        <v>146</v>
+        <f>(B3+7)</f>
+        <v>147</v>
       </c>
       <c r="C4" s="1">
         <f>(C3+4)</f>
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -525,20 +522,20 @@
         <v>3</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B68" si="0">(B4+6)</f>
-        <v>152</v>
+        <f t="shared" ref="B5:B68" si="0">(B4+7)</f>
+        <v>154</v>
       </c>
       <c r="C5" s="1">
         <f t="shared" ref="C5:C68" si="1">(C4+4)</f>
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D5" s="1">
-        <f>INT(D4*1.4)</f>
-        <v>30</v>
+        <f>INT(D4*1.35)</f>
+        <v>29</v>
       </c>
       <c r="E5" s="1">
         <f>D5+E4</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F5" s="3"/>
     </row>
@@ -549,19 +546,19 @@
       </c>
       <c r="B6" s="1">
         <f t="shared" si="0"/>
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D6" s="1">
-        <f t="shared" ref="D6:D23" si="3">INT(D5*1.4)</f>
-        <v>42</v>
+        <f t="shared" ref="D6:D23" si="3">INT(D5*1.35)</f>
+        <v>39</v>
       </c>
       <c r="E6" s="1">
         <f>D6+E5</f>
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F6" s="3"/>
     </row>
@@ -572,19 +569,19 @@
       </c>
       <c r="B7" s="1">
         <f t="shared" si="0"/>
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C7" s="1">
         <f t="shared" si="1"/>
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" si="3"/>
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="F7" s="3"/>
     </row>
@@ -595,19 +592,19 @@
       </c>
       <c r="B8" s="1">
         <f t="shared" si="0"/>
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C8" s="1">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="3"/>
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" si="4"/>
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="F8" s="3"/>
     </row>
@@ -618,19 +615,19 @@
       </c>
       <c r="B9" s="1">
         <f t="shared" si="0"/>
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C9" s="1">
-        <f t="shared" si="1"/>
-        <v>86</v>
+        <f>(C8+4)</f>
+        <v>76</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" si="3"/>
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="4"/>
-        <v>344</v>
+        <v>304</v>
       </c>
       <c r="F9" s="3"/>
     </row>
@@ -641,19 +638,19 @@
       </c>
       <c r="B10" s="1">
         <f t="shared" si="0"/>
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C10" s="1">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" si="3"/>
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="4"/>
-        <v>502</v>
+        <v>430</v>
       </c>
       <c r="F10" s="3"/>
     </row>
@@ -664,19 +661,19 @@
       </c>
       <c r="B11" s="1">
         <f t="shared" si="0"/>
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C11" s="1">
         <f t="shared" si="1"/>
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" si="3"/>
-        <v>221</v>
+        <v>170</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" si="4"/>
-        <v>723</v>
+        <v>600</v>
       </c>
       <c r="F11" s="3"/>
     </row>
@@ -687,19 +684,19 @@
       </c>
       <c r="B12" s="1">
         <f t="shared" si="0"/>
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="C12" s="1">
         <f t="shared" si="1"/>
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="3"/>
-        <v>309</v>
+        <v>229</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" si="4"/>
-        <v>1032</v>
+        <v>829</v>
       </c>
       <c r="F12" s="3"/>
     </row>
@@ -710,19 +707,19 @@
       </c>
       <c r="B13" s="1">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C13" s="1">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" si="3"/>
-        <v>432</v>
+        <v>309</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" si="4"/>
-        <v>1464</v>
+        <v>1138</v>
       </c>
       <c r="F13" s="3"/>
     </row>
@@ -733,19 +730,19 @@
       </c>
       <c r="B14" s="1">
         <f t="shared" si="0"/>
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="C14" s="1">
         <f t="shared" si="1"/>
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" si="3"/>
-        <v>604</v>
+        <v>417</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="4"/>
-        <v>2068</v>
+        <v>1555</v>
       </c>
       <c r="F14" s="3"/>
     </row>
@@ -756,19 +753,19 @@
       </c>
       <c r="B15" s="1">
         <f t="shared" si="0"/>
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C15" s="1">
         <f t="shared" si="1"/>
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" si="3"/>
-        <v>845</v>
+        <v>562</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" si="4"/>
-        <v>2913</v>
+        <v>2117</v>
       </c>
       <c r="F15" s="3"/>
     </row>
@@ -779,19 +776,19 @@
       </c>
       <c r="B16" s="1">
         <f t="shared" si="0"/>
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="C16" s="1">
         <f t="shared" si="1"/>
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" si="3"/>
-        <v>1183</v>
+        <v>758</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" si="4"/>
-        <v>4096</v>
+        <v>2875</v>
       </c>
       <c r="F16" s="3"/>
     </row>
@@ -802,19 +799,19 @@
       </c>
       <c r="B17" s="1">
         <f t="shared" si="0"/>
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="C17" s="1">
         <f t="shared" si="1"/>
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" si="3"/>
-        <v>1656</v>
+        <v>1023</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" si="4"/>
-        <v>5752</v>
+        <v>3898</v>
       </c>
       <c r="F17" s="3"/>
     </row>
@@ -825,19 +822,19 @@
       </c>
       <c r="B18" s="1">
         <f t="shared" si="0"/>
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="C18" s="1">
         <f t="shared" si="1"/>
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" si="3"/>
-        <v>2318</v>
+        <v>1381</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" si="4"/>
-        <v>8070</v>
+        <v>5279</v>
       </c>
       <c r="F18" s="3"/>
     </row>
@@ -848,19 +845,19 @@
       </c>
       <c r="B19" s="1">
         <f t="shared" si="0"/>
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="C19" s="1">
         <f t="shared" si="1"/>
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" si="3"/>
-        <v>3245</v>
+        <v>1864</v>
       </c>
       <c r="E19" s="1">
         <f t="shared" si="4"/>
-        <v>11315</v>
+        <v>7143</v>
       </c>
       <c r="F19" s="3"/>
     </row>
@@ -871,19 +868,19 @@
       </c>
       <c r="B20" s="1">
         <f t="shared" si="0"/>
-        <v>242</v>
+        <v>259</v>
       </c>
       <c r="C20" s="1">
         <f t="shared" si="1"/>
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" si="3"/>
-        <v>4543</v>
+        <v>2516</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" si="4"/>
-        <v>15858</v>
+        <v>9659</v>
       </c>
       <c r="F20" s="3"/>
     </row>
@@ -894,19 +891,19 @@
       </c>
       <c r="B21" s="1">
         <f t="shared" si="0"/>
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="C21" s="1">
         <f t="shared" si="1"/>
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" si="3"/>
-        <v>6360</v>
+        <v>3396</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
-        <v>22218</v>
+        <v>13055</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -916,19 +913,19 @@
       </c>
       <c r="B22" s="1">
         <f t="shared" si="0"/>
-        <v>254</v>
+        <v>273</v>
       </c>
       <c r="C22" s="1">
         <f t="shared" si="1"/>
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" si="3"/>
-        <v>8904</v>
+        <v>4584</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="5"/>
-        <v>31122</v>
+        <v>17639</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -938,19 +935,19 @@
       </c>
       <c r="B23" s="1">
         <f t="shared" si="0"/>
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="C23" s="1">
         <f t="shared" si="1"/>
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" si="3"/>
-        <v>12465</v>
+        <v>6188</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" ref="E23:E45" si="7">D23+E22</f>
-        <v>43587</v>
+        <v>23827</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -960,19 +957,19 @@
       </c>
       <c r="B24" s="1">
         <f t="shared" si="0"/>
-        <v>266</v>
+        <v>287</v>
       </c>
       <c r="C24" s="1">
         <f t="shared" si="1"/>
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D24" s="1">
-        <f>INT(D23*1.05)</f>
-        <v>13088</v>
+        <f>INT(D23*1.075)</f>
+        <v>6652</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" si="7"/>
-        <v>56675</v>
+        <v>30479</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -982,19 +979,19 @@
       </c>
       <c r="B25" s="1">
         <f t="shared" si="0"/>
-        <v>272</v>
+        <v>294</v>
       </c>
       <c r="C25" s="1">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D25" s="1">
-        <f t="shared" ref="D25:D53" si="8">INT(D24*1.05)</f>
-        <v>13742</v>
+        <f t="shared" ref="D25:D52" si="8">INT(D24*1.075)</f>
+        <v>7150</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" si="7"/>
-        <v>70417</v>
+        <v>37629</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1004,19 +1001,19 @@
       </c>
       <c r="B26" s="1">
         <f t="shared" si="0"/>
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C26" s="1">
         <f t="shared" si="1"/>
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" si="8"/>
-        <v>14429</v>
+        <v>7686</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" si="7"/>
-        <v>84846</v>
+        <v>45315</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1026,19 +1023,19 @@
       </c>
       <c r="B27" s="1">
         <f t="shared" si="0"/>
-        <v>284</v>
+        <v>308</v>
       </c>
       <c r="C27" s="1">
         <f t="shared" si="1"/>
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" si="8"/>
-        <v>15150</v>
+        <v>8262</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" si="7"/>
-        <v>99996</v>
+        <v>53577</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1048,19 +1045,19 @@
       </c>
       <c r="B28" s="1">
         <f t="shared" si="0"/>
-        <v>290</v>
+        <v>315</v>
       </c>
       <c r="C28" s="1">
         <f t="shared" si="1"/>
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" si="8"/>
-        <v>15907</v>
+        <v>8881</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" si="7"/>
-        <v>115903</v>
+        <v>62458</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1070,19 +1067,19 @@
       </c>
       <c r="B29" s="1">
         <f t="shared" si="0"/>
-        <v>296</v>
+        <v>322</v>
       </c>
       <c r="C29" s="1">
         <f t="shared" si="1"/>
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" si="8"/>
-        <v>16702</v>
+        <v>9547</v>
       </c>
       <c r="E29" s="1">
         <f t="shared" si="7"/>
-        <v>132605</v>
+        <v>72005</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1092,19 +1089,19 @@
       </c>
       <c r="B30" s="1">
         <f t="shared" si="0"/>
-        <v>302</v>
+        <v>329</v>
       </c>
       <c r="C30" s="1">
         <f t="shared" si="1"/>
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" si="8"/>
-        <v>17537</v>
+        <v>10263</v>
       </c>
       <c r="E30" s="1">
         <f t="shared" si="7"/>
-        <v>150142</v>
+        <v>82268</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1114,19 +1111,19 @@
       </c>
       <c r="B31" s="1">
         <f t="shared" si="0"/>
-        <v>308</v>
+        <v>336</v>
       </c>
       <c r="C31" s="1">
         <f t="shared" si="1"/>
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" si="8"/>
-        <v>18413</v>
+        <v>11032</v>
       </c>
       <c r="E31" s="1">
         <f t="shared" si="7"/>
-        <v>168555</v>
+        <v>93300</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1136,19 +1133,19 @@
       </c>
       <c r="B32" s="1">
         <f t="shared" si="0"/>
-        <v>314</v>
+        <v>343</v>
       </c>
       <c r="C32" s="1">
         <f t="shared" si="1"/>
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" si="8"/>
-        <v>19333</v>
+        <v>11859</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" si="7"/>
-        <v>187888</v>
+        <v>105159</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1158,19 +1155,19 @@
       </c>
       <c r="B33" s="1">
         <f t="shared" si="0"/>
-        <v>320</v>
+        <v>350</v>
       </c>
       <c r="C33" s="1">
         <f t="shared" si="1"/>
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" si="8"/>
-        <v>20299</v>
+        <v>12748</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" si="7"/>
-        <v>208187</v>
+        <v>117907</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1180,19 +1177,19 @@
       </c>
       <c r="B34" s="1">
         <f t="shared" si="0"/>
-        <v>326</v>
+        <v>357</v>
       </c>
       <c r="C34" s="1">
         <f t="shared" si="1"/>
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" si="8"/>
-        <v>21313</v>
+        <v>13704</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" si="7"/>
-        <v>229500</v>
+        <v>131611</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1202,19 +1199,19 @@
       </c>
       <c r="B35" s="1">
         <f t="shared" si="0"/>
-        <v>332</v>
+        <v>364</v>
       </c>
       <c r="C35" s="1">
         <f t="shared" si="1"/>
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" si="8"/>
-        <v>22378</v>
+        <v>14731</v>
       </c>
       <c r="E35" s="1">
         <f t="shared" si="7"/>
-        <v>251878</v>
+        <v>146342</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1224,19 +1221,19 @@
       </c>
       <c r="B36" s="1">
         <f t="shared" si="0"/>
-        <v>338</v>
+        <v>371</v>
       </c>
       <c r="C36" s="1">
         <f t="shared" si="1"/>
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" si="8"/>
-        <v>23496</v>
+        <v>15835</v>
       </c>
       <c r="E36" s="1">
         <f t="shared" si="7"/>
-        <v>275374</v>
+        <v>162177</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1246,19 +1243,19 @@
       </c>
       <c r="B37" s="1">
         <f t="shared" si="0"/>
-        <v>344</v>
+        <v>378</v>
       </c>
       <c r="C37" s="1">
         <f t="shared" si="1"/>
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" si="8"/>
-        <v>24670</v>
+        <v>17022</v>
       </c>
       <c r="E37" s="1">
         <f t="shared" si="7"/>
-        <v>300044</v>
+        <v>179199</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1268,19 +1265,19 @@
       </c>
       <c r="B38" s="1">
         <f t="shared" si="0"/>
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="C38" s="1">
         <f t="shared" si="1"/>
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" si="8"/>
-        <v>25903</v>
+        <v>18298</v>
       </c>
       <c r="E38" s="1">
         <f t="shared" si="7"/>
-        <v>325947</v>
+        <v>197497</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1290,19 +1287,19 @@
       </c>
       <c r="B39" s="1">
         <f t="shared" si="0"/>
-        <v>356</v>
+        <v>392</v>
       </c>
       <c r="C39" s="1">
         <f t="shared" si="1"/>
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" si="8"/>
-        <v>27198</v>
+        <v>19670</v>
       </c>
       <c r="E39" s="1">
         <f t="shared" si="7"/>
-        <v>353145</v>
+        <v>217167</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1312,19 +1309,19 @@
       </c>
       <c r="B40" s="1">
         <f t="shared" si="0"/>
-        <v>362</v>
+        <v>399</v>
       </c>
       <c r="C40" s="1">
         <f t="shared" si="1"/>
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" si="8"/>
-        <v>28557</v>
+        <v>21145</v>
       </c>
       <c r="E40" s="1">
         <f t="shared" si="7"/>
-        <v>381702</v>
+        <v>238312</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1334,19 +1331,19 @@
       </c>
       <c r="B41" s="1">
         <f t="shared" si="0"/>
-        <v>368</v>
+        <v>406</v>
       </c>
       <c r="C41" s="1">
         <f t="shared" si="1"/>
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" si="8"/>
-        <v>29984</v>
+        <v>22730</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" si="7"/>
-        <v>411686</v>
+        <v>261042</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1356,19 +1353,19 @@
       </c>
       <c r="B42" s="1">
         <f t="shared" si="0"/>
-        <v>374</v>
+        <v>413</v>
       </c>
       <c r="C42" s="1">
         <f t="shared" si="1"/>
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" si="8"/>
-        <v>31483</v>
+        <v>24434</v>
       </c>
       <c r="E42" s="1">
         <f t="shared" si="7"/>
-        <v>443169</v>
+        <v>285476</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1378,19 +1375,19 @@
       </c>
       <c r="B43" s="1">
         <f t="shared" si="0"/>
-        <v>380</v>
+        <v>420</v>
       </c>
       <c r="C43" s="1">
         <f t="shared" si="1"/>
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" si="8"/>
-        <v>33057</v>
+        <v>26266</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" si="7"/>
-        <v>476226</v>
+        <v>311742</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1400,19 +1397,19 @@
       </c>
       <c r="B44" s="1">
         <f t="shared" si="0"/>
-        <v>386</v>
+        <v>427</v>
       </c>
       <c r="C44" s="1">
         <f t="shared" si="1"/>
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" si="8"/>
-        <v>34709</v>
+        <v>28235</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" si="7"/>
-        <v>510935</v>
+        <v>339977</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1422,19 +1419,19 @@
       </c>
       <c r="B45" s="1">
         <f t="shared" si="0"/>
-        <v>392</v>
+        <v>434</v>
       </c>
       <c r="C45" s="1">
         <f t="shared" si="1"/>
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" si="8"/>
-        <v>36444</v>
+        <v>30352</v>
       </c>
       <c r="E45" s="1">
         <f t="shared" si="7"/>
-        <v>547379</v>
+        <v>370329</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1444,19 +1441,19 @@
       </c>
       <c r="B46" s="1">
         <f t="shared" si="0"/>
-        <v>398</v>
+        <v>441</v>
       </c>
       <c r="C46" s="1">
         <f t="shared" si="1"/>
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" si="8"/>
-        <v>38266</v>
+        <v>32628</v>
       </c>
       <c r="E46" s="1">
         <f t="shared" ref="E46:E88" si="10">D46+E45</f>
-        <v>585645</v>
+        <v>402957</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1466,19 +1463,19 @@
       </c>
       <c r="B47" s="1">
         <f t="shared" si="0"/>
-        <v>404</v>
+        <v>448</v>
       </c>
       <c r="C47" s="1">
         <f t="shared" si="1"/>
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D47" s="1">
         <f t="shared" si="8"/>
-        <v>40179</v>
+        <v>35075</v>
       </c>
       <c r="E47" s="1">
         <f t="shared" si="10"/>
-        <v>625824</v>
+        <v>438032</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1488,19 +1485,19 @@
       </c>
       <c r="B48" s="1">
         <f t="shared" si="0"/>
-        <v>410</v>
+        <v>455</v>
       </c>
       <c r="C48" s="1">
         <f t="shared" si="1"/>
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" si="8"/>
-        <v>42187</v>
+        <v>37705</v>
       </c>
       <c r="E48" s="1">
         <f t="shared" si="10"/>
-        <v>668011</v>
+        <v>475737</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1510,19 +1507,19 @@
       </c>
       <c r="B49" s="1">
         <f t="shared" si="0"/>
-        <v>416</v>
+        <v>462</v>
       </c>
       <c r="C49" s="1">
         <f t="shared" si="1"/>
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" si="8"/>
-        <v>44296</v>
+        <v>40532</v>
       </c>
       <c r="E49" s="1">
         <f t="shared" si="10"/>
-        <v>712307</v>
+        <v>516269</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1532,19 +1529,19 @@
       </c>
       <c r="B50" s="1">
         <f t="shared" si="0"/>
-        <v>422</v>
+        <v>469</v>
       </c>
       <c r="C50" s="1">
         <f t="shared" si="1"/>
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="D50" s="1">
         <f t="shared" si="8"/>
-        <v>46510</v>
+        <v>43571</v>
       </c>
       <c r="E50" s="1">
         <f t="shared" si="10"/>
-        <v>758817</v>
+        <v>559840</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -1554,19 +1551,19 @@
       </c>
       <c r="B51" s="1">
         <f t="shared" si="0"/>
-        <v>428</v>
+        <v>476</v>
       </c>
       <c r="C51" s="1">
         <f t="shared" si="1"/>
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" si="8"/>
-        <v>48835</v>
+        <v>46838</v>
       </c>
       <c r="E51" s="1">
         <f t="shared" si="10"/>
-        <v>807652</v>
+        <v>606678</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1576,19 +1573,19 @@
       </c>
       <c r="B52" s="1">
         <f t="shared" si="0"/>
-        <v>434</v>
+        <v>483</v>
       </c>
       <c r="C52" s="1">
         <f t="shared" si="1"/>
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D52" s="1">
         <f t="shared" si="8"/>
-        <v>51276</v>
+        <v>50350</v>
       </c>
       <c r="E52" s="1">
         <f t="shared" si="10"/>
-        <v>858928</v>
+        <v>657028</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -1598,19 +1595,19 @@
       </c>
       <c r="B53" s="1">
         <f t="shared" si="0"/>
-        <v>440</v>
+        <v>490</v>
       </c>
       <c r="C53" s="1">
         <f t="shared" si="1"/>
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D53" s="1">
-        <f t="shared" si="8"/>
-        <v>53839</v>
+        <f t="shared" ref="D25:D53" si="11">INT(D52*1.05)</f>
+        <v>52867</v>
       </c>
       <c r="E53" s="1">
         <f t="shared" si="10"/>
-        <v>912767</v>
+        <v>709895</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -1620,19 +1617,19 @@
       </c>
       <c r="B54" s="1">
         <f t="shared" si="0"/>
-        <v>446</v>
+        <v>497</v>
       </c>
       <c r="C54" s="1">
         <f t="shared" si="1"/>
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D54" s="1">
         <f>INT(D53*1.025)</f>
-        <v>55184</v>
+        <v>54188</v>
       </c>
       <c r="E54" s="1">
         <f t="shared" si="10"/>
-        <v>967951</v>
+        <v>764083</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1642,19 +1639,19 @@
       </c>
       <c r="B55" s="1">
         <f t="shared" si="0"/>
-        <v>452</v>
+        <v>504</v>
       </c>
       <c r="C55" s="1">
         <f t="shared" si="1"/>
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="D55" s="1">
-        <f t="shared" ref="D55:D101" si="11">INT(D54*1.025)</f>
-        <v>56563</v>
+        <f t="shared" ref="D55:D101" si="12">INT(D54*1.025)</f>
+        <v>55542</v>
       </c>
       <c r="E55" s="1">
         <f t="shared" si="10"/>
-        <v>1024514</v>
+        <v>819625</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -1664,19 +1661,19 @@
       </c>
       <c r="B56" s="1">
         <f t="shared" si="0"/>
-        <v>458</v>
+        <v>511</v>
       </c>
       <c r="C56" s="1">
         <f t="shared" si="1"/>
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="D56" s="1">
-        <f t="shared" si="11"/>
-        <v>57977</v>
+        <f t="shared" si="12"/>
+        <v>56930</v>
       </c>
       <c r="E56" s="1">
         <f t="shared" si="10"/>
-        <v>1082491</v>
+        <v>876555</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -1686,19 +1683,19 @@
       </c>
       <c r="B57" s="1">
         <f t="shared" si="0"/>
-        <v>464</v>
+        <v>518</v>
       </c>
       <c r="C57" s="1">
         <f t="shared" si="1"/>
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="D57" s="1">
-        <f t="shared" si="11"/>
-        <v>59426</v>
+        <f t="shared" si="12"/>
+        <v>58353</v>
       </c>
       <c r="E57" s="1">
         <f t="shared" si="10"/>
-        <v>1141917</v>
+        <v>934908</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -1708,19 +1705,19 @@
       </c>
       <c r="B58" s="1">
         <f t="shared" si="0"/>
-        <v>470</v>
+        <v>525</v>
       </c>
       <c r="C58" s="1">
         <f t="shared" si="1"/>
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="D58" s="1">
-        <f t="shared" si="11"/>
-        <v>60911</v>
+        <f t="shared" si="12"/>
+        <v>59811</v>
       </c>
       <c r="E58" s="1">
         <f t="shared" si="10"/>
-        <v>1202828</v>
+        <v>994719</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -1730,19 +1727,19 @@
       </c>
       <c r="B59" s="1">
         <f t="shared" si="0"/>
-        <v>476</v>
+        <v>532</v>
       </c>
       <c r="C59" s="1">
         <f t="shared" si="1"/>
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="D59" s="1">
-        <f t="shared" si="11"/>
-        <v>62433</v>
+        <f t="shared" si="12"/>
+        <v>61306</v>
       </c>
       <c r="E59" s="1">
         <f t="shared" si="10"/>
-        <v>1265261</v>
+        <v>1056025</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -1752,19 +1749,19 @@
       </c>
       <c r="B60" s="1">
         <f t="shared" si="0"/>
-        <v>482</v>
+        <v>539</v>
       </c>
       <c r="C60" s="1">
         <f t="shared" si="1"/>
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="11"/>
-        <v>63993</v>
+        <f t="shared" si="12"/>
+        <v>62838</v>
       </c>
       <c r="E60" s="1">
         <f t="shared" si="10"/>
-        <v>1329254</v>
+        <v>1118863</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1774,19 +1771,19 @@
       </c>
       <c r="B61" s="1">
         <f t="shared" si="0"/>
-        <v>488</v>
+        <v>546</v>
       </c>
       <c r="C61" s="1">
         <f t="shared" si="1"/>
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="11"/>
-        <v>65592</v>
+        <f t="shared" si="12"/>
+        <v>64408</v>
       </c>
       <c r="E61" s="1">
         <f t="shared" si="10"/>
-        <v>1394846</v>
+        <v>1183271</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1796,19 +1793,19 @@
       </c>
       <c r="B62" s="1">
         <f t="shared" si="0"/>
-        <v>494</v>
+        <v>553</v>
       </c>
       <c r="C62" s="1">
         <f t="shared" si="1"/>
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="D62" s="1">
-        <f t="shared" si="11"/>
-        <v>67231</v>
+        <f t="shared" si="12"/>
+        <v>66018</v>
       </c>
       <c r="E62" s="1">
         <f t="shared" si="10"/>
-        <v>1462077</v>
+        <v>1249289</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1818,19 +1815,19 @@
       </c>
       <c r="B63" s="1">
         <f t="shared" si="0"/>
-        <v>500</v>
+        <v>560</v>
       </c>
       <c r="C63" s="1">
         <f t="shared" si="1"/>
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="D63" s="1">
-        <f t="shared" si="11"/>
-        <v>68911</v>
+        <f t="shared" si="12"/>
+        <v>67668</v>
       </c>
       <c r="E63" s="1">
         <f t="shared" si="10"/>
-        <v>1530988</v>
+        <v>1316957</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -1840,481 +1837,481 @@
       </c>
       <c r="B64" s="1">
         <f t="shared" si="0"/>
-        <v>506</v>
+        <v>567</v>
       </c>
       <c r="C64" s="1">
         <f t="shared" si="1"/>
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="D64" s="1">
-        <f t="shared" si="11"/>
-        <v>70633</v>
+        <f t="shared" si="12"/>
+        <v>69359</v>
       </c>
       <c r="E64" s="1">
         <f t="shared" si="10"/>
-        <v>1601621</v>
+        <v>1386316</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <f t="shared" ref="A65:A85" si="12">A64+1</f>
+        <f t="shared" ref="A65:A85" si="13">A64+1</f>
         <v>63</v>
       </c>
       <c r="B65" s="1">
         <f t="shared" si="0"/>
-        <v>512</v>
+        <v>574</v>
       </c>
       <c r="C65" s="1">
         <f t="shared" si="1"/>
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="D65" s="1">
-        <f t="shared" si="11"/>
-        <v>72398</v>
+        <f t="shared" si="12"/>
+        <v>71092</v>
       </c>
       <c r="E65" s="1">
         <f t="shared" si="10"/>
-        <v>1674019</v>
+        <v>1457408</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>64</v>
       </c>
       <c r="B66" s="1">
         <f t="shared" si="0"/>
-        <v>518</v>
+        <v>581</v>
       </c>
       <c r="C66" s="1">
         <f t="shared" si="1"/>
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="D66" s="1">
-        <f t="shared" si="11"/>
-        <v>74207</v>
+        <f t="shared" si="12"/>
+        <v>72869</v>
       </c>
       <c r="E66" s="1">
         <f t="shared" si="10"/>
-        <v>1748226</v>
+        <v>1530277</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>65</v>
       </c>
       <c r="B67" s="1">
         <f t="shared" si="0"/>
-        <v>524</v>
+        <v>588</v>
       </c>
       <c r="C67" s="1">
         <f t="shared" si="1"/>
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="D67" s="1">
-        <f t="shared" si="11"/>
-        <v>76062</v>
+        <f t="shared" si="12"/>
+        <v>74690</v>
       </c>
       <c r="E67" s="1">
         <f t="shared" si="10"/>
-        <v>1824288</v>
+        <v>1604967</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>66</v>
       </c>
       <c r="B68" s="1">
         <f t="shared" si="0"/>
-        <v>530</v>
+        <v>595</v>
       </c>
       <c r="C68" s="1">
         <f t="shared" si="1"/>
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="D68" s="1">
-        <f t="shared" si="11"/>
-        <v>77963</v>
+        <f t="shared" si="12"/>
+        <v>76557</v>
       </c>
       <c r="E68" s="1">
         <f t="shared" si="10"/>
-        <v>1902251</v>
+        <v>1681524</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>67</v>
       </c>
       <c r="B69" s="1">
-        <f t="shared" ref="B69:B101" si="13">(B68+6)</f>
-        <v>536</v>
+        <f t="shared" ref="B69:B101" si="14">(B68+7)</f>
+        <v>602</v>
       </c>
       <c r="C69" s="1">
-        <f t="shared" ref="C69:C101" si="14">(C68+4)</f>
-        <v>326</v>
+        <f t="shared" ref="C69:C101" si="15">(C68+4)</f>
+        <v>316</v>
       </c>
       <c r="D69" s="1">
-        <f t="shared" si="11"/>
-        <v>79912</v>
+        <f t="shared" si="12"/>
+        <v>78470</v>
       </c>
       <c r="E69" s="1">
         <f t="shared" si="10"/>
-        <v>1982163</v>
+        <v>1759994</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>68</v>
       </c>
       <c r="B70" s="1">
-        <f t="shared" si="13"/>
-        <v>542</v>
+        <f t="shared" si="14"/>
+        <v>609</v>
       </c>
       <c r="C70" s="1">
-        <f t="shared" si="14"/>
-        <v>330</v>
+        <f t="shared" si="15"/>
+        <v>320</v>
       </c>
       <c r="D70" s="1">
-        <f t="shared" si="11"/>
-        <v>81909</v>
+        <f t="shared" si="12"/>
+        <v>80431</v>
       </c>
       <c r="E70" s="1">
         <f t="shared" si="10"/>
-        <v>2064072</v>
+        <v>1840425</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>69</v>
       </c>
       <c r="B71" s="1">
-        <f t="shared" si="13"/>
-        <v>548</v>
+        <f t="shared" si="14"/>
+        <v>616</v>
       </c>
       <c r="C71" s="1">
-        <f t="shared" si="14"/>
-        <v>334</v>
+        <f t="shared" si="15"/>
+        <v>324</v>
       </c>
       <c r="D71" s="1">
-        <f t="shared" si="11"/>
-        <v>83956</v>
+        <f t="shared" si="12"/>
+        <v>82441</v>
       </c>
       <c r="E71" s="1">
         <f t="shared" si="10"/>
-        <v>2148028</v>
+        <v>1922866</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>70</v>
       </c>
       <c r="B72" s="1">
-        <f t="shared" si="13"/>
-        <v>554</v>
+        <f t="shared" si="14"/>
+        <v>623</v>
       </c>
       <c r="C72" s="1">
-        <f t="shared" si="14"/>
-        <v>338</v>
+        <f t="shared" si="15"/>
+        <v>328</v>
       </c>
       <c r="D72" s="1">
-        <f t="shared" si="11"/>
-        <v>86054</v>
+        <f t="shared" si="12"/>
+        <v>84502</v>
       </c>
       <c r="E72" s="1">
         <f t="shared" si="10"/>
-        <v>2234082</v>
+        <v>2007368</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>71</v>
       </c>
       <c r="B73" s="1">
-        <f t="shared" si="13"/>
-        <v>560</v>
+        <f t="shared" si="14"/>
+        <v>630</v>
       </c>
       <c r="C73" s="1">
-        <f t="shared" si="14"/>
-        <v>342</v>
+        <f t="shared" si="15"/>
+        <v>332</v>
       </c>
       <c r="D73" s="1">
-        <f t="shared" si="11"/>
-        <v>88205</v>
+        <f t="shared" si="12"/>
+        <v>86614</v>
       </c>
       <c r="E73" s="1">
         <f t="shared" si="10"/>
-        <v>2322287</v>
+        <v>2093982</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>72</v>
       </c>
       <c r="B74" s="1">
-        <f t="shared" si="13"/>
-        <v>566</v>
+        <f t="shared" si="14"/>
+        <v>637</v>
       </c>
       <c r="C74" s="1">
-        <f t="shared" si="14"/>
-        <v>346</v>
+        <f t="shared" si="15"/>
+        <v>336</v>
       </c>
       <c r="D74" s="1">
-        <f t="shared" si="11"/>
-        <v>90410</v>
+        <f t="shared" si="12"/>
+        <v>88779</v>
       </c>
       <c r="E74" s="1">
         <f t="shared" si="10"/>
-        <v>2412697</v>
+        <v>2182761</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>73</v>
       </c>
       <c r="B75" s="1">
-        <f t="shared" si="13"/>
-        <v>572</v>
+        <f t="shared" si="14"/>
+        <v>644</v>
       </c>
       <c r="C75" s="1">
-        <f t="shared" si="14"/>
-        <v>350</v>
+        <f t="shared" si="15"/>
+        <v>340</v>
       </c>
       <c r="D75" s="1">
-        <f t="shared" si="11"/>
-        <v>92670</v>
+        <f t="shared" si="12"/>
+        <v>90998</v>
       </c>
       <c r="E75" s="1">
         <f t="shared" si="10"/>
-        <v>2505367</v>
+        <v>2273759</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>74</v>
       </c>
       <c r="B76" s="1">
-        <f t="shared" si="13"/>
-        <v>578</v>
+        <f t="shared" si="14"/>
+        <v>651</v>
       </c>
       <c r="C76" s="1">
-        <f t="shared" si="14"/>
-        <v>354</v>
+        <f t="shared" si="15"/>
+        <v>344</v>
       </c>
       <c r="D76" s="1">
-        <f t="shared" si="11"/>
-        <v>94986</v>
+        <f t="shared" si="12"/>
+        <v>93272</v>
       </c>
       <c r="E76" s="1">
         <f t="shared" si="10"/>
-        <v>2600353</v>
+        <v>2367031</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>75</v>
       </c>
       <c r="B77" s="1">
-        <f t="shared" si="13"/>
-        <v>584</v>
+        <f t="shared" si="14"/>
+        <v>658</v>
       </c>
       <c r="C77" s="1">
-        <f t="shared" si="14"/>
-        <v>358</v>
+        <f t="shared" si="15"/>
+        <v>348</v>
       </c>
       <c r="D77" s="1">
-        <f t="shared" si="11"/>
-        <v>97360</v>
+        <f t="shared" si="12"/>
+        <v>95603</v>
       </c>
       <c r="E77" s="1">
         <f t="shared" si="10"/>
-        <v>2697713</v>
+        <v>2462634</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>76</v>
       </c>
       <c r="B78" s="1">
-        <f t="shared" si="13"/>
-        <v>590</v>
+        <f t="shared" si="14"/>
+        <v>665</v>
       </c>
       <c r="C78" s="1">
-        <f t="shared" si="14"/>
-        <v>362</v>
+        <f t="shared" si="15"/>
+        <v>352</v>
       </c>
       <c r="D78" s="1">
-        <f t="shared" si="11"/>
-        <v>99794</v>
+        <f t="shared" si="12"/>
+        <v>97993</v>
       </c>
       <c r="E78" s="1">
         <f t="shared" si="10"/>
-        <v>2797507</v>
+        <v>2560627</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>77</v>
       </c>
       <c r="B79" s="1">
-        <f t="shared" si="13"/>
-        <v>596</v>
+        <f t="shared" si="14"/>
+        <v>672</v>
       </c>
       <c r="C79" s="1">
-        <f t="shared" si="14"/>
-        <v>366</v>
+        <f t="shared" si="15"/>
+        <v>356</v>
       </c>
       <c r="D79" s="1">
-        <f t="shared" si="11"/>
-        <v>102288</v>
+        <f t="shared" si="12"/>
+        <v>100442</v>
       </c>
       <c r="E79" s="1">
         <f t="shared" si="10"/>
-        <v>2899795</v>
+        <v>2661069</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>78</v>
       </c>
       <c r="B80" s="1">
-        <f t="shared" si="13"/>
-        <v>602</v>
+        <f t="shared" si="14"/>
+        <v>679</v>
       </c>
       <c r="C80" s="1">
-        <f t="shared" si="14"/>
-        <v>370</v>
+        <f t="shared" si="15"/>
+        <v>360</v>
       </c>
       <c r="D80" s="1">
-        <f t="shared" si="11"/>
-        <v>104845</v>
+        <f t="shared" si="12"/>
+        <v>102953</v>
       </c>
       <c r="E80" s="1">
         <f t="shared" si="10"/>
-        <v>3004640</v>
+        <v>2764022</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>79</v>
       </c>
       <c r="B81" s="1">
-        <f t="shared" si="13"/>
-        <v>608</v>
+        <f t="shared" si="14"/>
+        <v>686</v>
       </c>
       <c r="C81" s="1">
-        <f t="shared" si="14"/>
-        <v>374</v>
+        <f t="shared" si="15"/>
+        <v>364</v>
       </c>
       <c r="D81" s="1">
-        <f t="shared" si="11"/>
-        <v>107466</v>
+        <f t="shared" si="12"/>
+        <v>105526</v>
       </c>
       <c r="E81" s="1">
         <f t="shared" si="10"/>
-        <v>3112106</v>
+        <v>2869548</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>80</v>
       </c>
       <c r="B82" s="1">
-        <f t="shared" si="13"/>
-        <v>614</v>
+        <f t="shared" si="14"/>
+        <v>693</v>
       </c>
       <c r="C82" s="1">
-        <f t="shared" si="14"/>
-        <v>378</v>
+        <f t="shared" si="15"/>
+        <v>368</v>
       </c>
       <c r="D82" s="1">
-        <f t="shared" si="11"/>
-        <v>110152</v>
+        <f t="shared" si="12"/>
+        <v>108164</v>
       </c>
       <c r="E82" s="1">
         <f t="shared" si="10"/>
-        <v>3222258</v>
+        <v>2977712</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>81</v>
       </c>
       <c r="B83" s="1">
-        <f t="shared" si="13"/>
-        <v>620</v>
+        <f t="shared" si="14"/>
+        <v>700</v>
       </c>
       <c r="C83" s="1">
-        <f t="shared" si="14"/>
-        <v>382</v>
+        <f t="shared" si="15"/>
+        <v>372</v>
       </c>
       <c r="D83" s="1">
-        <f t="shared" si="11"/>
-        <v>112905</v>
+        <f t="shared" si="12"/>
+        <v>110868</v>
       </c>
       <c r="E83" s="1">
         <f t="shared" si="10"/>
-        <v>3335163</v>
+        <v>3088580</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>82</v>
       </c>
       <c r="B84" s="1">
-        <f t="shared" si="13"/>
-        <v>626</v>
+        <f t="shared" si="14"/>
+        <v>707</v>
       </c>
       <c r="C84" s="1">
-        <f t="shared" si="14"/>
-        <v>386</v>
+        <f t="shared" si="15"/>
+        <v>376</v>
       </c>
       <c r="D84" s="1">
-        <f t="shared" si="11"/>
-        <v>115727</v>
+        <f t="shared" si="12"/>
+        <v>113639</v>
       </c>
       <c r="E84" s="1">
         <f t="shared" si="10"/>
-        <v>3450890</v>
+        <v>3202219</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>83</v>
       </c>
       <c r="B85" s="1">
-        <f t="shared" si="13"/>
-        <v>632</v>
+        <f t="shared" si="14"/>
+        <v>714</v>
       </c>
       <c r="C85" s="1">
-        <f t="shared" si="14"/>
-        <v>390</v>
+        <f t="shared" si="15"/>
+        <v>380</v>
       </c>
       <c r="D85" s="1">
-        <f t="shared" si="11"/>
-        <v>118620</v>
+        <f t="shared" si="12"/>
+        <v>116479</v>
       </c>
       <c r="E85" s="1">
         <f t="shared" si="10"/>
-        <v>3569510</v>
+        <v>3318698</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2323,20 +2320,20 @@
         <v>84</v>
       </c>
       <c r="B86" s="1">
-        <f t="shared" si="13"/>
-        <v>638</v>
+        <f t="shared" si="14"/>
+        <v>721</v>
       </c>
       <c r="C86" s="1">
-        <f t="shared" si="14"/>
-        <v>394</v>
+        <f t="shared" si="15"/>
+        <v>384</v>
       </c>
       <c r="D86" s="1">
-        <f t="shared" si="11"/>
-        <v>121585</v>
+        <f t="shared" si="12"/>
+        <v>119390</v>
       </c>
       <c r="E86" s="1">
         <f t="shared" si="10"/>
-        <v>3691095</v>
+        <v>3438088</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2345,328 +2342,328 @@
         <v>85</v>
       </c>
       <c r="B87" s="1">
-        <f t="shared" si="13"/>
-        <v>644</v>
+        <f t="shared" si="14"/>
+        <v>728</v>
       </c>
       <c r="C87" s="1">
-        <f t="shared" si="14"/>
-        <v>398</v>
+        <f t="shared" si="15"/>
+        <v>388</v>
       </c>
       <c r="D87" s="1">
-        <f t="shared" si="11"/>
-        <v>124624</v>
+        <f t="shared" si="12"/>
+        <v>122374</v>
       </c>
       <c r="E87" s="1">
         <f t="shared" si="10"/>
-        <v>3815719</v>
+        <v>3560462</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <f t="shared" ref="A88:A101" si="15">A87+1</f>
+        <f t="shared" ref="A88:A101" si="16">A87+1</f>
         <v>86</v>
       </c>
       <c r="B88" s="1">
-        <f t="shared" si="13"/>
-        <v>650</v>
+        <f t="shared" si="14"/>
+        <v>735</v>
       </c>
       <c r="C88" s="1">
-        <f t="shared" si="14"/>
-        <v>402</v>
+        <f t="shared" si="15"/>
+        <v>392</v>
       </c>
       <c r="D88" s="1">
-        <f t="shared" si="11"/>
-        <v>127739</v>
+        <f t="shared" si="12"/>
+        <v>125433</v>
       </c>
       <c r="E88" s="1">
         <f t="shared" si="10"/>
-        <v>3943458</v>
+        <v>3685895</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>87</v>
       </c>
       <c r="B89" s="1">
-        <f t="shared" si="13"/>
-        <v>656</v>
+        <f t="shared" si="14"/>
+        <v>742</v>
       </c>
       <c r="C89" s="1">
-        <f t="shared" si="14"/>
-        <v>406</v>
+        <f t="shared" si="15"/>
+        <v>396</v>
       </c>
       <c r="D89" s="1">
-        <f t="shared" si="11"/>
-        <v>130932</v>
+        <f t="shared" si="12"/>
+        <v>128568</v>
       </c>
       <c r="E89" s="1">
-        <f t="shared" ref="E89:E101" si="16">D89+E88</f>
-        <v>4074390</v>
+        <f t="shared" ref="E89:E101" si="17">D89+E88</f>
+        <v>3814463</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>88</v>
       </c>
       <c r="B90" s="1">
-        <f t="shared" si="13"/>
-        <v>662</v>
+        <f t="shared" si="14"/>
+        <v>749</v>
       </c>
       <c r="C90" s="1">
-        <f t="shared" si="14"/>
-        <v>410</v>
+        <f t="shared" si="15"/>
+        <v>400</v>
       </c>
       <c r="D90" s="1">
-        <f t="shared" si="11"/>
-        <v>134205</v>
+        <f t="shared" si="12"/>
+        <v>131782</v>
       </c>
       <c r="E90" s="1">
-        <f t="shared" si="16"/>
-        <v>4208595</v>
+        <f t="shared" si="17"/>
+        <v>3946245</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>89</v>
       </c>
       <c r="B91" s="1">
-        <f t="shared" si="13"/>
-        <v>668</v>
+        <f t="shared" si="14"/>
+        <v>756</v>
       </c>
       <c r="C91" s="1">
-        <f t="shared" si="14"/>
-        <v>414</v>
+        <f t="shared" si="15"/>
+        <v>404</v>
       </c>
       <c r="D91" s="1">
-        <f t="shared" si="11"/>
-        <v>137560</v>
+        <f t="shared" si="12"/>
+        <v>135076</v>
       </c>
       <c r="E91" s="1">
-        <f t="shared" si="16"/>
-        <v>4346155</v>
+        <f t="shared" si="17"/>
+        <v>4081321</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>90</v>
       </c>
       <c r="B92" s="1">
-        <f t="shared" si="13"/>
-        <v>674</v>
+        <f t="shared" si="14"/>
+        <v>763</v>
       </c>
       <c r="C92" s="1">
-        <f t="shared" si="14"/>
-        <v>418</v>
+        <f t="shared" si="15"/>
+        <v>408</v>
       </c>
       <c r="D92" s="1">
-        <f t="shared" si="11"/>
-        <v>140999</v>
+        <f t="shared" si="12"/>
+        <v>138452</v>
       </c>
       <c r="E92" s="1">
-        <f t="shared" si="16"/>
-        <v>4487154</v>
+        <f t="shared" si="17"/>
+        <v>4219773</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>91</v>
       </c>
       <c r="B93" s="1">
-        <f t="shared" si="13"/>
-        <v>680</v>
+        <f t="shared" si="14"/>
+        <v>770</v>
       </c>
       <c r="C93" s="1">
-        <f t="shared" si="14"/>
-        <v>422</v>
+        <f t="shared" si="15"/>
+        <v>412</v>
       </c>
       <c r="D93" s="1">
-        <f t="shared" si="11"/>
-        <v>144523</v>
+        <f t="shared" si="12"/>
+        <v>141913</v>
       </c>
       <c r="E93" s="1">
-        <f t="shared" si="16"/>
-        <v>4631677</v>
+        <f t="shared" si="17"/>
+        <v>4361686</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>92</v>
       </c>
       <c r="B94" s="1">
-        <f t="shared" si="13"/>
-        <v>686</v>
+        <f t="shared" si="14"/>
+        <v>777</v>
       </c>
       <c r="C94" s="1">
-        <f t="shared" si="14"/>
-        <v>426</v>
+        <f t="shared" si="15"/>
+        <v>416</v>
       </c>
       <c r="D94" s="1">
-        <f t="shared" si="11"/>
-        <v>148136</v>
+        <f t="shared" si="12"/>
+        <v>145460</v>
       </c>
       <c r="E94" s="1">
-        <f t="shared" si="16"/>
-        <v>4779813</v>
+        <f t="shared" si="17"/>
+        <v>4507146</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>93</v>
       </c>
       <c r="B95" s="1">
-        <f t="shared" si="13"/>
-        <v>692</v>
+        <f t="shared" si="14"/>
+        <v>784</v>
       </c>
       <c r="C95" s="1">
-        <f t="shared" si="14"/>
-        <v>430</v>
+        <f t="shared" si="15"/>
+        <v>420</v>
       </c>
       <c r="D95" s="1">
-        <f t="shared" si="11"/>
-        <v>151839</v>
+        <f t="shared" si="12"/>
+        <v>149096</v>
       </c>
       <c r="E95" s="1">
-        <f t="shared" si="16"/>
-        <v>4931652</v>
+        <f t="shared" si="17"/>
+        <v>4656242</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>94</v>
       </c>
       <c r="B96" s="1">
-        <f t="shared" si="13"/>
-        <v>698</v>
+        <f t="shared" si="14"/>
+        <v>791</v>
       </c>
       <c r="C96" s="1">
-        <f t="shared" si="14"/>
-        <v>434</v>
+        <f t="shared" si="15"/>
+        <v>424</v>
       </c>
       <c r="D96" s="1">
-        <f t="shared" si="11"/>
-        <v>155634</v>
+        <f t="shared" si="12"/>
+        <v>152823</v>
       </c>
       <c r="E96" s="1">
-        <f t="shared" si="16"/>
-        <v>5087286</v>
+        <f t="shared" si="17"/>
+        <v>4809065</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>95</v>
       </c>
       <c r="B97" s="1">
-        <f t="shared" si="13"/>
-        <v>704</v>
+        <f t="shared" si="14"/>
+        <v>798</v>
       </c>
       <c r="C97" s="1">
-        <f t="shared" si="14"/>
-        <v>438</v>
+        <f t="shared" si="15"/>
+        <v>428</v>
       </c>
       <c r="D97" s="1">
-        <f t="shared" si="11"/>
-        <v>159524</v>
+        <f t="shared" si="12"/>
+        <v>156643</v>
       </c>
       <c r="E97" s="1">
-        <f t="shared" si="16"/>
-        <v>5246810</v>
+        <f t="shared" si="17"/>
+        <v>4965708</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>96</v>
       </c>
       <c r="B98" s="1">
-        <f t="shared" si="13"/>
-        <v>710</v>
+        <f t="shared" si="14"/>
+        <v>805</v>
       </c>
       <c r="C98" s="1">
-        <f t="shared" si="14"/>
-        <v>442</v>
+        <f t="shared" si="15"/>
+        <v>432</v>
       </c>
       <c r="D98" s="1">
-        <f t="shared" si="11"/>
-        <v>163512</v>
+        <f t="shared" si="12"/>
+        <v>160559</v>
       </c>
       <c r="E98" s="1">
-        <f t="shared" si="16"/>
-        <v>5410322</v>
+        <f t="shared" si="17"/>
+        <v>5126267</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>97</v>
       </c>
       <c r="B99" s="1">
-        <f t="shared" si="13"/>
-        <v>716</v>
+        <f t="shared" si="14"/>
+        <v>812</v>
       </c>
       <c r="C99" s="1">
-        <f t="shared" si="14"/>
-        <v>446</v>
+        <f t="shared" si="15"/>
+        <v>436</v>
       </c>
       <c r="D99" s="1">
-        <f t="shared" si="11"/>
-        <v>167599</v>
+        <f t="shared" si="12"/>
+        <v>164572</v>
       </c>
       <c r="E99" s="1">
-        <f t="shared" si="16"/>
-        <v>5577921</v>
+        <f t="shared" si="17"/>
+        <v>5290839</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>98</v>
       </c>
       <c r="B100" s="1">
-        <f t="shared" si="13"/>
-        <v>722</v>
+        <f t="shared" si="14"/>
+        <v>819</v>
       </c>
       <c r="C100" s="1">
-        <f t="shared" si="14"/>
-        <v>450</v>
+        <f t="shared" si="15"/>
+        <v>440</v>
       </c>
       <c r="D100" s="1">
-        <f t="shared" si="11"/>
-        <v>171788</v>
+        <f t="shared" si="12"/>
+        <v>168686</v>
       </c>
       <c r="E100" s="1">
-        <f t="shared" si="16"/>
-        <v>5749709</v>
+        <f t="shared" si="17"/>
+        <v>5459525</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>99</v>
       </c>
       <c r="B101" s="1">
-        <f t="shared" si="13"/>
-        <v>728</v>
+        <f t="shared" si="14"/>
+        <v>826</v>
       </c>
       <c r="C101" s="1">
-        <f t="shared" si="14"/>
-        <v>454</v>
+        <f t="shared" si="15"/>
+        <v>444</v>
       </c>
       <c r="D101" s="1">
-        <f t="shared" si="11"/>
-        <v>176082</v>
+        <f t="shared" si="12"/>
+        <v>172903</v>
       </c>
       <c r="E101" s="1">
-        <f t="shared" si="16"/>
-        <v>5925791</v>
+        <f t="shared" si="17"/>
+        <v>5632428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Animated EXP after battle
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAC1C04-F1AD-4181-A80F-FE4153CB4315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05872086-26F9-4CEB-B8B4-B3A008DC6A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25905" yWindow="990" windowWidth="21585" windowHeight="12690" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
@@ -1602,12 +1602,12 @@
         <v>252</v>
       </c>
       <c r="D53" s="1">
-        <f t="shared" ref="D25:D53" si="11">INT(D52*1.05)</f>
-        <v>52867</v>
+        <f>INT(D52*1.03)</f>
+        <v>51860</v>
       </c>
       <c r="E53" s="1">
         <f t="shared" si="10"/>
-        <v>709895</v>
+        <v>708888</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -1624,12 +1624,12 @@
         <v>256</v>
       </c>
       <c r="D54" s="1">
-        <f>INT(D53*1.025)</f>
-        <v>54188</v>
+        <f t="shared" ref="D54:D101" si="11">INT(D53*1.03)</f>
+        <v>53415</v>
       </c>
       <c r="E54" s="1">
         <f t="shared" si="10"/>
-        <v>764083</v>
+        <v>762303</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1646,12 +1646,12 @@
         <v>260</v>
       </c>
       <c r="D55" s="1">
-        <f t="shared" ref="D55:D101" si="12">INT(D54*1.025)</f>
-        <v>55542</v>
+        <f t="shared" si="11"/>
+        <v>55017</v>
       </c>
       <c r="E55" s="1">
         <f t="shared" si="10"/>
-        <v>819625</v>
+        <v>817320</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -1668,12 +1668,12 @@
         <v>264</v>
       </c>
       <c r="D56" s="1">
-        <f t="shared" si="12"/>
-        <v>56930</v>
+        <f t="shared" si="11"/>
+        <v>56667</v>
       </c>
       <c r="E56" s="1">
         <f t="shared" si="10"/>
-        <v>876555</v>
+        <v>873987</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -1690,12 +1690,12 @@
         <v>268</v>
       </c>
       <c r="D57" s="1">
-        <f t="shared" si="12"/>
-        <v>58353</v>
+        <f t="shared" si="11"/>
+        <v>58367</v>
       </c>
       <c r="E57" s="1">
         <f t="shared" si="10"/>
-        <v>934908</v>
+        <v>932354</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -1712,12 +1712,12 @@
         <v>272</v>
       </c>
       <c r="D58" s="1">
-        <f t="shared" si="12"/>
-        <v>59811</v>
+        <f t="shared" si="11"/>
+        <v>60118</v>
       </c>
       <c r="E58" s="1">
         <f t="shared" si="10"/>
-        <v>994719</v>
+        <v>992472</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -1734,12 +1734,12 @@
         <v>276</v>
       </c>
       <c r="D59" s="1">
-        <f t="shared" si="12"/>
-        <v>61306</v>
+        <f t="shared" si="11"/>
+        <v>61921</v>
       </c>
       <c r="E59" s="1">
         <f t="shared" si="10"/>
-        <v>1056025</v>
+        <v>1054393</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -1756,12 +1756,12 @@
         <v>280</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="12"/>
-        <v>62838</v>
+        <f t="shared" si="11"/>
+        <v>63778</v>
       </c>
       <c r="E60" s="1">
         <f t="shared" si="10"/>
-        <v>1118863</v>
+        <v>1118171</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1778,12 +1778,12 @@
         <v>284</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="12"/>
-        <v>64408</v>
+        <f t="shared" si="11"/>
+        <v>65691</v>
       </c>
       <c r="E61" s="1">
         <f t="shared" si="10"/>
-        <v>1183271</v>
+        <v>1183862</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1800,12 +1800,12 @@
         <v>288</v>
       </c>
       <c r="D62" s="1">
-        <f t="shared" si="12"/>
-        <v>66018</v>
+        <f t="shared" si="11"/>
+        <v>67661</v>
       </c>
       <c r="E62" s="1">
         <f t="shared" si="10"/>
-        <v>1249289</v>
+        <v>1251523</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1822,12 +1822,12 @@
         <v>292</v>
       </c>
       <c r="D63" s="1">
-        <f t="shared" si="12"/>
-        <v>67668</v>
+        <f t="shared" si="11"/>
+        <v>69690</v>
       </c>
       <c r="E63" s="1">
         <f t="shared" si="10"/>
-        <v>1316957</v>
+        <v>1321213</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -1844,17 +1844,17 @@
         <v>296</v>
       </c>
       <c r="D64" s="1">
-        <f t="shared" si="12"/>
-        <v>69359</v>
+        <f t="shared" si="11"/>
+        <v>71780</v>
       </c>
       <c r="E64" s="1">
         <f t="shared" si="10"/>
-        <v>1386316</v>
+        <v>1392993</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <f t="shared" ref="A65:A85" si="13">A64+1</f>
+        <f t="shared" ref="A65:A85" si="12">A64+1</f>
         <v>63</v>
       </c>
       <c r="B65" s="1">
@@ -1866,17 +1866,17 @@
         <v>300</v>
       </c>
       <c r="D65" s="1">
-        <f t="shared" si="12"/>
-        <v>71092</v>
+        <f t="shared" si="11"/>
+        <v>73933</v>
       </c>
       <c r="E65" s="1">
         <f t="shared" si="10"/>
-        <v>1457408</v>
+        <v>1466926</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>64</v>
       </c>
       <c r="B66" s="1">
@@ -1888,17 +1888,17 @@
         <v>304</v>
       </c>
       <c r="D66" s="1">
-        <f t="shared" si="12"/>
-        <v>72869</v>
+        <f t="shared" si="11"/>
+        <v>76150</v>
       </c>
       <c r="E66" s="1">
         <f t="shared" si="10"/>
-        <v>1530277</v>
+        <v>1543076</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>65</v>
       </c>
       <c r="B67" s="1">
@@ -1910,17 +1910,17 @@
         <v>308</v>
       </c>
       <c r="D67" s="1">
-        <f t="shared" si="12"/>
-        <v>74690</v>
+        <f t="shared" si="11"/>
+        <v>78434</v>
       </c>
       <c r="E67" s="1">
         <f t="shared" si="10"/>
-        <v>1604967</v>
+        <v>1621510</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>66</v>
       </c>
       <c r="B68" s="1">
@@ -1932,386 +1932,386 @@
         <v>312</v>
       </c>
       <c r="D68" s="1">
-        <f t="shared" si="12"/>
-        <v>76557</v>
+        <f t="shared" si="11"/>
+        <v>80787</v>
       </c>
       <c r="E68" s="1">
         <f t="shared" si="10"/>
-        <v>1681524</v>
+        <v>1702297</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>67</v>
       </c>
       <c r="B69" s="1">
-        <f t="shared" ref="B69:B101" si="14">(B68+7)</f>
+        <f t="shared" ref="B69:B101" si="13">(B68+7)</f>
         <v>602</v>
       </c>
       <c r="C69" s="1">
-        <f t="shared" ref="C69:C101" si="15">(C68+4)</f>
+        <f t="shared" ref="C69:C101" si="14">(C68+4)</f>
         <v>316</v>
       </c>
       <c r="D69" s="1">
-        <f t="shared" si="12"/>
-        <v>78470</v>
+        <f t="shared" si="11"/>
+        <v>83210</v>
       </c>
       <c r="E69" s="1">
         <f t="shared" si="10"/>
-        <v>1759994</v>
+        <v>1785507</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>68</v>
       </c>
       <c r="B70" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>609</v>
       </c>
       <c r="C70" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>320</v>
       </c>
       <c r="D70" s="1">
-        <f t="shared" si="12"/>
-        <v>80431</v>
+        <f t="shared" si="11"/>
+        <v>85706</v>
       </c>
       <c r="E70" s="1">
         <f t="shared" si="10"/>
-        <v>1840425</v>
+        <v>1871213</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>69</v>
       </c>
       <c r="B71" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>616</v>
       </c>
       <c r="C71" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>324</v>
       </c>
       <c r="D71" s="1">
-        <f t="shared" si="12"/>
-        <v>82441</v>
+        <f t="shared" si="11"/>
+        <v>88277</v>
       </c>
       <c r="E71" s="1">
         <f t="shared" si="10"/>
-        <v>1922866</v>
+        <v>1959490</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>70</v>
       </c>
       <c r="B72" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>623</v>
       </c>
       <c r="C72" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>328</v>
       </c>
       <c r="D72" s="1">
-        <f t="shared" si="12"/>
-        <v>84502</v>
+        <f t="shared" si="11"/>
+        <v>90925</v>
       </c>
       <c r="E72" s="1">
         <f t="shared" si="10"/>
-        <v>2007368</v>
+        <v>2050415</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>71</v>
       </c>
       <c r="B73" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>630</v>
       </c>
       <c r="C73" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>332</v>
       </c>
       <c r="D73" s="1">
-        <f t="shared" si="12"/>
-        <v>86614</v>
+        <f t="shared" si="11"/>
+        <v>93652</v>
       </c>
       <c r="E73" s="1">
         <f t="shared" si="10"/>
-        <v>2093982</v>
+        <v>2144067</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>72</v>
       </c>
       <c r="B74" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>637</v>
       </c>
       <c r="C74" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>336</v>
       </c>
       <c r="D74" s="1">
-        <f t="shared" si="12"/>
-        <v>88779</v>
+        <f t="shared" si="11"/>
+        <v>96461</v>
       </c>
       <c r="E74" s="1">
         <f t="shared" si="10"/>
-        <v>2182761</v>
+        <v>2240528</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>73</v>
       </c>
       <c r="B75" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>644</v>
       </c>
       <c r="C75" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>340</v>
       </c>
       <c r="D75" s="1">
-        <f t="shared" si="12"/>
-        <v>90998</v>
+        <f t="shared" si="11"/>
+        <v>99354</v>
       </c>
       <c r="E75" s="1">
         <f t="shared" si="10"/>
-        <v>2273759</v>
+        <v>2339882</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>74</v>
       </c>
       <c r="B76" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>651</v>
       </c>
       <c r="C76" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>344</v>
       </c>
       <c r="D76" s="1">
-        <f t="shared" si="12"/>
-        <v>93272</v>
+        <f t="shared" si="11"/>
+        <v>102334</v>
       </c>
       <c r="E76" s="1">
         <f t="shared" si="10"/>
-        <v>2367031</v>
+        <v>2442216</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>75</v>
       </c>
       <c r="B77" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>658</v>
       </c>
       <c r="C77" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>348</v>
       </c>
       <c r="D77" s="1">
-        <f t="shared" si="12"/>
-        <v>95603</v>
+        <f t="shared" si="11"/>
+        <v>105404</v>
       </c>
       <c r="E77" s="1">
         <f t="shared" si="10"/>
-        <v>2462634</v>
+        <v>2547620</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>76</v>
       </c>
       <c r="B78" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>665</v>
       </c>
       <c r="C78" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>352</v>
       </c>
       <c r="D78" s="1">
-        <f t="shared" si="12"/>
-        <v>97993</v>
+        <f t="shared" si="11"/>
+        <v>108566</v>
       </c>
       <c r="E78" s="1">
         <f t="shared" si="10"/>
-        <v>2560627</v>
+        <v>2656186</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>77</v>
       </c>
       <c r="B79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>672</v>
       </c>
       <c r="C79" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>356</v>
       </c>
       <c r="D79" s="1">
-        <f t="shared" si="12"/>
-        <v>100442</v>
+        <f t="shared" si="11"/>
+        <v>111822</v>
       </c>
       <c r="E79" s="1">
         <f t="shared" si="10"/>
-        <v>2661069</v>
+        <v>2768008</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>78</v>
       </c>
       <c r="B80" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>679</v>
       </c>
       <c r="C80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>360</v>
       </c>
       <c r="D80" s="1">
-        <f t="shared" si="12"/>
-        <v>102953</v>
+        <f t="shared" si="11"/>
+        <v>115176</v>
       </c>
       <c r="E80" s="1">
         <f t="shared" si="10"/>
-        <v>2764022</v>
+        <v>2883184</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>79</v>
       </c>
       <c r="B81" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>686</v>
       </c>
       <c r="C81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>364</v>
       </c>
       <c r="D81" s="1">
-        <f t="shared" si="12"/>
-        <v>105526</v>
+        <f t="shared" si="11"/>
+        <v>118631</v>
       </c>
       <c r="E81" s="1">
         <f t="shared" si="10"/>
-        <v>2869548</v>
+        <v>3001815</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>80</v>
       </c>
       <c r="B82" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>693</v>
       </c>
       <c r="C82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>368</v>
       </c>
       <c r="D82" s="1">
-        <f t="shared" si="12"/>
-        <v>108164</v>
+        <f t="shared" si="11"/>
+        <v>122189</v>
       </c>
       <c r="E82" s="1">
         <f t="shared" si="10"/>
-        <v>2977712</v>
+        <v>3124004</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>81</v>
       </c>
       <c r="B83" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>700</v>
       </c>
       <c r="C83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>372</v>
       </c>
       <c r="D83" s="1">
-        <f t="shared" si="12"/>
-        <v>110868</v>
+        <f t="shared" si="11"/>
+        <v>125854</v>
       </c>
       <c r="E83" s="1">
         <f t="shared" si="10"/>
-        <v>3088580</v>
+        <v>3249858</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>82</v>
       </c>
       <c r="B84" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>707</v>
       </c>
       <c r="C84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>376</v>
       </c>
       <c r="D84" s="1">
-        <f t="shared" si="12"/>
-        <v>113639</v>
+        <f t="shared" si="11"/>
+        <v>129629</v>
       </c>
       <c r="E84" s="1">
         <f t="shared" si="10"/>
-        <v>3202219</v>
+        <v>3379487</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>83</v>
       </c>
       <c r="B85" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>714</v>
       </c>
       <c r="C85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>380</v>
       </c>
       <c r="D85" s="1">
-        <f t="shared" si="12"/>
-        <v>116479</v>
+        <f t="shared" si="11"/>
+        <v>133517</v>
       </c>
       <c r="E85" s="1">
         <f t="shared" si="10"/>
-        <v>3318698</v>
+        <v>3513004</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2320,20 +2320,20 @@
         <v>84</v>
       </c>
       <c r="B86" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>721</v>
       </c>
       <c r="C86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>384</v>
       </c>
       <c r="D86" s="1">
-        <f t="shared" si="12"/>
-        <v>119390</v>
+        <f t="shared" si="11"/>
+        <v>137522</v>
       </c>
       <c r="E86" s="1">
         <f t="shared" si="10"/>
-        <v>3438088</v>
+        <v>3650526</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2342,328 +2342,328 @@
         <v>85</v>
       </c>
       <c r="B87" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>728</v>
       </c>
       <c r="C87" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>388</v>
       </c>
       <c r="D87" s="1">
-        <f t="shared" si="12"/>
-        <v>122374</v>
+        <f t="shared" si="11"/>
+        <v>141647</v>
       </c>
       <c r="E87" s="1">
         <f t="shared" si="10"/>
-        <v>3560462</v>
+        <v>3792173</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <f t="shared" ref="A88:A101" si="16">A87+1</f>
+        <f t="shared" ref="A88:A101" si="15">A87+1</f>
         <v>86</v>
       </c>
       <c r="B88" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>735</v>
       </c>
       <c r="C88" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>392</v>
       </c>
       <c r="D88" s="1">
-        <f t="shared" si="12"/>
-        <v>125433</v>
+        <f t="shared" si="11"/>
+        <v>145896</v>
       </c>
       <c r="E88" s="1">
         <f t="shared" si="10"/>
-        <v>3685895</v>
+        <v>3938069</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>87</v>
       </c>
       <c r="B89" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>742</v>
       </c>
       <c r="C89" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>396</v>
       </c>
       <c r="D89" s="1">
-        <f t="shared" si="12"/>
-        <v>128568</v>
+        <f t="shared" si="11"/>
+        <v>150272</v>
       </c>
       <c r="E89" s="1">
-        <f t="shared" ref="E89:E101" si="17">D89+E88</f>
-        <v>3814463</v>
+        <f t="shared" ref="E89:E101" si="16">D89+E88</f>
+        <v>4088341</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
+        <f t="shared" si="15"/>
+        <v>88</v>
+      </c>
+      <c r="B90" s="1">
+        <f t="shared" si="13"/>
+        <v>749</v>
+      </c>
+      <c r="C90" s="1">
+        <f t="shared" si="14"/>
+        <v>400</v>
+      </c>
+      <c r="D90" s="1">
+        <f t="shared" si="11"/>
+        <v>154780</v>
+      </c>
+      <c r="E90" s="1">
         <f t="shared" si="16"/>
-        <v>88</v>
-      </c>
-      <c r="B90" s="1">
-        <f t="shared" si="14"/>
-        <v>749</v>
-      </c>
-      <c r="C90" s="1">
-        <f t="shared" si="15"/>
-        <v>400</v>
-      </c>
-      <c r="D90" s="1">
-        <f t="shared" si="12"/>
-        <v>131782</v>
-      </c>
-      <c r="E90" s="1">
-        <f t="shared" si="17"/>
-        <v>3946245</v>
+        <v>4243121</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
+        <f t="shared" si="15"/>
+        <v>89</v>
+      </c>
+      <c r="B91" s="1">
+        <f t="shared" si="13"/>
+        <v>756</v>
+      </c>
+      <c r="C91" s="1">
+        <f t="shared" si="14"/>
+        <v>404</v>
+      </c>
+      <c r="D91" s="1">
+        <f t="shared" si="11"/>
+        <v>159423</v>
+      </c>
+      <c r="E91" s="1">
         <f t="shared" si="16"/>
-        <v>89</v>
-      </c>
-      <c r="B91" s="1">
-        <f t="shared" si="14"/>
-        <v>756</v>
-      </c>
-      <c r="C91" s="1">
-        <f t="shared" si="15"/>
-        <v>404</v>
-      </c>
-      <c r="D91" s="1">
-        <f t="shared" si="12"/>
-        <v>135076</v>
-      </c>
-      <c r="E91" s="1">
-        <f t="shared" si="17"/>
-        <v>4081321</v>
+        <v>4402544</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
+        <f t="shared" si="15"/>
+        <v>90</v>
+      </c>
+      <c r="B92" s="1">
+        <f t="shared" si="13"/>
+        <v>763</v>
+      </c>
+      <c r="C92" s="1">
+        <f t="shared" si="14"/>
+        <v>408</v>
+      </c>
+      <c r="D92" s="1">
+        <f t="shared" si="11"/>
+        <v>164205</v>
+      </c>
+      <c r="E92" s="1">
         <f t="shared" si="16"/>
-        <v>90</v>
-      </c>
-      <c r="B92" s="1">
-        <f t="shared" si="14"/>
-        <v>763</v>
-      </c>
-      <c r="C92" s="1">
-        <f t="shared" si="15"/>
-        <v>408</v>
-      </c>
-      <c r="D92" s="1">
-        <f t="shared" si="12"/>
-        <v>138452</v>
-      </c>
-      <c r="E92" s="1">
-        <f t="shared" si="17"/>
-        <v>4219773</v>
+        <v>4566749</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
+        <f t="shared" si="15"/>
+        <v>91</v>
+      </c>
+      <c r="B93" s="1">
+        <f t="shared" si="13"/>
+        <v>770</v>
+      </c>
+      <c r="C93" s="1">
+        <f t="shared" si="14"/>
+        <v>412</v>
+      </c>
+      <c r="D93" s="1">
+        <f t="shared" si="11"/>
+        <v>169131</v>
+      </c>
+      <c r="E93" s="1">
         <f t="shared" si="16"/>
-        <v>91</v>
-      </c>
-      <c r="B93" s="1">
-        <f t="shared" si="14"/>
-        <v>770</v>
-      </c>
-      <c r="C93" s="1">
-        <f t="shared" si="15"/>
-        <v>412</v>
-      </c>
-      <c r="D93" s="1">
-        <f t="shared" si="12"/>
-        <v>141913</v>
-      </c>
-      <c r="E93" s="1">
-        <f t="shared" si="17"/>
-        <v>4361686</v>
+        <v>4735880</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
+        <f t="shared" si="15"/>
+        <v>92</v>
+      </c>
+      <c r="B94" s="1">
+        <f t="shared" si="13"/>
+        <v>777</v>
+      </c>
+      <c r="C94" s="1">
+        <f t="shared" si="14"/>
+        <v>416</v>
+      </c>
+      <c r="D94" s="1">
+        <f t="shared" si="11"/>
+        <v>174204</v>
+      </c>
+      <c r="E94" s="1">
         <f t="shared" si="16"/>
-        <v>92</v>
-      </c>
-      <c r="B94" s="1">
-        <f t="shared" si="14"/>
-        <v>777</v>
-      </c>
-      <c r="C94" s="1">
-        <f t="shared" si="15"/>
-        <v>416</v>
-      </c>
-      <c r="D94" s="1">
-        <f t="shared" si="12"/>
-        <v>145460</v>
-      </c>
-      <c r="E94" s="1">
-        <f t="shared" si="17"/>
-        <v>4507146</v>
+        <v>4910084</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
+        <f t="shared" si="15"/>
+        <v>93</v>
+      </c>
+      <c r="B95" s="1">
+        <f t="shared" si="13"/>
+        <v>784</v>
+      </c>
+      <c r="C95" s="1">
+        <f t="shared" si="14"/>
+        <v>420</v>
+      </c>
+      <c r="D95" s="1">
+        <f t="shared" si="11"/>
+        <v>179430</v>
+      </c>
+      <c r="E95" s="1">
         <f t="shared" si="16"/>
-        <v>93</v>
-      </c>
-      <c r="B95" s="1">
-        <f t="shared" si="14"/>
-        <v>784</v>
-      </c>
-      <c r="C95" s="1">
-        <f t="shared" si="15"/>
-        <v>420</v>
-      </c>
-      <c r="D95" s="1">
-        <f t="shared" si="12"/>
-        <v>149096</v>
-      </c>
-      <c r="E95" s="1">
-        <f t="shared" si="17"/>
-        <v>4656242</v>
+        <v>5089514</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
+        <f t="shared" si="15"/>
+        <v>94</v>
+      </c>
+      <c r="B96" s="1">
+        <f t="shared" si="13"/>
+        <v>791</v>
+      </c>
+      <c r="C96" s="1">
+        <f t="shared" si="14"/>
+        <v>424</v>
+      </c>
+      <c r="D96" s="1">
+        <f t="shared" si="11"/>
+        <v>184812</v>
+      </c>
+      <c r="E96" s="1">
         <f t="shared" si="16"/>
-        <v>94</v>
-      </c>
-      <c r="B96" s="1">
-        <f t="shared" si="14"/>
-        <v>791</v>
-      </c>
-      <c r="C96" s="1">
-        <f t="shared" si="15"/>
-        <v>424</v>
-      </c>
-      <c r="D96" s="1">
-        <f t="shared" si="12"/>
-        <v>152823</v>
-      </c>
-      <c r="E96" s="1">
-        <f t="shared" si="17"/>
-        <v>4809065</v>
+        <v>5274326</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
+        <f t="shared" si="15"/>
+        <v>95</v>
+      </c>
+      <c r="B97" s="1">
+        <f t="shared" si="13"/>
+        <v>798</v>
+      </c>
+      <c r="C97" s="1">
+        <f t="shared" si="14"/>
+        <v>428</v>
+      </c>
+      <c r="D97" s="1">
+        <f t="shared" si="11"/>
+        <v>190356</v>
+      </c>
+      <c r="E97" s="1">
         <f t="shared" si="16"/>
-        <v>95</v>
-      </c>
-      <c r="B97" s="1">
-        <f t="shared" si="14"/>
-        <v>798</v>
-      </c>
-      <c r="C97" s="1">
-        <f t="shared" si="15"/>
-        <v>428</v>
-      </c>
-      <c r="D97" s="1">
-        <f t="shared" si="12"/>
-        <v>156643</v>
-      </c>
-      <c r="E97" s="1">
-        <f t="shared" si="17"/>
-        <v>4965708</v>
+        <v>5464682</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
+        <f t="shared" si="15"/>
+        <v>96</v>
+      </c>
+      <c r="B98" s="1">
+        <f t="shared" si="13"/>
+        <v>805</v>
+      </c>
+      <c r="C98" s="1">
+        <f t="shared" si="14"/>
+        <v>432</v>
+      </c>
+      <c r="D98" s="1">
+        <f t="shared" si="11"/>
+        <v>196066</v>
+      </c>
+      <c r="E98" s="1">
         <f t="shared" si="16"/>
-        <v>96</v>
-      </c>
-      <c r="B98" s="1">
-        <f t="shared" si="14"/>
-        <v>805</v>
-      </c>
-      <c r="C98" s="1">
-        <f t="shared" si="15"/>
-        <v>432</v>
-      </c>
-      <c r="D98" s="1">
-        <f t="shared" si="12"/>
-        <v>160559</v>
-      </c>
-      <c r="E98" s="1">
-        <f t="shared" si="17"/>
-        <v>5126267</v>
+        <v>5660748</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
+        <f t="shared" si="15"/>
+        <v>97</v>
+      </c>
+      <c r="B99" s="1">
+        <f t="shared" si="13"/>
+        <v>812</v>
+      </c>
+      <c r="C99" s="1">
+        <f t="shared" si="14"/>
+        <v>436</v>
+      </c>
+      <c r="D99" s="1">
+        <f t="shared" si="11"/>
+        <v>201947</v>
+      </c>
+      <c r="E99" s="1">
         <f t="shared" si="16"/>
-        <v>97</v>
-      </c>
-      <c r="B99" s="1">
-        <f t="shared" si="14"/>
-        <v>812</v>
-      </c>
-      <c r="C99" s="1">
-        <f t="shared" si="15"/>
-        <v>436</v>
-      </c>
-      <c r="D99" s="1">
-        <f t="shared" si="12"/>
-        <v>164572</v>
-      </c>
-      <c r="E99" s="1">
-        <f t="shared" si="17"/>
-        <v>5290839</v>
+        <v>5862695</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
+        <f t="shared" si="15"/>
+        <v>98</v>
+      </c>
+      <c r="B100" s="1">
+        <f t="shared" si="13"/>
+        <v>819</v>
+      </c>
+      <c r="C100" s="1">
+        <f t="shared" si="14"/>
+        <v>440</v>
+      </c>
+      <c r="D100" s="1">
+        <f t="shared" si="11"/>
+        <v>208005</v>
+      </c>
+      <c r="E100" s="1">
         <f t="shared" si="16"/>
-        <v>98</v>
-      </c>
-      <c r="B100" s="1">
-        <f t="shared" si="14"/>
-        <v>819</v>
-      </c>
-      <c r="C100" s="1">
-        <f t="shared" si="15"/>
-        <v>440</v>
-      </c>
-      <c r="D100" s="1">
-        <f t="shared" si="12"/>
-        <v>168686</v>
-      </c>
-      <c r="E100" s="1">
-        <f t="shared" si="17"/>
-        <v>5459525</v>
+        <v>6070700</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
+        <f t="shared" si="15"/>
+        <v>99</v>
+      </c>
+      <c r="B101" s="1">
+        <f t="shared" si="13"/>
+        <v>826</v>
+      </c>
+      <c r="C101" s="1">
+        <f t="shared" si="14"/>
+        <v>444</v>
+      </c>
+      <c r="D101" s="1">
+        <f t="shared" si="11"/>
+        <v>214245</v>
+      </c>
+      <c r="E101" s="1">
         <f t="shared" si="16"/>
-        <v>99</v>
-      </c>
-      <c r="B101" s="1">
-        <f t="shared" si="14"/>
-        <v>826</v>
-      </c>
-      <c r="C101" s="1">
-        <f t="shared" si="15"/>
-        <v>444</v>
-      </c>
-      <c r="D101" s="1">
-        <f t="shared" si="12"/>
-        <v>172903</v>
-      </c>
-      <c r="E101" s="1">
-        <f t="shared" si="17"/>
-        <v>5632428</v>
+        <v>6284945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added real-time movement and mini-boss dialogue
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05872086-26F9-4CEB-B8B4-B3A008DC6A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4B4799-0D9C-41F1-AC0D-6CB3EA07553C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25905" yWindow="990" windowWidth="21585" windowHeight="12690" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="10965" yWindow="1350" windowWidth="21585" windowHeight="11610" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -905,6 +905,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -2668,7 +2669,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F3:F20"/>
+    <mergeCell ref="F3:F21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Quick Travel and Element "Water"
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4B4799-0D9C-41F1-AC0D-6CB3EA07553C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A2FD0B-CC4B-4E0C-8A71-5EF707AC12D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10965" yWindow="1350" windowWidth="21585" windowHeight="11610" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Levels" sheetId="1" r:id="rId1"/>
+    <sheet name="Shopkeeper" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>Lv</t>
   </si>
@@ -57,13 +58,130 @@
   </si>
   <si>
     <t>STA</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Dmg/Inherit</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Orb of the Arctic</t>
+  </si>
+  <si>
+    <t>Freezadia</t>
+  </si>
+  <si>
+    <t>Skill</t>
+  </si>
+  <si>
+    <t>x2 Crystalised Flake</t>
+  </si>
+  <si>
+    <t>x5 Ice Shard</t>
+  </si>
+  <si>
+    <t>x10 Ice Core</t>
+  </si>
+  <si>
+    <t>Melee</t>
+  </si>
+  <si>
+    <t>x5 Scratched Coin</t>
+  </si>
+  <si>
+    <t>x5 Foreign Coin</t>
+  </si>
+  <si>
+    <t>Atlantis Ruins</t>
+  </si>
+  <si>
+    <t>4*</t>
+  </si>
+  <si>
+    <t>5*</t>
+  </si>
+  <si>
+    <t>M4 Garand</t>
+  </si>
+  <si>
+    <t>x10 Gun Fragment</t>
+  </si>
+  <si>
+    <t>Snow Sword</t>
+  </si>
+  <si>
+    <t>TRADER</t>
+  </si>
+  <si>
+    <t>Orb of the Ocean</t>
+  </si>
+  <si>
+    <t>Hexaon</t>
+  </si>
+  <si>
+    <t>x10 Ink Vial</t>
+  </si>
+  <si>
+    <t>x5 Squid Head</t>
+  </si>
+  <si>
+    <t>x3 Ice Shard</t>
+  </si>
+  <si>
+    <t>x8 Ice Core</t>
+  </si>
+  <si>
+    <t>x10 Water Balloon</t>
+  </si>
+  <si>
+    <t>Diamond Sword</t>
+  </si>
+  <si>
+    <t>x2 Diamond</t>
+  </si>
+  <si>
+    <t>x3 Chipped Diamond</t>
+  </si>
+  <si>
+    <t>Junk Stick</t>
+  </si>
+  <si>
+    <t>3*</t>
+  </si>
+  <si>
+    <t>x3 Thawn Bandage</t>
+  </si>
+  <si>
+    <t>x3 Foreign Coin</t>
+  </si>
+  <si>
+    <t>x3 Ripped Shoes</t>
+  </si>
+  <si>
+    <t>x3 Snowball</t>
+  </si>
+  <si>
+    <t>Jar of Coins</t>
+  </si>
+  <si>
+    <t>x2 Gold Coin</t>
+  </si>
+  <si>
+    <t>x20 Snowball</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,19 +204,143 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="11">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -107,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -117,6 +359,116 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,6 +804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C80B310D-5657-4E61-A0DA-301A4716D270}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A2:F101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -488,7 +841,7 @@
         <v>140</v>
       </c>
       <c r="C3" s="1">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -506,7 +859,7 @@
       </c>
       <c r="C4" s="1">
         <f>(C3+4)</f>
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D4" s="1">
         <v>22</v>
@@ -527,7 +880,7 @@
       </c>
       <c r="C5" s="1">
         <f t="shared" ref="C5:C68" si="1">(C4+4)</f>
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D5" s="1">
         <f>INT(D4*1.35)</f>
@@ -550,7 +903,7 @@
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" ref="D6:D23" si="3">INT(D5*1.35)</f>
@@ -573,7 +926,7 @@
       </c>
       <c r="C7" s="1">
         <f t="shared" si="1"/>
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="D7" s="1">
         <f t="shared" si="3"/>
@@ -596,7 +949,7 @@
       </c>
       <c r="C8" s="1">
         <f t="shared" si="1"/>
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="3"/>
@@ -619,7 +972,7 @@
       </c>
       <c r="C9" s="1">
         <f>(C8+4)</f>
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" si="3"/>
@@ -642,7 +995,7 @@
       </c>
       <c r="C10" s="1">
         <f t="shared" si="1"/>
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D10" s="1">
         <f t="shared" si="3"/>
@@ -665,7 +1018,7 @@
       </c>
       <c r="C11" s="1">
         <f t="shared" si="1"/>
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" si="3"/>
@@ -688,7 +1041,7 @@
       </c>
       <c r="C12" s="1">
         <f t="shared" si="1"/>
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="3"/>
@@ -711,7 +1064,7 @@
       </c>
       <c r="C13" s="1">
         <f t="shared" si="1"/>
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" si="3"/>
@@ -734,7 +1087,7 @@
       </c>
       <c r="C14" s="1">
         <f t="shared" si="1"/>
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" si="3"/>
@@ -757,7 +1110,7 @@
       </c>
       <c r="C15" s="1">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D15" s="1">
         <f t="shared" si="3"/>
@@ -780,7 +1133,7 @@
       </c>
       <c r="C16" s="1">
         <f t="shared" si="1"/>
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="D16" s="1">
         <f t="shared" si="3"/>
@@ -803,7 +1156,7 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" si="1"/>
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="D17" s="1">
         <f t="shared" si="3"/>
@@ -826,7 +1179,7 @@
       </c>
       <c r="C18" s="1">
         <f t="shared" si="1"/>
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="D18" s="1">
         <f t="shared" si="3"/>
@@ -849,7 +1202,7 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" si="1"/>
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="D19" s="1">
         <f t="shared" si="3"/>
@@ -872,7 +1225,7 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" si="1"/>
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D20" s="1">
         <f t="shared" si="3"/>
@@ -895,7 +1248,7 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" si="1"/>
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D21" s="1">
         <f t="shared" si="3"/>
@@ -918,7 +1271,7 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" si="1"/>
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" si="3"/>
@@ -940,7 +1293,7 @@
       </c>
       <c r="C23" s="1">
         <f t="shared" si="1"/>
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" si="3"/>
@@ -962,7 +1315,7 @@
       </c>
       <c r="C24" s="1">
         <f t="shared" si="1"/>
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="D24" s="1">
         <f>INT(D23*1.075)</f>
@@ -984,7 +1337,7 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" si="1"/>
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D25" s="1">
         <f t="shared" ref="D25:D52" si="8">INT(D24*1.075)</f>
@@ -1006,7 +1359,7 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" si="1"/>
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="D26" s="1">
         <f t="shared" si="8"/>
@@ -1028,7 +1381,7 @@
       </c>
       <c r="C27" s="1">
         <f t="shared" si="1"/>
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D27" s="1">
         <f t="shared" si="8"/>
@@ -1050,7 +1403,7 @@
       </c>
       <c r="C28" s="1">
         <f t="shared" si="1"/>
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="D28" s="1">
         <f t="shared" si="8"/>
@@ -1072,7 +1425,7 @@
       </c>
       <c r="C29" s="1">
         <f t="shared" si="1"/>
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="D29" s="1">
         <f t="shared" si="8"/>
@@ -1094,7 +1447,7 @@
       </c>
       <c r="C30" s="1">
         <f t="shared" si="1"/>
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="D30" s="1">
         <f t="shared" si="8"/>
@@ -1116,7 +1469,7 @@
       </c>
       <c r="C31" s="1">
         <f t="shared" si="1"/>
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="D31" s="1">
         <f t="shared" si="8"/>
@@ -1138,7 +1491,7 @@
       </c>
       <c r="C32" s="1">
         <f t="shared" si="1"/>
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="D32" s="1">
         <f t="shared" si="8"/>
@@ -1160,7 +1513,7 @@
       </c>
       <c r="C33" s="1">
         <f t="shared" si="1"/>
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D33" s="1">
         <f t="shared" si="8"/>
@@ -1182,7 +1535,7 @@
       </c>
       <c r="C34" s="1">
         <f t="shared" si="1"/>
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" si="8"/>
@@ -1204,7 +1557,7 @@
       </c>
       <c r="C35" s="1">
         <f t="shared" si="1"/>
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="D35" s="1">
         <f t="shared" si="8"/>
@@ -1226,7 +1579,7 @@
       </c>
       <c r="C36" s="1">
         <f t="shared" si="1"/>
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="D36" s="1">
         <f t="shared" si="8"/>
@@ -1248,7 +1601,7 @@
       </c>
       <c r="C37" s="1">
         <f t="shared" si="1"/>
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="D37" s="1">
         <f t="shared" si="8"/>
@@ -1270,7 +1623,7 @@
       </c>
       <c r="C38" s="1">
         <f t="shared" si="1"/>
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="D38" s="1">
         <f t="shared" si="8"/>
@@ -1292,7 +1645,7 @@
       </c>
       <c r="C39" s="1">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="D39" s="1">
         <f t="shared" si="8"/>
@@ -1314,7 +1667,7 @@
       </c>
       <c r="C40" s="1">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="D40" s="1">
         <f t="shared" si="8"/>
@@ -1336,7 +1689,7 @@
       </c>
       <c r="C41" s="1">
         <f t="shared" si="1"/>
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="D41" s="1">
         <f t="shared" si="8"/>
@@ -1358,7 +1711,7 @@
       </c>
       <c r="C42" s="1">
         <f t="shared" si="1"/>
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="D42" s="1">
         <f t="shared" si="8"/>
@@ -1380,7 +1733,7 @@
       </c>
       <c r="C43" s="1">
         <f t="shared" si="1"/>
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" si="8"/>
@@ -1402,7 +1755,7 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" si="1"/>
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" si="8"/>
@@ -1424,7 +1777,7 @@
       </c>
       <c r="C45" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="D45" s="1">
         <f t="shared" si="8"/>
@@ -1446,7 +1799,7 @@
       </c>
       <c r="C46" s="1">
         <f t="shared" si="1"/>
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="D46" s="1">
         <f t="shared" si="8"/>
@@ -1468,7 +1821,7 @@
       </c>
       <c r="C47" s="1">
         <f t="shared" si="1"/>
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="D47" s="1">
         <f t="shared" si="8"/>
@@ -1490,7 +1843,7 @@
       </c>
       <c r="C48" s="1">
         <f t="shared" si="1"/>
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="D48" s="1">
         <f t="shared" si="8"/>
@@ -1512,7 +1865,7 @@
       </c>
       <c r="C49" s="1">
         <f t="shared" si="1"/>
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="D49" s="1">
         <f t="shared" si="8"/>
@@ -1534,7 +1887,7 @@
       </c>
       <c r="C50" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="D50" s="1">
         <f t="shared" si="8"/>
@@ -1556,7 +1909,7 @@
       </c>
       <c r="C51" s="1">
         <f t="shared" si="1"/>
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="D51" s="1">
         <f t="shared" si="8"/>
@@ -1578,7 +1931,7 @@
       </c>
       <c r="C52" s="1">
         <f t="shared" si="1"/>
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="D52" s="1">
         <f t="shared" si="8"/>
@@ -1600,7 +1953,7 @@
       </c>
       <c r="C53" s="1">
         <f t="shared" si="1"/>
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="D53" s="1">
         <f>INT(D52*1.03)</f>
@@ -1622,7 +1975,7 @@
       </c>
       <c r="C54" s="1">
         <f t="shared" si="1"/>
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="D54" s="1">
         <f t="shared" ref="D54:D101" si="11">INT(D53*1.03)</f>
@@ -1644,7 +1997,7 @@
       </c>
       <c r="C55" s="1">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="D55" s="1">
         <f t="shared" si="11"/>
@@ -1666,7 +2019,7 @@
       </c>
       <c r="C56" s="1">
         <f t="shared" si="1"/>
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="D56" s="1">
         <f t="shared" si="11"/>
@@ -1688,7 +2041,7 @@
       </c>
       <c r="C57" s="1">
         <f t="shared" si="1"/>
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="D57" s="1">
         <f t="shared" si="11"/>
@@ -1710,7 +2063,7 @@
       </c>
       <c r="C58" s="1">
         <f t="shared" si="1"/>
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="D58" s="1">
         <f t="shared" si="11"/>
@@ -1732,7 +2085,7 @@
       </c>
       <c r="C59" s="1">
         <f t="shared" si="1"/>
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="D59" s="1">
         <f t="shared" si="11"/>
@@ -1754,7 +2107,7 @@
       </c>
       <c r="C60" s="1">
         <f t="shared" si="1"/>
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="D60" s="1">
         <f t="shared" si="11"/>
@@ -1776,7 +2129,7 @@
       </c>
       <c r="C61" s="1">
         <f t="shared" si="1"/>
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="D61" s="1">
         <f t="shared" si="11"/>
@@ -1798,7 +2151,7 @@
       </c>
       <c r="C62" s="1">
         <f t="shared" si="1"/>
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="D62" s="1">
         <f t="shared" si="11"/>
@@ -1820,7 +2173,7 @@
       </c>
       <c r="C63" s="1">
         <f t="shared" si="1"/>
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="D63" s="1">
         <f t="shared" si="11"/>
@@ -1842,7 +2195,7 @@
       </c>
       <c r="C64" s="1">
         <f t="shared" si="1"/>
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="D64" s="1">
         <f t="shared" si="11"/>
@@ -1864,7 +2217,7 @@
       </c>
       <c r="C65" s="1">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="D65" s="1">
         <f t="shared" si="11"/>
@@ -1886,7 +2239,7 @@
       </c>
       <c r="C66" s="1">
         <f t="shared" si="1"/>
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="D66" s="1">
         <f t="shared" si="11"/>
@@ -1908,7 +2261,7 @@
       </c>
       <c r="C67" s="1">
         <f t="shared" si="1"/>
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="D67" s="1">
         <f t="shared" si="11"/>
@@ -1930,7 +2283,7 @@
       </c>
       <c r="C68" s="1">
         <f t="shared" si="1"/>
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="D68" s="1">
         <f t="shared" si="11"/>
@@ -1952,7 +2305,7 @@
       </c>
       <c r="C69" s="1">
         <f t="shared" ref="C69:C101" si="14">(C68+4)</f>
-        <v>316</v>
+        <v>326</v>
       </c>
       <c r="D69" s="1">
         <f t="shared" si="11"/>
@@ -1974,7 +2327,7 @@
       </c>
       <c r="C70" s="1">
         <f t="shared" si="14"/>
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="D70" s="1">
         <f t="shared" si="11"/>
@@ -1996,7 +2349,7 @@
       </c>
       <c r="C71" s="1">
         <f t="shared" si="14"/>
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="D71" s="1">
         <f t="shared" si="11"/>
@@ -2018,7 +2371,7 @@
       </c>
       <c r="C72" s="1">
         <f t="shared" si="14"/>
-        <v>328</v>
+        <v>338</v>
       </c>
       <c r="D72" s="1">
         <f t="shared" si="11"/>
@@ -2040,7 +2393,7 @@
       </c>
       <c r="C73" s="1">
         <f t="shared" si="14"/>
-        <v>332</v>
+        <v>342</v>
       </c>
       <c r="D73" s="1">
         <f t="shared" si="11"/>
@@ -2062,7 +2415,7 @@
       </c>
       <c r="C74" s="1">
         <f t="shared" si="14"/>
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="D74" s="1">
         <f t="shared" si="11"/>
@@ -2084,7 +2437,7 @@
       </c>
       <c r="C75" s="1">
         <f t="shared" si="14"/>
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="D75" s="1">
         <f t="shared" si="11"/>
@@ -2106,7 +2459,7 @@
       </c>
       <c r="C76" s="1">
         <f t="shared" si="14"/>
-        <v>344</v>
+        <v>354</v>
       </c>
       <c r="D76" s="1">
         <f t="shared" si="11"/>
@@ -2128,7 +2481,7 @@
       </c>
       <c r="C77" s="1">
         <f t="shared" si="14"/>
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="D77" s="1">
         <f t="shared" si="11"/>
@@ -2150,7 +2503,7 @@
       </c>
       <c r="C78" s="1">
         <f t="shared" si="14"/>
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="D78" s="1">
         <f t="shared" si="11"/>
@@ -2172,7 +2525,7 @@
       </c>
       <c r="C79" s="1">
         <f t="shared" si="14"/>
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="D79" s="1">
         <f t="shared" si="11"/>
@@ -2194,7 +2547,7 @@
       </c>
       <c r="C80" s="1">
         <f t="shared" si="14"/>
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="D80" s="1">
         <f t="shared" si="11"/>
@@ -2216,7 +2569,7 @@
       </c>
       <c r="C81" s="1">
         <f t="shared" si="14"/>
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="D81" s="1">
         <f t="shared" si="11"/>
@@ -2238,7 +2591,7 @@
       </c>
       <c r="C82" s="1">
         <f t="shared" si="14"/>
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="D82" s="1">
         <f t="shared" si="11"/>
@@ -2260,7 +2613,7 @@
       </c>
       <c r="C83" s="1">
         <f t="shared" si="14"/>
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="D83" s="1">
         <f t="shared" si="11"/>
@@ -2282,7 +2635,7 @@
       </c>
       <c r="C84" s="1">
         <f t="shared" si="14"/>
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="D84" s="1">
         <f t="shared" si="11"/>
@@ -2304,7 +2657,7 @@
       </c>
       <c r="C85" s="1">
         <f t="shared" si="14"/>
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="D85" s="1">
         <f t="shared" si="11"/>
@@ -2326,7 +2679,7 @@
       </c>
       <c r="C86" s="1">
         <f t="shared" si="14"/>
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="D86" s="1">
         <f t="shared" si="11"/>
@@ -2348,7 +2701,7 @@
       </c>
       <c r="C87" s="1">
         <f t="shared" si="14"/>
-        <v>388</v>
+        <v>398</v>
       </c>
       <c r="D87" s="1">
         <f t="shared" si="11"/>
@@ -2370,7 +2723,7 @@
       </c>
       <c r="C88" s="1">
         <f t="shared" si="14"/>
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="D88" s="1">
         <f t="shared" si="11"/>
@@ -2392,7 +2745,7 @@
       </c>
       <c r="C89" s="1">
         <f t="shared" si="14"/>
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="D89" s="1">
         <f t="shared" si="11"/>
@@ -2414,7 +2767,7 @@
       </c>
       <c r="C90" s="1">
         <f t="shared" si="14"/>
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="D90" s="1">
         <f t="shared" si="11"/>
@@ -2436,7 +2789,7 @@
       </c>
       <c r="C91" s="1">
         <f t="shared" si="14"/>
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="D91" s="1">
         <f t="shared" si="11"/>
@@ -2458,7 +2811,7 @@
       </c>
       <c r="C92" s="1">
         <f t="shared" si="14"/>
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="D92" s="1">
         <f t="shared" si="11"/>
@@ -2480,7 +2833,7 @@
       </c>
       <c r="C93" s="1">
         <f t="shared" si="14"/>
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="D93" s="1">
         <f t="shared" si="11"/>
@@ -2502,7 +2855,7 @@
       </c>
       <c r="C94" s="1">
         <f t="shared" si="14"/>
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="D94" s="1">
         <f t="shared" si="11"/>
@@ -2524,7 +2877,7 @@
       </c>
       <c r="C95" s="1">
         <f t="shared" si="14"/>
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="D95" s="1">
         <f t="shared" si="11"/>
@@ -2546,7 +2899,7 @@
       </c>
       <c r="C96" s="1">
         <f t="shared" si="14"/>
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="D96" s="1">
         <f t="shared" si="11"/>
@@ -2568,7 +2921,7 @@
       </c>
       <c r="C97" s="1">
         <f t="shared" si="14"/>
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="D97" s="1">
         <f t="shared" si="11"/>
@@ -2590,7 +2943,7 @@
       </c>
       <c r="C98" s="1">
         <f t="shared" si="14"/>
-        <v>432</v>
+        <v>442</v>
       </c>
       <c r="D98" s="1">
         <f t="shared" si="11"/>
@@ -2612,7 +2965,7 @@
       </c>
       <c r="C99" s="1">
         <f t="shared" si="14"/>
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="D99" s="1">
         <f t="shared" si="11"/>
@@ -2634,7 +2987,7 @@
       </c>
       <c r="C100" s="1">
         <f t="shared" si="14"/>
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="D100" s="1">
         <f t="shared" si="11"/>
@@ -2656,7 +3009,7 @@
       </c>
       <c r="C101" s="1">
         <f t="shared" si="14"/>
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="D101" s="1">
         <f t="shared" si="11"/>
@@ -2673,4 +3026,343 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46073598-FE75-40E6-92C9-07FD455292EE}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" customWidth="1"/>
+    <col min="6" max="6" width="26.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="18"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="32">
+        <v>52</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="33"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="33"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="39"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="4">
+        <v>96</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="4">
+        <v>137</v>
+      </c>
+      <c r="E17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="4"/>
+      <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="14">
+        <v>184</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="10">
+        <v>209</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="7"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="D4:D7"/>
+    <mergeCell ref="F4:F7"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="C11:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added Atlantis Floor 4
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A2FD0B-CC4B-4E0C-8A71-5EF707AC12D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5D9E8E-AD57-46D6-ACC0-FED8FECCBCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="6135" yWindow="1365" windowWidth="21585" windowHeight="13440" activeTab="1" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -123,9 +123,6 @@
     <t>Orb of the Ocean</t>
   </si>
   <si>
-    <t>Hexaon</t>
-  </si>
-  <si>
     <t>x10 Ink Vial</t>
   </si>
   <si>
@@ -175,6 +172,9 @@
   </si>
   <si>
     <t>x20 Snowball</t>
+  </si>
+  <si>
+    <t>Splashadia</t>
   </si>
 </sst>
 </file>
@@ -349,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -357,39 +357,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -398,6 +376,58 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -408,67 +438,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -845,7 +816,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="21" t="s">
         <v>4</v>
       </c>
     </row>
@@ -867,7 +838,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="3"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -890,7 +861,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="21"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -913,7 +884,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="21"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -936,7 +907,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="3"/>
+      <c r="F7" s="21"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -959,7 +930,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="21"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -982,7 +953,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="21"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1005,7 +976,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1028,7 +999,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="3"/>
+      <c r="F11" s="21"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1051,7 +1022,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="3"/>
+      <c r="F12" s="21"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1074,7 +1045,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="3"/>
+      <c r="F13" s="21"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1097,7 +1068,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="F14" s="21"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1120,7 +1091,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="21"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1143,7 +1114,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="21"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1166,7 +1137,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="3"/>
+      <c r="F17" s="21"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1189,7 +1160,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="21"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1212,7 +1183,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="3"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1235,7 +1206,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="3"/>
+      <c r="F20" s="21"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1258,7 +1229,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="3"/>
+      <c r="F21" s="21"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -3043,324 +3014,324 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="18"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="26" t="s">
+      <c r="B3" s="32"/>
+      <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="C4" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="17">
+        <v>52</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="18"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="21"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="18"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="21"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="19"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="F7" s="22"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="21"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="32">
-        <v>52</v>
-      </c>
-      <c r="E4" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="27" t="s">
+      <c r="D11" s="18">
+        <v>96</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="21" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="37"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="35" t="s">
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="21"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="19"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="22"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="21"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="22"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="6"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="37"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="6"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="9"/>
-    </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="B17" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="22" t="s">
+      <c r="C17" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="4">
-        <v>96</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="6"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="9"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="6" t="s">
+      <c r="D17" s="18">
+        <v>137</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="9"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="4">
-        <v>137</v>
-      </c>
-      <c r="E17" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="4"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="18"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="21"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
+      <c r="A19" s="19"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="24"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="30" t="s">
+      <c r="D19" s="19"/>
+      <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="9"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="25" t="s">
+      <c r="C20" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="6">
         <v>184</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="16" t="s">
+      <c r="F20" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="17">
+        <v>209</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="10">
-        <v>209</v>
-      </c>
-      <c r="E21" s="31" t="s">
+      <c r="F21" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="19"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F21" s="27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F22" s="9"/>
+      <c r="F22" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
     <mergeCell ref="D21:D22"/>
     <mergeCell ref="C21:C22"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
     <mergeCell ref="D11:D13"/>
     <mergeCell ref="F11:F13"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
     <mergeCell ref="D14:D16"/>
     <mergeCell ref="F14:F16"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="D8:D10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="A8:A10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="C11:C13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added Facility Floor 1
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5D9E8E-AD57-46D6-ACC0-FED8FECCBCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6135" yWindow="1365" windowWidth="21585" windowHeight="13440" activeTab="1" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="6135" yWindow="1365" windowWidth="21585" windowHeight="13440" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -393,6 +393,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -402,28 +405,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -438,8 +432,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,7 +816,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="31" t="s">
         <v>4</v>
       </c>
     </row>
@@ -838,7 +838,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="21"/>
+      <c r="F4" s="31"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -861,7 +861,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="21"/>
+      <c r="F5" s="31"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -884,7 +884,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="21"/>
+      <c r="F6" s="31"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -907,7 +907,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="21"/>
+      <c r="F7" s="31"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -930,7 +930,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="21"/>
+      <c r="F8" s="31"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -953,7 +953,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="21"/>
+      <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -976,7 +976,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="21"/>
+      <c r="F10" s="31"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -999,7 +999,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="21"/>
+      <c r="F11" s="31"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1022,7 +1022,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="21"/>
+      <c r="F12" s="31"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1045,7 +1045,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="21"/>
+      <c r="F13" s="31"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1068,7 +1068,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="21"/>
+      <c r="F14" s="31"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1091,7 +1091,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="21"/>
+      <c r="F15" s="31"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1114,7 +1114,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="21"/>
+      <c r="F16" s="31"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1137,7 +1137,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="21"/>
+      <c r="F17" s="31"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1160,7 +1160,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="21"/>
+      <c r="F18" s="31"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1183,7 +1183,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="21"/>
+      <c r="F19" s="31"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1206,7 +1206,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="21"/>
+      <c r="F20" s="31"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1229,7 +1229,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="21"/>
+      <c r="F21" s="31"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -3022,10 +3022,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="17"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3040,214 +3040,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="21" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="18">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="30" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="18"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="19"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="21"/>
+      <c r="F5" s="31"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="18"/>
+      <c r="A6" s="19"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="19"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="21"/>
+      <c r="F6" s="31"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="19"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="22"/>
+      <c r="F7" s="32"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="31" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="18"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="21"/>
+      <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="19"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="22"/>
+      <c r="F10" s="32"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="19">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="31" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="18"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="19"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="21"/>
+      <c r="F12" s="31"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="19"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="20"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="22"/>
+      <c r="F13" s="32"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="31" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="18"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="19"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="21"/>
+      <c r="F15" s="31"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="19"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="20"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="22"/>
+      <c r="F16" s="32"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="18" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="19">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="31" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="18"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="18"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="19"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="21"/>
+      <c r="F18" s="31"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="19"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="20"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="22"/>
+      <c r="F19" s="32"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3270,55 +3270,37 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="21" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="18">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="F21" s="30" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="19"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="19"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="20"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="22"/>
+      <c r="F22" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -3332,6 +3314,24 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added Facility Floor 2 and Melee damage offsets
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5D9E8E-AD57-46D6-ACC0-FED8FECCBCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F947B2-C332-4CDD-BD78-7ED79AFAD49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6135" yWindow="1365" windowWidth="21585" windowHeight="13440" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
     <sheet name="Shopkeeper" sheetId="2" r:id="rId2"/>
+    <sheet name="Items" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="199">
   <si>
     <t>Lv</t>
   </si>
@@ -175,6 +176,465 @@
   </si>
   <si>
     <t>Splashadia</t>
+  </si>
+  <si>
+    <t>ITEMS</t>
+  </si>
+  <si>
+    <t>First Found</t>
+  </si>
+  <si>
+    <t>Snowball</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Ripped Shoes</t>
+  </si>
+  <si>
+    <t>Foreign Coin</t>
+  </si>
+  <si>
+    <t>Chipped Diamond</t>
+  </si>
+  <si>
+    <t>Half Eaten Sandwich</t>
+  </si>
+  <si>
+    <t>Crocodile Floaty</t>
+  </si>
+  <si>
+    <t>Gold Coin</t>
+  </si>
+  <si>
+    <t>Test Tube</t>
+  </si>
+  <si>
+    <t>Scratched Coin</t>
+  </si>
+  <si>
+    <t>Facility</t>
+  </si>
+  <si>
+    <t>Gun Fragment</t>
+  </si>
+  <si>
+    <t>Seaweed</t>
+  </si>
+  <si>
+    <t>Fish Tooth</t>
+  </si>
+  <si>
+    <t>Mermaid Tail</t>
+  </si>
+  <si>
+    <t>£10 Coin</t>
+  </si>
+  <si>
+    <t>Diamond</t>
+  </si>
+  <si>
+    <t>Emerald</t>
+  </si>
+  <si>
+    <t>Old Cross</t>
+  </si>
+  <si>
+    <t>Blight</t>
+  </si>
+  <si>
+    <t>Shattered Molotov</t>
+  </si>
+  <si>
+    <t>Flame</t>
+  </si>
+  <si>
+    <t>Box of Matches</t>
+  </si>
+  <si>
+    <t>Meflame</t>
+  </si>
+  <si>
+    <t>Goat Horn</t>
+  </si>
+  <si>
+    <t>Electrical Wire</t>
+  </si>
+  <si>
+    <t>Zapao</t>
+  </si>
+  <si>
+    <t>Megust</t>
+  </si>
+  <si>
+    <t>Old Pendant</t>
+  </si>
+  <si>
+    <t>Heal</t>
+  </si>
+  <si>
+    <t>Vial of Ink</t>
+  </si>
+  <si>
+    <t>Hex</t>
+  </si>
+  <si>
+    <t>Glass Pendant</t>
+  </si>
+  <si>
+    <t>Healan</t>
+  </si>
+  <si>
+    <t>Waterproof Flamethrower</t>
+  </si>
+  <si>
+    <t>Flamadia</t>
+  </si>
+  <si>
+    <t>Ice Core</t>
+  </si>
+  <si>
+    <t>Freeze</t>
+  </si>
+  <si>
+    <t>Ice Shard</t>
+  </si>
+  <si>
+    <t>Mefreeze</t>
+  </si>
+  <si>
+    <t>Crystalised Flake</t>
+  </si>
+  <si>
+    <t>Freezan</t>
+  </si>
+  <si>
+    <t>Dented Airhorn</t>
+  </si>
+  <si>
+    <t>Gust</t>
+  </si>
+  <si>
+    <t>Cold Hairdryer</t>
+  </si>
+  <si>
+    <t>Gustan</t>
+  </si>
+  <si>
+    <t>Firecracker</t>
+  </si>
+  <si>
+    <t>Meflamao</t>
+  </si>
+  <si>
+    <t>Squid Head</t>
+  </si>
+  <si>
+    <t>Mehex</t>
+  </si>
+  <si>
+    <t>Jellyfish Tenticle</t>
+  </si>
+  <si>
+    <t>Zapadia</t>
+  </si>
+  <si>
+    <t>Dark Staff</t>
+  </si>
+  <si>
+    <t>Mehexo</t>
+  </si>
+  <si>
+    <t>Radioactive Core</t>
+  </si>
+  <si>
+    <t>Frei</t>
+  </si>
+  <si>
+    <t>Radioactive Chunk</t>
+  </si>
+  <si>
+    <t>Freila</t>
+  </si>
+  <si>
+    <t>Water Blaster 9000</t>
+  </si>
+  <si>
+    <t>Splashan</t>
+  </si>
+  <si>
+    <t>Fire Hydrant</t>
+  </si>
+  <si>
+    <t>Live Cables</t>
+  </si>
+  <si>
+    <t>Mezap</t>
+  </si>
+  <si>
+    <t>Water Balloon</t>
+  </si>
+  <si>
+    <t>Mesplash</t>
+  </si>
+  <si>
+    <t>Sharp Stick</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>Sharp Icicle</t>
+  </si>
+  <si>
+    <t>Nail Board</t>
+  </si>
+  <si>
+    <t>Ice-Axe</t>
+  </si>
+  <si>
+    <t>Ice Crossbow</t>
+  </si>
+  <si>
+    <t>Wingman</t>
+  </si>
+  <si>
+    <t>Rusty Anchor</t>
+  </si>
+  <si>
+    <t>Trident</t>
+  </si>
+  <si>
+    <t>Iron Spear</t>
+  </si>
+  <si>
+    <t>Glock-17</t>
+  </si>
+  <si>
+    <t>Royal Trident</t>
+  </si>
+  <si>
+    <t>Breach Hammer</t>
+  </si>
+  <si>
+    <t>Consumable</t>
+  </si>
+  <si>
+    <t>Thawn Bandage</t>
+  </si>
+  <si>
+    <t>Effect</t>
+  </si>
+  <si>
+    <t>+40 HP</t>
+  </si>
+  <si>
+    <t>Energy Pills</t>
+  </si>
+  <si>
+    <t>+15 STA</t>
+  </si>
+  <si>
+    <t>Worn Field Kit</t>
+  </si>
+  <si>
+    <t>+100 HP</t>
+  </si>
+  <si>
+    <t>Bottle o' Spirit</t>
+  </si>
+  <si>
+    <t>+35 STA</t>
+  </si>
+  <si>
+    <t>Medkit</t>
+  </si>
+  <si>
+    <t>+200 HP</t>
+  </si>
+  <si>
+    <t>Holy Water</t>
+  </si>
+  <si>
+    <t>+80 STA</t>
+  </si>
+  <si>
+    <t>Power Supplements</t>
+  </si>
+  <si>
+    <t>x2.5 Melee</t>
+  </si>
+  <si>
+    <t>Concentration Pills</t>
+  </si>
+  <si>
+    <t>x2.5 Skill</t>
+  </si>
+  <si>
+    <t>Overpower Capsules</t>
+  </si>
+  <si>
+    <t>x2.5 Melee/Skill</t>
+  </si>
+  <si>
+    <t>x4 Melee</t>
+  </si>
+  <si>
+    <t>x4 Skill</t>
+  </si>
+  <si>
+    <t>Concentration Pills X</t>
+  </si>
+  <si>
+    <t>Power Supplements X</t>
+  </si>
+  <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Bless</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Wind</t>
+  </si>
+  <si>
+    <t>Curse</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>Suction Device</t>
+  </si>
+  <si>
+    <t>Gustadia</t>
+  </si>
+  <si>
+    <t>Bag of Powdered Snow</t>
+  </si>
+  <si>
+    <t>Beam Saber</t>
+  </si>
+  <si>
+    <t>Acid Injected Sword</t>
+  </si>
+  <si>
+    <t>Glass Shard</t>
+  </si>
+  <si>
+    <t>Screwdriver</t>
+  </si>
+  <si>
+    <t>Prototype Heat Rod</t>
+  </si>
+  <si>
+    <t>Glacier F3 Key</t>
+  </si>
+  <si>
+    <t>Glacier F5 Key</t>
+  </si>
+  <si>
+    <t>Atlantis F2 Key</t>
+  </si>
+  <si>
+    <t>Atlantis F4 Key</t>
+  </si>
+  <si>
+    <t>Atlantis F5 Key A</t>
+  </si>
+  <si>
+    <t>Atlantis F5 Key B</t>
+  </si>
+  <si>
+    <t>Facility F3 Key</t>
+  </si>
+  <si>
+    <t>Facility F5 Key A</t>
+  </si>
+  <si>
+    <t>Facility F5 Key B</t>
+  </si>
+  <si>
+    <t>Facility F5 Key C</t>
+  </si>
+  <si>
+    <t>Battery Reserve</t>
+  </si>
+  <si>
+    <t>Mezapao</t>
+  </si>
+  <si>
+    <t>Reactor Heart</t>
+  </si>
+  <si>
+    <t>Freiladia</t>
+  </si>
+  <si>
+    <t>Cracked Syringe</t>
+  </si>
+  <si>
+    <t>Holy Cross</t>
+  </si>
+  <si>
+    <t>Blighta</t>
+  </si>
+  <si>
+    <t>Ruby</t>
+  </si>
+  <si>
+    <t>Portable Mini Cannon</t>
+  </si>
+  <si>
+    <t>Flamao</t>
+  </si>
+  <si>
+    <t>Enchanted Pendant</t>
+  </si>
+  <si>
+    <t>Healadia</t>
+  </si>
+  <si>
+    <t>Potion of Instant Health</t>
+  </si>
+  <si>
+    <t>+350 HP</t>
+  </si>
+  <si>
+    <t>Potion of Mutated Souls</t>
+  </si>
+  <si>
+    <t>+150 STA</t>
+  </si>
+  <si>
+    <t>Barrier</t>
+  </si>
+  <si>
+    <t>Nul next ATK</t>
+  </si>
+  <si>
+    <t>+999 HP</t>
+  </si>
+  <si>
+    <t>+60 HP</t>
+  </si>
+  <si>
+    <t>+150 HP</t>
   </si>
 </sst>
 </file>
@@ -213,7 +673,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -232,8 +692,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -345,11 +823,128 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -393,53 +988,161 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,7 +1519,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="31" t="s">
+      <c r="F3" s="42" t="s">
         <v>4</v>
       </c>
     </row>
@@ -838,7 +1541,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="31"/>
+      <c r="F4" s="42"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -861,7 +1564,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="31"/>
+      <c r="F5" s="42"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -884,7 +1587,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="31"/>
+      <c r="F6" s="42"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -907,7 +1610,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="31"/>
+      <c r="F7" s="42"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -930,7 +1633,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="31"/>
+      <c r="F8" s="42"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -953,7 +1656,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -976,7 +1679,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="31"/>
+      <c r="F10" s="42"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -999,7 +1702,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="31"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1022,7 +1725,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="31"/>
+      <c r="F12" s="42"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1045,7 +1748,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="31"/>
+      <c r="F13" s="42"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1068,7 +1771,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="31"/>
+      <c r="F14" s="42"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1091,7 +1794,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="31"/>
+      <c r="F15" s="42"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1114,7 +1817,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="31"/>
+      <c r="F16" s="42"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1137,7 +1840,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="31"/>
+      <c r="F17" s="42"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1160,7 +1863,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="31"/>
+      <c r="F18" s="42"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1183,7 +1886,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="31"/>
+      <c r="F19" s="42"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1206,7 +1909,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="31"/>
+      <c r="F20" s="42"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1229,7 +1932,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="31"/>
+      <c r="F21" s="42"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -3022,10 +3725,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="17"/>
+      <c r="B3" s="57"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3040,214 +3743,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="43">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="46" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="19"/>
+      <c r="A5" s="44"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="31"/>
+      <c r="F5" s="42"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="19"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="44"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="31"/>
+      <c r="F6" s="42"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="20"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="20"/>
+      <c r="A7" s="45"/>
+      <c r="B7" s="51"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="45"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="32"/>
+      <c r="F7" s="47"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="44" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="42" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="19"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="20"/>
+      <c r="A10" s="45"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="45"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="32"/>
+      <c r="F10" s="47"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="44">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="42" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="19"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="44"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="31"/>
+      <c r="F12" s="42"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="20"/>
+      <c r="A13" s="45"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="45"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="32"/>
+      <c r="F13" s="47"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="44" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="19"/>
+      <c r="A15" s="44"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="44"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="31"/>
+      <c r="F15" s="42"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="20"/>
+      <c r="A16" s="45"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="45"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="32"/>
+      <c r="F16" s="47"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="44">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="31" t="s">
+      <c r="F17" s="42" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="19"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="44"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="31"/>
+      <c r="F18" s="42"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="20"/>
+      <c r="A19" s="45"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="45"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="32"/>
+      <c r="F19" s="47"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3270,37 +3973,55 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="18">
+      <c r="D21" s="43">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="30" t="s">
+      <c r="F21" s="46" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="20"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="20"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="45"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="32"/>
+      <c r="F22" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -3314,26 +4035,1541 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36AA0E8-4612-49A3-9CD4-2D5734B3DCEA}">
+  <dimension ref="A1:W34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" customWidth="1"/>
+    <col min="6" max="6" width="3.140625" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="22.5703125" customWidth="1"/>
+    <col min="13" max="13" width="25.140625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.140625" style="1" customWidth="1"/>
+    <col min="15" max="16" width="9.140625" style="1"/>
+    <col min="17" max="17" width="22.5703125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="24.85546875" customWidth="1"/>
+    <col min="20" max="20" width="3" customWidth="1"/>
+    <col min="21" max="21" width="12.7109375" customWidth="1"/>
+    <col min="22" max="22" width="12.85546875" customWidth="1"/>
+    <col min="23" max="23" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="37"/>
+    </row>
+    <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="41"/>
+      <c r="C3" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="41"/>
+      <c r="G3" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="J3" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="K3" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="M3" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="39"/>
+      <c r="O3" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="P3" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q3" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="S3" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="T3" s="41"/>
+      <c r="U3" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="V3" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="W3" s="35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4" s="25">
+        <v>1</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" s="25">
+        <v>1</v>
+      </c>
+      <c r="G4" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="25">
+        <v>44</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="K4" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="M4" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="N4" s="25">
+        <v>1</v>
+      </c>
+      <c r="O4" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="25">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="S4" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="T4" s="25">
+        <v>1</v>
+      </c>
+      <c r="U4" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="V4" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="W4" s="26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="62">
+        <v>1</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="58" t="s">
+        <v>183</v>
+      </c>
+      <c r="F5" s="59">
+        <v>3</v>
+      </c>
+      <c r="G5" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="I5" s="59">
+        <v>70</v>
+      </c>
+      <c r="J5" s="59" t="s">
+        <v>151</v>
+      </c>
+      <c r="K5" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="N5" s="1">
+        <v>1</v>
+      </c>
+      <c r="O5" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P5" s="1">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="S5" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="T5" s="62">
+        <v>1</v>
+      </c>
+      <c r="U5" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V5" s="67" t="s">
+        <v>131</v>
+      </c>
+      <c r="W5" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="62">
+        <v>1</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="62">
+        <v>1</v>
+      </c>
+      <c r="G6" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" s="62">
+        <v>44</v>
+      </c>
+      <c r="J6" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1</v>
+      </c>
+      <c r="O6" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="1">
+        <v>39</v>
+      </c>
+      <c r="Q6" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="S6" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="T6" s="62">
+        <v>2</v>
+      </c>
+      <c r="U6" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V6" s="67" t="s">
+        <v>133</v>
+      </c>
+      <c r="W6" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="62">
+        <v>1</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="62">
+        <v>2</v>
+      </c>
+      <c r="G7" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="I7" s="62">
+        <v>35</v>
+      </c>
+      <c r="J7" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="N7" s="1">
+        <v>2</v>
+      </c>
+      <c r="O7" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P7" s="1">
+        <v>21</v>
+      </c>
+      <c r="Q7" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="S7" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="T7" s="62">
+        <v>2</v>
+      </c>
+      <c r="U7" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V7" s="67" t="s">
+        <v>135</v>
+      </c>
+      <c r="W7" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="62">
+        <v>1</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" s="62">
+        <v>4</v>
+      </c>
+      <c r="G8" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="62" t="s">
+        <v>101</v>
+      </c>
+      <c r="I8" s="62">
+        <v>56</v>
+      </c>
+      <c r="J8" s="62" t="s">
+        <v>155</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="N8" s="1">
+        <v>2</v>
+      </c>
+      <c r="O8" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P8" s="1">
+        <v>56</v>
+      </c>
+      <c r="Q8" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="S8" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="T8" s="62">
+        <v>3</v>
+      </c>
+      <c r="U8" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V8" s="67" t="s">
+        <v>137</v>
+      </c>
+      <c r="W8" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="62">
+        <v>1</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="F9" s="62">
+        <v>2</v>
+      </c>
+      <c r="G9" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="62" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9" s="62">
+        <v>32</v>
+      </c>
+      <c r="J9" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M9" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="N9" s="1">
+        <v>2</v>
+      </c>
+      <c r="O9" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P9" s="1">
+        <v>73</v>
+      </c>
+      <c r="Q9" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="S9" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="T9" s="62">
+        <v>3</v>
+      </c>
+      <c r="U9" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V9" s="67" t="s">
+        <v>139</v>
+      </c>
+      <c r="W9" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="62">
+        <v>1</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" s="62">
+        <v>3</v>
+      </c>
+      <c r="G10" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="62" t="s">
+        <v>74</v>
+      </c>
+      <c r="I10" s="62">
+        <v>65</v>
+      </c>
+      <c r="J10" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="N10" s="1">
+        <v>3</v>
+      </c>
+      <c r="O10" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P10" s="1">
+        <v>36</v>
+      </c>
+      <c r="Q10" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="S10" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="T10" s="62">
+        <v>3</v>
+      </c>
+      <c r="U10" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V10" s="62" t="s">
+        <v>141</v>
+      </c>
+      <c r="W10" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="62">
+        <v>2</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="F11" s="62">
+        <v>4</v>
+      </c>
+      <c r="G11" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="62" t="s">
+        <v>179</v>
+      </c>
+      <c r="I11" s="62">
+        <v>52</v>
+      </c>
+      <c r="J11" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="N11" s="1">
+        <v>3</v>
+      </c>
+      <c r="O11" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P11" s="1">
+        <v>46</v>
+      </c>
+      <c r="Q11" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="S11" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="T11" s="62">
+        <v>3</v>
+      </c>
+      <c r="U11" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V11" s="62" t="s">
+        <v>143</v>
+      </c>
+      <c r="W11" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="62">
+        <v>2</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="62">
+        <v>4</v>
+      </c>
+      <c r="G12" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="62" t="s">
+        <v>99</v>
+      </c>
+      <c r="I12" s="62">
+        <v>105</v>
+      </c>
+      <c r="J12" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="N12" s="1">
+        <v>3</v>
+      </c>
+      <c r="O12" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P12" s="1">
+        <v>71</v>
+      </c>
+      <c r="Q12" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="S12" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="T12" s="62">
+        <v>4</v>
+      </c>
+      <c r="U12" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V12" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="W12" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="62">
+        <v>2</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="62">
+        <v>1</v>
+      </c>
+      <c r="G13" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="62">
+        <v>40</v>
+      </c>
+      <c r="J13" s="62" t="s">
+        <v>152</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M13" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="N13" s="1">
+        <v>3</v>
+      </c>
+      <c r="O13" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P13" s="1">
+        <v>78</v>
+      </c>
+      <c r="Q13" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="S13" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="T13" s="62">
+        <v>4</v>
+      </c>
+      <c r="U13" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V13" s="62" t="s">
+        <v>146</v>
+      </c>
+      <c r="W13" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="62">
+        <v>2</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="62">
+        <v>2</v>
+      </c>
+      <c r="G14" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="62" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" s="62">
+        <v>32</v>
+      </c>
+      <c r="J14" s="62" t="s">
+        <v>152</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="N14" s="1">
+        <v>3</v>
+      </c>
+      <c r="O14" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P14" s="1">
+        <v>86</v>
+      </c>
+      <c r="Q14" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="S14" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="T14" s="62">
+        <v>4</v>
+      </c>
+      <c r="U14" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V14" s="62" t="s">
+        <v>147</v>
+      </c>
+      <c r="W14" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="62">
+        <v>2</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="58" t="s">
+        <v>186</v>
+      </c>
+      <c r="F15" s="59">
+        <v>3</v>
+      </c>
+      <c r="G15" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="59" t="s">
+        <v>187</v>
+      </c>
+      <c r="I15" s="59">
+        <v>65</v>
+      </c>
+      <c r="J15" s="59" t="s">
+        <v>152</v>
+      </c>
+      <c r="K15" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="M15" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="N15" s="1">
+        <v>3</v>
+      </c>
+      <c r="O15" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P15" s="1">
+        <v>109</v>
+      </c>
+      <c r="Q15" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="S15" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="T15" s="62">
+        <v>4</v>
+      </c>
+      <c r="U15" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V15" s="67" t="s">
+        <v>191</v>
+      </c>
+      <c r="W15" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="62">
+        <v>3</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" s="62">
+        <v>4</v>
+      </c>
+      <c r="G16" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="62" t="s">
+        <v>95</v>
+      </c>
+      <c r="I16" s="62">
+        <v>52</v>
+      </c>
+      <c r="J16" s="62" t="s">
+        <v>152</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M16" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="N16" s="1">
+        <v>4</v>
+      </c>
+      <c r="O16" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P16" s="1">
+        <v>67</v>
+      </c>
+      <c r="Q16" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="S16" s="58" t="s">
+        <v>192</v>
+      </c>
+      <c r="T16" s="62">
+        <v>4</v>
+      </c>
+      <c r="U16" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="V16" s="66" t="s">
+        <v>193</v>
+      </c>
+      <c r="W16" s="61" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="62">
+        <v>3</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="62">
+        <v>4</v>
+      </c>
+      <c r="G17" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="I17" s="62">
+        <v>105</v>
+      </c>
+      <c r="J17" s="62" t="s">
+        <v>152</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M17" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="N17" s="1">
+        <v>4</v>
+      </c>
+      <c r="O17" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P17" s="1">
+        <v>103</v>
+      </c>
+      <c r="Q17" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="S17" s="63" t="s">
+        <v>194</v>
+      </c>
+      <c r="T17" s="20">
+        <v>5</v>
+      </c>
+      <c r="U17" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="V17" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="W17" s="64" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="62">
+        <v>3</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" s="62">
+        <v>1</v>
+      </c>
+      <c r="G18" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="62" t="s">
+        <v>85</v>
+      </c>
+      <c r="I18" s="62">
+        <v>36</v>
+      </c>
+      <c r="J18" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="N18" s="1">
+        <v>4</v>
+      </c>
+      <c r="O18" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P18" s="1">
+        <v>139</v>
+      </c>
+      <c r="Q18" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="62">
+        <v>3</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="62">
+        <v>2</v>
+      </c>
+      <c r="G19" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="62" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" s="62">
+        <v>29</v>
+      </c>
+      <c r="J19" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M19" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="N19" s="1">
+        <v>4</v>
+      </c>
+      <c r="O19" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="P19" s="1">
+        <v>165</v>
+      </c>
+      <c r="Q19" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="62">
+        <v>3</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="62">
+        <v>3</v>
+      </c>
+      <c r="G20" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="62" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="62">
+        <v>60</v>
+      </c>
+      <c r="J20" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M20" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="N20" s="20">
+        <v>5</v>
+      </c>
+      <c r="O20" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="P20" s="20">
+        <v>214</v>
+      </c>
+      <c r="Q20" s="21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="62">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="F21" s="62">
+        <v>4</v>
+      </c>
+      <c r="G21" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="62">
+        <v>95</v>
+      </c>
+      <c r="J21" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="K21" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="62">
+        <v>3</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="62">
+        <v>3</v>
+      </c>
+      <c r="G22" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="62" t="s">
+        <v>103</v>
+      </c>
+      <c r="I22" s="62">
+        <v>98</v>
+      </c>
+      <c r="J22" s="62" t="s">
+        <v>158</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="62">
+        <v>3</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F23" s="62">
+        <v>4</v>
+      </c>
+      <c r="G23" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="62" t="s">
+        <v>105</v>
+      </c>
+      <c r="I23" s="62">
+        <v>174</v>
+      </c>
+      <c r="J23" s="62" t="s">
+        <v>158</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="62">
+        <v>3</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="58" t="s">
+        <v>180</v>
+      </c>
+      <c r="F24" s="59">
+        <v>5</v>
+      </c>
+      <c r="G24" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="59" t="s">
+        <v>181</v>
+      </c>
+      <c r="I24" s="59">
+        <v>269</v>
+      </c>
+      <c r="J24" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="K24" s="61" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B25" s="62">
+        <v>3</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="62">
+        <v>3</v>
+      </c>
+      <c r="G25" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="I25" s="67" t="s">
+        <v>197</v>
+      </c>
+      <c r="J25" s="62" t="s">
+        <v>159</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26" s="62">
+        <v>3</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="F26" s="62">
+        <v>4</v>
+      </c>
+      <c r="G26" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="I26" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="J26" s="62" t="s">
+        <v>159</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="62">
+        <v>3</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="58" t="s">
+        <v>188</v>
+      </c>
+      <c r="F27" s="59">
+        <v>5</v>
+      </c>
+      <c r="G27" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="59" t="s">
+        <v>189</v>
+      </c>
+      <c r="I27" s="66" t="s">
+        <v>196</v>
+      </c>
+      <c r="J27" s="59" t="s">
+        <v>159</v>
+      </c>
+      <c r="K27" s="61" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="62">
+        <v>4</v>
+      </c>
+      <c r="C28" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" s="62">
+        <v>2</v>
+      </c>
+      <c r="G28" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="62" t="s">
+        <v>112</v>
+      </c>
+      <c r="I28" s="62">
+        <v>29</v>
+      </c>
+      <c r="J28" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="62">
+        <v>5</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" s="62">
+        <v>3</v>
+      </c>
+      <c r="G29" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="62" t="s">
+        <v>107</v>
+      </c>
+      <c r="I29" s="62">
+        <v>60</v>
+      </c>
+      <c r="J29" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="62">
+        <v>5</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="62">
+        <v>4</v>
+      </c>
+      <c r="G30" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="62" t="s">
+        <v>45</v>
+      </c>
+      <c r="I30" s="62">
+        <v>95</v>
+      </c>
+      <c r="J30" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="B31" s="20">
+        <v>5</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F31" s="62">
+        <v>1</v>
+      </c>
+      <c r="G31" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="62" t="s">
+        <v>91</v>
+      </c>
+      <c r="I31" s="62">
+        <v>36</v>
+      </c>
+      <c r="J31" s="62" t="s">
+        <v>154</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="E32" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F32" s="62">
+        <v>2</v>
+      </c>
+      <c r="G32" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="62" t="s">
+        <v>75</v>
+      </c>
+      <c r="I32" s="62">
+        <v>29</v>
+      </c>
+      <c r="J32" s="62" t="s">
+        <v>154</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="5:11" x14ac:dyDescent="0.25">
+      <c r="E33" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="F33" s="62">
+        <v>3</v>
+      </c>
+      <c r="G33" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="62" t="s">
+        <v>93</v>
+      </c>
+      <c r="I33" s="62">
+        <v>60</v>
+      </c>
+      <c r="J33" s="62" t="s">
+        <v>154</v>
+      </c>
+      <c r="K33" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="5:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E34" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="F34" s="20">
+        <v>4</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I34" s="20">
+        <v>95</v>
+      </c>
+      <c r="J34" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="K34" s="21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E4:K34">
+    <sortCondition ref="J4:J34"/>
+    <sortCondition ref="F4:F34"/>
+    <sortCondition ref="I4:I34"/>
+  </sortState>
+  <mergeCells count="5">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="S3:T3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Colours! Added increases Melee/Magic damage from Melee attributes
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F947B2-C332-4CDD-BD78-7ED79AFAD49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABAF0DD-C8DB-4D62-BC3E-1BC96EA4103E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-26535" yWindow="585" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -944,7 +944,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1048,24 +1048,39 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1075,74 +1090,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1519,7 +1498,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="42" t="s">
+      <c r="F3" s="46" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1541,7 +1520,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="42"/>
+      <c r="F4" s="46"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1564,7 +1543,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="42"/>
+      <c r="F5" s="46"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1587,7 +1566,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="42"/>
+      <c r="F6" s="46"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1610,7 +1589,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="42"/>
+      <c r="F7" s="46"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1633,7 +1612,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="42"/>
+      <c r="F8" s="46"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1656,7 +1635,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="42"/>
+      <c r="F9" s="46"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1679,7 +1658,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="42"/>
+      <c r="F10" s="46"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1702,7 +1681,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="42"/>
+      <c r="F11" s="46"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1725,7 +1704,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="42"/>
+      <c r="F12" s="46"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1748,7 +1727,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="42"/>
+      <c r="F13" s="46"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1771,7 +1750,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="42"/>
+      <c r="F14" s="46"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1794,7 +1773,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="42"/>
+      <c r="F15" s="46"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1817,7 +1796,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="42"/>
+      <c r="F16" s="46"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1840,7 +1819,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="42"/>
+      <c r="F17" s="46"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1863,7 +1842,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="42"/>
+      <c r="F18" s="46"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1886,7 +1865,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="42"/>
+      <c r="F19" s="46"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1909,7 +1888,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="42"/>
+      <c r="F20" s="46"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1932,7 +1911,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="42"/>
+      <c r="F21" s="46"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -3725,10 +3704,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="57"/>
+      <c r="B3" s="47"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3743,214 +3722,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="43">
+      <c r="D4" s="48">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="46" t="s">
+      <c r="F4" s="60" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="44"/>
-      <c r="B5" s="53"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="44"/>
+      <c r="A5" s="49"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="49"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="42"/>
+      <c r="F5" s="46"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
-      <c r="B6" s="53"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="44"/>
+      <c r="A6" s="49"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="49"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="42"/>
+      <c r="F6" s="46"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="45"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="45"/>
+      <c r="A7" s="50"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="50"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="47"/>
+      <c r="F7" s="61"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D8" s="49" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="42" t="s">
+      <c r="F8" s="46" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="44"/>
+      <c r="A9" s="49"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="58"/>
+      <c r="D9" s="49"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="42"/>
+      <c r="F9" s="46"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="45"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="45"/>
+      <c r="A10" s="50"/>
+      <c r="B10" s="50"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="50"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="47"/>
+      <c r="F10" s="61"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="49">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="42" t="s">
+      <c r="F11" s="46" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="44"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="52"/>
-      <c r="D12" s="44"/>
+      <c r="A12" s="49"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="49"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="42"/>
+      <c r="F12" s="46"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="45"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="45"/>
+      <c r="A13" s="50"/>
+      <c r="B13" s="50"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="50"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="47"/>
+      <c r="F13" s="61"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="44" t="s">
+      <c r="D14" s="49" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="42" t="s">
+      <c r="F14" s="46" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
-      <c r="B15" s="44"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="44"/>
+      <c r="A15" s="49"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="49"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="42"/>
+      <c r="F15" s="46"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="45"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="56"/>
-      <c r="D16" s="45"/>
+      <c r="A16" s="50"/>
+      <c r="B16" s="50"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="50"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="47"/>
+      <c r="F16" s="61"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="44">
+      <c r="D17" s="49">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="42" t="s">
+      <c r="F17" s="46" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
-      <c r="B18" s="44"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="44"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="49"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="42"/>
+      <c r="F18" s="46"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="45"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="45"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="50"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="50"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="47"/>
+      <c r="F19" s="61"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3973,55 +3952,37 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="43">
+      <c r="D21" s="48">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="46" t="s">
+      <c r="F21" s="60" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="45"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="45"/>
+      <c r="A22" s="50"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="50"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="47"/>
+      <c r="F22" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -4035,6 +3996,24 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4067,24 +4046,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="37"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="41"/>
+      <c r="B3" s="43"/>
       <c r="C3" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="40" t="s">
+      <c r="E3" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="41"/>
+      <c r="F3" s="43"/>
       <c r="G3" s="34" t="s">
         <v>8</v>
       </c>
@@ -4100,10 +4079,10 @@
       <c r="K3" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="M3" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="39"/>
+      <c r="N3" s="45"/>
       <c r="O3" s="22" t="s">
         <v>8</v>
       </c>
@@ -4113,10 +4092,10 @@
       <c r="Q3" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="S3" s="40" t="s">
+      <c r="S3" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="41"/>
+      <c r="T3" s="43"/>
       <c r="U3" s="34" t="s">
         <v>8</v>
       </c>
@@ -4193,31 +4172,31 @@
       <c r="A5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="62">
+      <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="58" t="s">
+      <c r="E5" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="F5" s="59">
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="60" t="s">
+      <c r="G5" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="59" t="s">
+      <c r="H5" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I5" s="59">
+      <c r="I5" s="1">
         <v>70</v>
       </c>
-      <c r="J5" s="59" t="s">
+      <c r="J5" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="K5" s="61" t="s">
+      <c r="K5" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M5" s="17" t="s">
@@ -4238,13 +4217,13 @@
       <c r="S5" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="T5" s="62">
+      <c r="T5" s="1">
         <v>1</v>
       </c>
-      <c r="U5" s="65" t="s">
+      <c r="U5" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V5" s="67" t="s">
+      <c r="V5" s="39" t="s">
         <v>131</v>
       </c>
       <c r="W5" s="18" t="s">
@@ -4255,7 +4234,7 @@
       <c r="A6" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="62">
+      <c r="B6" s="1">
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
@@ -4264,19 +4243,19 @@
       <c r="E6" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="62">
+      <c r="F6" s="1">
         <v>1</v>
       </c>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="62" t="s">
+      <c r="H6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="I6" s="62">
+      <c r="I6" s="1">
         <v>44</v>
       </c>
-      <c r="J6" s="62" t="s">
+      <c r="J6" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K6" s="18" t="s">
@@ -4300,13 +4279,13 @@
       <c r="S6" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="T6" s="62">
+      <c r="T6" s="1">
         <v>2</v>
       </c>
-      <c r="U6" s="65" t="s">
+      <c r="U6" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V6" s="67" t="s">
+      <c r="V6" s="39" t="s">
         <v>133</v>
       </c>
       <c r="W6" s="18" t="s">
@@ -4317,7 +4296,7 @@
       <c r="A7" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="62">
+      <c r="B7" s="1">
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -4326,19 +4305,19 @@
       <c r="E7" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="62">
+      <c r="F7" s="1">
         <v>2</v>
       </c>
-      <c r="G7" s="60" t="s">
+      <c r="G7" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="62" t="s">
+      <c r="H7" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I7" s="62">
+      <c r="I7" s="1">
         <v>35</v>
       </c>
-      <c r="J7" s="62" t="s">
+      <c r="J7" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K7" s="18" t="s">
@@ -4362,13 +4341,13 @@
       <c r="S7" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="T7" s="62">
+      <c r="T7" s="1">
         <v>2</v>
       </c>
-      <c r="U7" s="65" t="s">
+      <c r="U7" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V7" s="67" t="s">
+      <c r="V7" s="39" t="s">
         <v>135</v>
       </c>
       <c r="W7" s="18" t="s">
@@ -4379,7 +4358,7 @@
       <c r="A8" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="62">
+      <c r="B8" s="1">
         <v>1</v>
       </c>
       <c r="C8" s="18" t="s">
@@ -4388,19 +4367,19 @@
       <c r="E8" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="62">
+      <c r="F8" s="1">
         <v>4</v>
       </c>
-      <c r="G8" s="60" t="s">
+      <c r="G8" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="62" t="s">
+      <c r="H8" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="62">
+      <c r="I8" s="1">
         <v>56</v>
       </c>
-      <c r="J8" s="62" t="s">
+      <c r="J8" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K8" s="18" t="s">
@@ -4424,13 +4403,13 @@
       <c r="S8" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="T8" s="62">
+      <c r="T8" s="1">
         <v>3</v>
       </c>
-      <c r="U8" s="65" t="s">
+      <c r="U8" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V8" s="67" t="s">
+      <c r="V8" s="39" t="s">
         <v>137</v>
       </c>
       <c r="W8" s="18" t="s">
@@ -4441,7 +4420,7 @@
       <c r="A9" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="62">
+      <c r="B9" s="1">
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
@@ -4450,19 +4429,19 @@
       <c r="E9" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="F9" s="62">
+      <c r="F9" s="1">
         <v>2</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="62" t="s">
+      <c r="H9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="1">
         <v>32</v>
       </c>
-      <c r="J9" s="62" t="s">
+      <c r="J9" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K9" s="18" t="s">
@@ -4486,13 +4465,13 @@
       <c r="S9" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="T9" s="62">
+      <c r="T9" s="1">
         <v>3</v>
       </c>
-      <c r="U9" s="65" t="s">
+      <c r="U9" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V9" s="67" t="s">
+      <c r="V9" s="39" t="s">
         <v>139</v>
       </c>
       <c r="W9" s="18" t="s">
@@ -4503,7 +4482,7 @@
       <c r="A10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="62">
+      <c r="B10" s="1">
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
@@ -4512,19 +4491,19 @@
       <c r="E10" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="62">
+      <c r="F10" s="1">
         <v>3</v>
       </c>
-      <c r="G10" s="60" t="s">
+      <c r="G10" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="62" t="s">
+      <c r="H10" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="62">
+      <c r="I10" s="1">
         <v>65</v>
       </c>
-      <c r="J10" s="62" t="s">
+      <c r="J10" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K10" s="18" t="s">
@@ -4548,13 +4527,13 @@
       <c r="S10" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="T10" s="62">
+      <c r="T10" s="1">
         <v>3</v>
       </c>
-      <c r="U10" s="65" t="s">
+      <c r="U10" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V10" s="62" t="s">
+      <c r="V10" s="1" t="s">
         <v>141</v>
       </c>
       <c r="W10" s="18" t="s">
@@ -4565,7 +4544,7 @@
       <c r="A11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="62">
+      <c r="B11" s="1">
         <v>2</v>
       </c>
       <c r="C11" s="18" t="s">
@@ -4574,19 +4553,19 @@
       <c r="E11" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="F11" s="62">
+      <c r="F11" s="1">
         <v>4</v>
       </c>
-      <c r="G11" s="60" t="s">
+      <c r="G11" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="62" t="s">
+      <c r="H11" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I11" s="62">
+      <c r="I11" s="1">
         <v>52</v>
       </c>
-      <c r="J11" s="62" t="s">
+      <c r="J11" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K11" s="18" t="s">
@@ -4610,13 +4589,13 @@
       <c r="S11" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="T11" s="62">
+      <c r="T11" s="1">
         <v>3</v>
       </c>
-      <c r="U11" s="65" t="s">
+      <c r="U11" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V11" s="62" t="s">
+      <c r="V11" s="1" t="s">
         <v>143</v>
       </c>
       <c r="W11" s="18" t="s">
@@ -4627,7 +4606,7 @@
       <c r="A12" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="62">
+      <c r="B12" s="1">
         <v>2</v>
       </c>
       <c r="C12" s="18" t="s">
@@ -4636,19 +4615,19 @@
       <c r="E12" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="F12" s="62">
+      <c r="F12" s="1">
         <v>4</v>
       </c>
-      <c r="G12" s="60" t="s">
+      <c r="G12" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="62" t="s">
+      <c r="H12" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="I12" s="62">
+      <c r="I12" s="1">
         <v>105</v>
       </c>
-      <c r="J12" s="62" t="s">
+      <c r="J12" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K12" s="18" t="s">
@@ -4672,13 +4651,13 @@
       <c r="S12" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="T12" s="62">
+      <c r="T12" s="1">
         <v>4</v>
       </c>
-      <c r="U12" s="65" t="s">
+      <c r="U12" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V12" s="68" t="s">
+      <c r="V12" s="40" t="s">
         <v>145</v>
       </c>
       <c r="W12" s="18" t="s">
@@ -4689,7 +4668,7 @@
       <c r="A13" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="62">
+      <c r="B13" s="1">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="s">
@@ -4698,19 +4677,19 @@
       <c r="E13" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="62">
+      <c r="F13" s="1">
         <v>1</v>
       </c>
-      <c r="G13" s="60" t="s">
+      <c r="G13" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="62" t="s">
+      <c r="H13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I13" s="62">
+      <c r="I13" s="1">
         <v>40</v>
       </c>
-      <c r="J13" s="62" t="s">
+      <c r="J13" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K13" s="18" t="s">
@@ -4734,13 +4713,13 @@
       <c r="S13" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="T13" s="62">
+      <c r="T13" s="1">
         <v>4</v>
       </c>
-      <c r="U13" s="65" t="s">
+      <c r="U13" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V13" s="62" t="s">
+      <c r="V13" s="1" t="s">
         <v>146</v>
       </c>
       <c r="W13" s="18" t="s">
@@ -4751,7 +4730,7 @@
       <c r="A14" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="62">
+      <c r="B14" s="1">
         <v>2</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -4760,19 +4739,19 @@
       <c r="E14" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="F14" s="62">
+      <c r="F14" s="1">
         <v>2</v>
       </c>
-      <c r="G14" s="60" t="s">
+      <c r="G14" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="62" t="s">
+      <c r="H14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I14" s="62">
+      <c r="I14" s="1">
         <v>32</v>
       </c>
-      <c r="J14" s="62" t="s">
+      <c r="J14" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K14" s="18" t="s">
@@ -4796,13 +4775,13 @@
       <c r="S14" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="T14" s="62">
+      <c r="T14" s="1">
         <v>4</v>
       </c>
-      <c r="U14" s="65" t="s">
+      <c r="U14" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V14" s="62" t="s">
+      <c r="V14" s="1" t="s">
         <v>147</v>
       </c>
       <c r="W14" s="18" t="s">
@@ -4813,31 +4792,31 @@
       <c r="A15" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="62">
+      <c r="B15" s="1">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="58" t="s">
+      <c r="E15" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="F15" s="59">
+      <c r="F15" s="1">
         <v>3</v>
       </c>
-      <c r="G15" s="60" t="s">
+      <c r="G15" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="59" t="s">
+      <c r="H15" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="1">
         <v>65</v>
       </c>
-      <c r="J15" s="59" t="s">
+      <c r="J15" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="K15" s="61" t="s">
+      <c r="K15" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M15" s="17" t="s">
@@ -4858,13 +4837,13 @@
       <c r="S15" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="T15" s="62">
+      <c r="T15" s="1">
         <v>4</v>
       </c>
-      <c r="U15" s="65" t="s">
+      <c r="U15" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V15" s="67" t="s">
+      <c r="V15" s="39" t="s">
         <v>191</v>
       </c>
       <c r="W15" s="18" t="s">
@@ -4875,7 +4854,7 @@
       <c r="A16" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="62">
+      <c r="B16" s="1">
         <v>3</v>
       </c>
       <c r="C16" s="18" t="s">
@@ -4884,19 +4863,19 @@
       <c r="E16" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="F16" s="62">
+      <c r="F16" s="1">
         <v>4</v>
       </c>
-      <c r="G16" s="60" t="s">
+      <c r="G16" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="62" t="s">
+      <c r="H16" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="I16" s="62">
+      <c r="I16" s="1">
         <v>52</v>
       </c>
-      <c r="J16" s="62" t="s">
+      <c r="J16" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K16" s="18" t="s">
@@ -4917,19 +4896,19 @@
       <c r="Q16" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="S16" s="58" t="s">
+      <c r="S16" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="T16" s="62">
+      <c r="T16" s="1">
         <v>4</v>
       </c>
-      <c r="U16" s="65" t="s">
+      <c r="U16" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="V16" s="66" t="s">
+      <c r="V16" s="39" t="s">
         <v>193</v>
       </c>
-      <c r="W16" s="61" t="s">
+      <c r="W16" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -4937,7 +4916,7 @@
       <c r="A17" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="B17" s="62">
+      <c r="B17" s="1">
         <v>3</v>
       </c>
       <c r="C17" s="18" t="s">
@@ -4946,19 +4925,19 @@
       <c r="E17" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="F17" s="62">
+      <c r="F17" s="1">
         <v>4</v>
       </c>
-      <c r="G17" s="60" t="s">
+      <c r="G17" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="62" t="s">
+      <c r="H17" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I17" s="62">
+      <c r="I17" s="1">
         <v>105</v>
       </c>
-      <c r="J17" s="62" t="s">
+      <c r="J17" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K17" s="18" t="s">
@@ -4979,7 +4958,7 @@
       <c r="Q17" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="S17" s="63" t="s">
+      <c r="S17" s="19" t="s">
         <v>194</v>
       </c>
       <c r="T17" s="20">
@@ -4991,7 +4970,7 @@
       <c r="V17" s="20" t="s">
         <v>195</v>
       </c>
-      <c r="W17" s="64" t="s">
+      <c r="W17" s="21" t="s">
         <v>58</v>
       </c>
     </row>
@@ -4999,7 +4978,7 @@
       <c r="A18" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="B18" s="62">
+      <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
@@ -5008,19 +4987,19 @@
       <c r="E18" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="F18" s="62">
+      <c r="F18" s="1">
         <v>1</v>
       </c>
-      <c r="G18" s="60" t="s">
+      <c r="G18" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="62" t="s">
+      <c r="H18" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="I18" s="62">
+      <c r="I18" s="1">
         <v>36</v>
       </c>
-      <c r="J18" s="62" t="s">
+      <c r="J18" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K18" s="18" t="s">
@@ -5046,7 +5025,7 @@
       <c r="A19" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="B19" s="62">
+      <c r="B19" s="1">
         <v>3</v>
       </c>
       <c r="C19" s="18" t="s">
@@ -5055,19 +5034,19 @@
       <c r="E19" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="62">
+      <c r="F19" s="1">
         <v>2</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="62" t="s">
+      <c r="H19" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I19" s="62">
+      <c r="I19" s="1">
         <v>29</v>
       </c>
-      <c r="J19" s="62" t="s">
+      <c r="J19" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K19" s="18" t="s">
@@ -5093,7 +5072,7 @@
       <c r="A20" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="B20" s="62">
+      <c r="B20" s="1">
         <v>3</v>
       </c>
       <c r="C20" s="18" t="s">
@@ -5102,19 +5081,19 @@
       <c r="E20" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="62">
+      <c r="F20" s="1">
         <v>3</v>
       </c>
-      <c r="G20" s="60" t="s">
+      <c r="G20" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="62" t="s">
+      <c r="H20" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I20" s="62">
+      <c r="I20" s="1">
         <v>60</v>
       </c>
-      <c r="J20" s="62" t="s">
+      <c r="J20" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K20" s="18" t="s">
@@ -5140,7 +5119,7 @@
       <c r="A21" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="B21" s="62">
+      <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="C21" s="18" t="s">
@@ -5149,19 +5128,19 @@
       <c r="E21" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="F21" s="62">
+      <c r="F21" s="1">
         <v>4</v>
       </c>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="62" t="s">
+      <c r="H21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I21" s="62">
+      <c r="I21" s="1">
         <v>95</v>
       </c>
-      <c r="J21" s="62" t="s">
+      <c r="J21" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K21" s="18" t="s">
@@ -5172,7 +5151,7 @@
       <c r="A22" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="B22" s="62">
+      <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="18" t="s">
@@ -5181,19 +5160,19 @@
       <c r="E22" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="F22" s="62">
+      <c r="F22" s="1">
         <v>3</v>
       </c>
-      <c r="G22" s="60" t="s">
+      <c r="G22" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="62" t="s">
+      <c r="H22" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="I22" s="62">
+      <c r="I22" s="1">
         <v>98</v>
       </c>
-      <c r="J22" s="62" t="s">
+      <c r="J22" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K22" s="18" t="s">
@@ -5204,7 +5183,7 @@
       <c r="A23" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="B23" s="62">
+      <c r="B23" s="1">
         <v>3</v>
       </c>
       <c r="C23" s="18" t="s">
@@ -5213,19 +5192,19 @@
       <c r="E23" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="F23" s="62">
+      <c r="F23" s="1">
         <v>4</v>
       </c>
-      <c r="G23" s="60" t="s">
+      <c r="G23" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="62" t="s">
+      <c r="H23" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I23" s="62">
+      <c r="I23" s="1">
         <v>174</v>
       </c>
-      <c r="J23" s="62" t="s">
+      <c r="J23" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K23" s="18" t="s">
@@ -5236,31 +5215,31 @@
       <c r="A24" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="B24" s="62">
+      <c r="B24" s="1">
         <v>3</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="58" t="s">
+      <c r="E24" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="F24" s="59">
+      <c r="F24" s="1">
         <v>5</v>
       </c>
-      <c r="G24" s="60" t="s">
+      <c r="G24" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="59" t="s">
+      <c r="H24" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="I24" s="59">
+      <c r="I24" s="1">
         <v>269</v>
       </c>
-      <c r="J24" s="59" t="s">
+      <c r="J24" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K24" s="61" t="s">
+      <c r="K24" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5268,7 +5247,7 @@
       <c r="A25" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="B25" s="62">
+      <c r="B25" s="1">
         <v>3</v>
       </c>
       <c r="C25" s="18" t="s">
@@ -5277,19 +5256,19 @@
       <c r="E25" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="F25" s="62">
+      <c r="F25" s="1">
         <v>3</v>
       </c>
-      <c r="G25" s="60" t="s">
+      <c r="G25" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="62" t="s">
+      <c r="H25" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="I25" s="67" t="s">
+      <c r="I25" s="39" t="s">
         <v>197</v>
       </c>
-      <c r="J25" s="62" t="s">
+      <c r="J25" s="1" t="s">
         <v>159</v>
       </c>
       <c r="K25" s="18" t="s">
@@ -5300,7 +5279,7 @@
       <c r="A26" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="B26" s="62">
+      <c r="B26" s="1">
         <v>3</v>
       </c>
       <c r="C26" s="18" t="s">
@@ -5309,19 +5288,19 @@
       <c r="E26" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="F26" s="62">
+      <c r="F26" s="1">
         <v>4</v>
       </c>
-      <c r="G26" s="60" t="s">
+      <c r="G26" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="62" t="s">
+      <c r="H26" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I26" s="67" t="s">
+      <c r="I26" s="39" t="s">
         <v>198</v>
       </c>
-      <c r="J26" s="62" t="s">
+      <c r="J26" s="1" t="s">
         <v>159</v>
       </c>
       <c r="K26" s="18" t="s">
@@ -5332,31 +5311,31 @@
       <c r="A27" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="62">
+      <c r="B27" s="1">
         <v>3</v>
       </c>
       <c r="C27" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E27" s="58" t="s">
+      <c r="E27" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="F27" s="59">
+      <c r="F27" s="1">
         <v>5</v>
       </c>
-      <c r="G27" s="60" t="s">
+      <c r="G27" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="59" t="s">
+      <c r="H27" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="I27" s="66" t="s">
+      <c r="I27" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="J27" s="59" t="s">
+      <c r="J27" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="K27" s="61" t="s">
+      <c r="K27" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5364,7 +5343,7 @@
       <c r="A28" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="62">
+      <c r="B28" s="1">
         <v>4</v>
       </c>
       <c r="C28" s="18" t="s">
@@ -5373,19 +5352,19 @@
       <c r="E28" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="62">
+      <c r="F28" s="1">
         <v>2</v>
       </c>
-      <c r="G28" s="60" t="s">
+      <c r="G28" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="62" t="s">
+      <c r="H28" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="I28" s="62">
+      <c r="I28" s="1">
         <v>29</v>
       </c>
-      <c r="J28" s="62" t="s">
+      <c r="J28" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K28" s="18" t="s">
@@ -5396,7 +5375,7 @@
       <c r="A29" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="62">
+      <c r="B29" s="1">
         <v>5</v>
       </c>
       <c r="C29" s="18" t="s">
@@ -5405,19 +5384,19 @@
       <c r="E29" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="F29" s="62">
+      <c r="F29" s="1">
         <v>3</v>
       </c>
-      <c r="G29" s="60" t="s">
+      <c r="G29" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="62" t="s">
+      <c r="H29" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="I29" s="62">
+      <c r="I29" s="1">
         <v>60</v>
       </c>
-      <c r="J29" s="62" t="s">
+      <c r="J29" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K29" s="18" t="s">
@@ -5428,7 +5407,7 @@
       <c r="A30" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="62">
+      <c r="B30" s="1">
         <v>5</v>
       </c>
       <c r="C30" s="18" t="s">
@@ -5437,19 +5416,19 @@
       <c r="E30" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="F30" s="62">
+      <c r="F30" s="1">
         <v>4</v>
       </c>
-      <c r="G30" s="60" t="s">
+      <c r="G30" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="62" t="s">
+      <c r="H30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I30" s="62">
+      <c r="I30" s="1">
         <v>95</v>
       </c>
-      <c r="J30" s="62" t="s">
+      <c r="J30" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K30" s="18" t="s">
@@ -5469,19 +5448,19 @@
       <c r="E31" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="F31" s="62">
+      <c r="F31" s="1">
         <v>1</v>
       </c>
-      <c r="G31" s="60" t="s">
+      <c r="G31" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="62" t="s">
+      <c r="H31" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="I31" s="62">
+      <c r="I31" s="1">
         <v>36</v>
       </c>
-      <c r="J31" s="62" t="s">
+      <c r="J31" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K31" s="18" t="s">
@@ -5492,19 +5471,19 @@
       <c r="E32" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F32" s="62">
+      <c r="F32" s="1">
         <v>2</v>
       </c>
-      <c r="G32" s="60" t="s">
+      <c r="G32" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="62" t="s">
+      <c r="H32" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I32" s="62">
+      <c r="I32" s="1">
         <v>29</v>
       </c>
-      <c r="J32" s="62" t="s">
+      <c r="J32" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K32" s="18" t="s">
@@ -5515,19 +5494,19 @@
       <c r="E33" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="F33" s="62">
+      <c r="F33" s="1">
         <v>3</v>
       </c>
-      <c r="G33" s="60" t="s">
+      <c r="G33" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="62" t="s">
+      <c r="H33" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I33" s="62">
+      <c r="I33" s="1">
         <v>60</v>
       </c>
-      <c r="J33" s="62" t="s">
+      <c r="J33" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K33" s="18" t="s">

</xml_diff>

<commit_message>
Added Facility Floor 3 and able to use Consumables in the inventory
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABAF0DD-C8DB-4D62-BC3E-1BC96EA4103E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0226933-E691-4631-A925-DD786D2DBA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26535" yWindow="585" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="4710" yWindow="1635" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="213">
   <si>
     <t>Lv</t>
   </si>
@@ -229,9 +229,6 @@
     <t>Mermaid Tail</t>
   </si>
   <si>
-    <t>£10 Coin</t>
-  </si>
-  <si>
     <t>Diamond</t>
   </si>
   <si>
@@ -562,18 +559,6 @@
     <t>Atlantis F5 Key B</t>
   </si>
   <si>
-    <t>Facility F3 Key</t>
-  </si>
-  <si>
-    <t>Facility F5 Key A</t>
-  </si>
-  <si>
-    <t>Facility F5 Key B</t>
-  </si>
-  <si>
-    <t>Facility F5 Key C</t>
-  </si>
-  <si>
     <t>Battery Reserve</t>
   </si>
   <si>
@@ -635,6 +620,63 @@
   </si>
   <si>
     <t>+150 HP</t>
+  </si>
+  <si>
+    <t>Explosive TNT</t>
+  </si>
+  <si>
+    <t>World's Biggest Hose</t>
+  </si>
+  <si>
+    <t>Frosted Railgun</t>
+  </si>
+  <si>
+    <t>Broken Powerline</t>
+  </si>
+  <si>
+    <t>Portable Black Hole</t>
+  </si>
+  <si>
+    <t>Meflamadia</t>
+  </si>
+  <si>
+    <t>Mesplashadia</t>
+  </si>
+  <si>
+    <t>Mefreezadia</t>
+  </si>
+  <si>
+    <t>Mezapadia</t>
+  </si>
+  <si>
+    <t>Megustadia</t>
+  </si>
+  <si>
+    <t>WInd</t>
+  </si>
+  <si>
+    <t>AK-47</t>
+  </si>
+  <si>
+    <t>10 Pound Coin</t>
+  </si>
+  <si>
+    <t>10 Euro Coin</t>
+  </si>
+  <si>
+    <t>Jar of Substance</t>
+  </si>
+  <si>
+    <t>Facility F3 Keycard</t>
+  </si>
+  <si>
+    <t>Facility F5 Keycard A</t>
+  </si>
+  <si>
+    <t>Facility F5 Keycard B</t>
+  </si>
+  <si>
+    <t>Facility F5 Keycard C</t>
   </si>
 </sst>
 </file>
@@ -711,7 +753,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -903,48 +945,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1003,12 +1008,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1036,9 +1035,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1048,9 +1044,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1069,59 +1062,83 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1498,7 +1515,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="46" t="s">
+      <c r="F3" s="40" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1520,7 +1537,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="46"/>
+      <c r="F4" s="40"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1543,7 +1560,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="46"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1566,7 +1583,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="46"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1589,7 +1606,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="46"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1612,7 +1629,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="46"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1635,7 +1652,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="46"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1658,7 +1675,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="46"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1681,7 +1698,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="46"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1704,7 +1721,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="46"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1727,7 +1744,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="46"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1750,7 +1767,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="46"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1773,7 +1790,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="46"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1796,7 +1813,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="46"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1819,7 +1836,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="46"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1842,7 +1859,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="46"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1865,7 +1882,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="46"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1888,7 +1905,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="46"/>
+      <c r="F20" s="40"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1911,7 +1928,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="46"/>
+      <c r="F21" s="40"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -3704,10 +3721,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="47"/>
+      <c r="B3" s="55"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3722,214 +3739,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="53" t="s">
+      <c r="C4" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="48">
+      <c r="D4" s="41">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="60" t="s">
+      <c r="F4" s="44" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="49"/>
-      <c r="B5" s="56"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="49"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="42"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="46"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="49"/>
-      <c r="B6" s="56"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="49"/>
+      <c r="A6" s="42"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="42"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="46"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="52"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="50"/>
+      <c r="A7" s="43"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="43"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="61"/>
+      <c r="F7" s="45"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="58" t="s">
+      <c r="C8" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="49" t="s">
+      <c r="D8" s="42" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="46" t="s">
+      <c r="F8" s="40" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="49"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="49"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="42"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="46"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="50"/>
-      <c r="B10" s="50"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="50"/>
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="43"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="61"/>
+      <c r="F10" s="45"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="48" t="s">
+      <c r="A11" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="49">
+      <c r="D11" s="42">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="46" t="s">
+      <c r="F11" s="40" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="49"/>
-      <c r="B12" s="49"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="49"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="42"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="46"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="50"/>
-      <c r="B13" s="50"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="50"/>
+      <c r="A13" s="43"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="43"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="61"/>
+      <c r="F13" s="45"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="49" t="s">
+      <c r="A14" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="57" t="s">
+      <c r="C14" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="49" t="s">
+      <c r="D14" s="42" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="46" t="s">
+      <c r="F14" s="40" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="49"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="49"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="53"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="46"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="50"/>
-      <c r="B16" s="50"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="50"/>
+      <c r="A16" s="43"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="43"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="61"/>
+      <c r="F16" s="45"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="53" t="s">
+      <c r="C17" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="49">
+      <c r="D17" s="42">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="46" t="s">
+      <c r="F17" s="40" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="49"/>
-      <c r="B18" s="49"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="49"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="42"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="46"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="50"/>
-      <c r="B19" s="50"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="50"/>
+      <c r="A19" s="43"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="43"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="61"/>
+      <c r="F19" s="45"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3952,37 +3969,55 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="48" t="s">
+      <c r="A21" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="51" t="s">
+      <c r="B21" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="53" t="s">
+      <c r="C21" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="48">
+      <c r="D21" s="41">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="60" t="s">
+      <c r="F21" s="44" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="50"/>
-      <c r="B22" s="52"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="50"/>
+      <c r="A22" s="43"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="43"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="61"/>
+      <c r="F22" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -3996,24 +4031,6 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4022,7 +4039,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36AA0E8-4612-49A3-9CD4-2D5734B3DCEA}">
-  <dimension ref="A1:W34"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -4046,125 +4063,125 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="41"/>
+      <c r="B1" s="37"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="35" t="s">
+      <c r="B3" s="39"/>
+      <c r="C3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="43"/>
-      <c r="G3" s="34" t="s">
+      <c r="F3" s="39"/>
+      <c r="G3" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="J3" s="34" t="s">
+      <c r="I3" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="J3" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="K3" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="M3" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="39"/>
+      <c r="O3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="P3" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q3" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="S3" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="T3" s="39"/>
+      <c r="U3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="V3" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="W3" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="23">
+        <v>1</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="23">
+        <v>1</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" s="23">
+        <v>44</v>
+      </c>
+      <c r="J4" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="K3" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="M3" s="44" t="s">
-        <v>7</v>
-      </c>
-      <c r="N3" s="45"/>
-      <c r="O3" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="P3" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q3" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="S3" s="42" t="s">
-        <v>7</v>
-      </c>
-      <c r="T3" s="43"/>
-      <c r="U3" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="V3" s="34" t="s">
+      <c r="K4" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="N4" s="23">
+        <v>1</v>
+      </c>
+      <c r="O4" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="23">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="S4" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="T4" s="23">
+        <v>1</v>
+      </c>
+      <c r="U4" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="V4" s="30" t="s">
         <v>128</v>
       </c>
-      <c r="W3" s="35" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="24" t="s">
-        <v>182</v>
-      </c>
-      <c r="B4" s="25">
-        <v>1</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="25">
-        <v>1</v>
-      </c>
-      <c r="G4" s="36" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="I4" s="25">
-        <v>44</v>
-      </c>
-      <c r="J4" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="K4" s="26" t="s">
-        <v>4</v>
-      </c>
-      <c r="M4" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="N4" s="25">
-        <v>1</v>
-      </c>
-      <c r="O4" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="P4" s="25">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="S4" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="T4" s="25">
-        <v>1</v>
-      </c>
-      <c r="U4" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>129</v>
-      </c>
-      <c r="W4" s="26" t="s">
+      <c r="W4" s="24" t="s">
         <v>4</v>
       </c>
     </row>
@@ -4172,59 +4189,59 @@
       <c r="A5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="59">
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="F5" s="1">
+        <v>178</v>
+      </c>
+      <c r="F5" s="59">
         <v>3</v>
       </c>
-      <c r="G5" s="37" t="s">
+      <c r="G5" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="I5" s="1">
+      <c r="H5" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="I5" s="59">
         <v>70</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>151</v>
+      <c r="J5" s="59" t="s">
+        <v>150</v>
       </c>
       <c r="K5" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M5" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="N5" s="1">
+        <v>114</v>
+      </c>
+      <c r="N5" s="59">
         <v>1</v>
       </c>
-      <c r="O5" s="33" t="s">
+      <c r="O5" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="59">
         <v>13</v>
       </c>
       <c r="Q5" s="18" t="s">
         <v>4</v>
       </c>
       <c r="S5" s="17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="T5" s="1">
         <v>1</v>
       </c>
-      <c r="U5" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V5" s="39" t="s">
-        <v>131</v>
+      <c r="U5" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V5" s="35" t="s">
+        <v>130</v>
       </c>
       <c r="W5" s="18" t="s">
         <v>4</v>
@@ -4234,59 +4251,59 @@
       <c r="A6" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="59">
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E6" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="59">
+        <v>1</v>
+      </c>
+      <c r="G6" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I6" s="1">
+      <c r="I6" s="59">
         <v>44</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>155</v>
+      <c r="J6" s="59" t="s">
+        <v>154</v>
       </c>
       <c r="K6" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M6" s="17" t="s">
-        <v>166</v>
-      </c>
-      <c r="N6" s="1">
+        <v>165</v>
+      </c>
+      <c r="N6" s="59">
         <v>1</v>
       </c>
-      <c r="O6" s="33" t="s">
+      <c r="O6" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="59">
         <v>39</v>
       </c>
       <c r="Q6" s="18" t="s">
         <v>58</v>
       </c>
       <c r="S6" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T6" s="1">
         <v>2</v>
       </c>
-      <c r="U6" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V6" s="39" t="s">
-        <v>133</v>
+      <c r="U6" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V6" s="35" t="s">
+        <v>132</v>
       </c>
       <c r="W6" s="18" t="s">
         <v>4</v>
@@ -4296,59 +4313,59 @@
       <c r="A7" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="59">
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7" s="59">
+        <v>2</v>
+      </c>
+      <c r="G7" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="F7" s="1">
-        <v>2</v>
-      </c>
-      <c r="G7" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I7" s="1">
+      <c r="I7" s="59">
         <v>35</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>155</v>
+      <c r="J7" s="59" t="s">
+        <v>154</v>
       </c>
       <c r="K7" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M7" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="N7" s="1">
+        <v>115</v>
+      </c>
+      <c r="N7" s="59">
         <v>2</v>
       </c>
-      <c r="O7" s="33" t="s">
+      <c r="O7" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="59">
         <v>21</v>
       </c>
       <c r="Q7" s="18" t="s">
         <v>4</v>
       </c>
       <c r="S7" s="17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="T7" s="1">
         <v>2</v>
       </c>
-      <c r="U7" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V7" s="39" t="s">
-        <v>135</v>
+      <c r="U7" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V7" s="35" t="s">
+        <v>134</v>
       </c>
       <c r="W7" s="18" t="s">
         <v>4</v>
@@ -4358,59 +4375,59 @@
       <c r="A8" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="59">
         <v>1</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" s="59">
+        <v>4</v>
+      </c>
+      <c r="G8" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="59" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="1">
-        <v>4</v>
-      </c>
-      <c r="G8" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="I8" s="1">
+      <c r="I8" s="59">
         <v>56</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>155</v>
+      <c r="J8" s="59" t="s">
+        <v>154</v>
       </c>
       <c r="K8" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="N8" s="1">
+        <v>119</v>
+      </c>
+      <c r="N8" s="59">
         <v>2</v>
       </c>
-      <c r="O8" s="33" t="s">
+      <c r="O8" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="59">
         <v>56</v>
       </c>
       <c r="Q8" s="18" t="s">
         <v>20</v>
       </c>
       <c r="S8" s="17" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T8" s="1">
         <v>3</v>
       </c>
-      <c r="U8" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V8" s="39" t="s">
-        <v>137</v>
+      <c r="U8" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V8" s="35" t="s">
+        <v>136</v>
       </c>
       <c r="W8" s="18" t="s">
         <v>4</v>
@@ -4420,59 +4437,59 @@
       <c r="A9" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="59">
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="59">
+        <v>2</v>
+      </c>
+      <c r="G9" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="59" t="s">
         <v>109</v>
       </c>
-      <c r="F9" s="1">
-        <v>2</v>
-      </c>
-      <c r="G9" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="I9" s="1">
+      <c r="I9" s="59">
         <v>32</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>157</v>
+      <c r="J9" s="59" t="s">
+        <v>156</v>
       </c>
       <c r="K9" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M9" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="N9" s="1">
+        <v>164</v>
+      </c>
+      <c r="N9" s="59">
         <v>2</v>
       </c>
-      <c r="O9" s="33" t="s">
+      <c r="O9" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="59">
         <v>73</v>
       </c>
       <c r="Q9" s="18" t="s">
         <v>58</v>
       </c>
       <c r="S9" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="T9" s="1">
         <v>3</v>
       </c>
-      <c r="U9" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V9" s="39" t="s">
-        <v>139</v>
+      <c r="U9" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V9" s="35" t="s">
+        <v>138</v>
       </c>
       <c r="W9" s="18" t="s">
         <v>20</v>
@@ -4482,59 +4499,59 @@
       <c r="A10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="59">
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E10" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="59">
+        <v>3</v>
+      </c>
+      <c r="G10" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="1">
-        <v>3</v>
-      </c>
-      <c r="G10" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I10" s="1">
+      <c r="I10" s="59">
         <v>65</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>157</v>
+      <c r="J10" s="59" t="s">
+        <v>156</v>
       </c>
       <c r="K10" s="18" t="s">
         <v>4</v>
       </c>
       <c r="M10" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="N10" s="1">
+        <v>116</v>
+      </c>
+      <c r="N10" s="59">
         <v>3</v>
       </c>
-      <c r="O10" s="33" t="s">
+      <c r="O10" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="59">
         <v>36</v>
       </c>
       <c r="Q10" s="18" t="s">
         <v>4</v>
       </c>
       <c r="S10" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="T10" s="1">
         <v>3</v>
       </c>
-      <c r="U10" s="38" t="s">
-        <v>126</v>
+      <c r="U10" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="W10" s="18" t="s">
         <v>20</v>
@@ -4544,59 +4561,59 @@
       <c r="A11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="59">
         <v>2</v>
       </c>
       <c r="C11" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="F11" s="1">
+        <v>173</v>
+      </c>
+      <c r="F11" s="59">
         <v>4</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="I11" s="1">
+      <c r="H11" s="59" t="s">
+        <v>174</v>
+      </c>
+      <c r="I11" s="59">
         <v>52</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>157</v>
+      <c r="J11" s="59" t="s">
+        <v>156</v>
       </c>
       <c r="K11" s="18" t="s">
         <v>4</v>
       </c>
       <c r="M11" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="N11" s="1">
+        <v>117</v>
+      </c>
+      <c r="N11" s="59">
         <v>3</v>
       </c>
-      <c r="O11" s="33" t="s">
+      <c r="O11" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="59">
         <v>46</v>
       </c>
       <c r="Q11" s="18" t="s">
         <v>4</v>
       </c>
       <c r="S11" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="T11" s="1">
         <v>3</v>
       </c>
-      <c r="U11" s="38" t="s">
-        <v>126</v>
+      <c r="U11" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="W11" s="18" t="s">
         <v>20</v>
@@ -4606,59 +4623,59 @@
       <c r="A12" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="59">
         <v>2</v>
       </c>
       <c r="C12" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="F12" s="59">
+        <v>4</v>
+      </c>
+      <c r="G12" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="F12" s="1">
-        <v>4</v>
-      </c>
-      <c r="G12" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="I12" s="1">
+      <c r="I12" s="59">
         <v>105</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>157</v>
+      <c r="J12" s="59" t="s">
+        <v>156</v>
       </c>
       <c r="K12" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M12" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="N12" s="1">
+        <v>120</v>
+      </c>
+      <c r="N12" s="59">
         <v>3</v>
       </c>
-      <c r="O12" s="33" t="s">
+      <c r="O12" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="59">
         <v>71</v>
       </c>
       <c r="Q12" s="18" t="s">
         <v>20</v>
       </c>
       <c r="S12" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="T12" s="1">
         <v>4</v>
       </c>
-      <c r="U12" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V12" s="40" t="s">
-        <v>145</v>
+      <c r="U12" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V12" s="36" t="s">
+        <v>144</v>
       </c>
       <c r="W12" s="18" t="s">
         <v>20</v>
@@ -4668,59 +4685,59 @@
       <c r="A13" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="59">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" s="1">
-        <v>1</v>
-      </c>
-      <c r="G13" s="37" t="s">
+      <c r="E13" s="56" t="s">
+        <v>197</v>
+      </c>
+      <c r="F13" s="57">
+        <v>5</v>
+      </c>
+      <c r="G13" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="1">
-        <v>40</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K13" s="18" t="s">
-        <v>4</v>
+      <c r="H13" s="57" t="s">
+        <v>202</v>
+      </c>
+      <c r="I13" s="57">
+        <v>84</v>
+      </c>
+      <c r="J13" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="K13" s="58" t="s">
+        <v>58</v>
       </c>
       <c r="M13" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="N13" s="1">
+        <v>122</v>
+      </c>
+      <c r="N13" s="59">
         <v>3</v>
       </c>
-      <c r="O13" s="33" t="s">
+      <c r="O13" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="59">
         <v>78</v>
       </c>
       <c r="Q13" s="18" t="s">
         <v>20</v>
       </c>
       <c r="S13" s="17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="T13" s="1">
         <v>4</v>
       </c>
-      <c r="U13" s="38" t="s">
-        <v>126</v>
+      <c r="U13" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="W13" s="18" t="s">
         <v>20</v>
@@ -4728,61 +4745,61 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B14" s="1">
+        <v>208</v>
+      </c>
+      <c r="B14" s="59">
         <v>2</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="1">
-        <v>2</v>
-      </c>
-      <c r="G14" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="59">
+        <v>1</v>
+      </c>
+      <c r="G14" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="I14" s="1">
-        <v>32</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>152</v>
+      <c r="H14" s="59" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="59">
+        <v>40</v>
+      </c>
+      <c r="J14" s="59" t="s">
+        <v>151</v>
       </c>
       <c r="K14" s="18" t="s">
         <v>4</v>
       </c>
       <c r="M14" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="N14" s="1">
+        <v>121</v>
+      </c>
+      <c r="N14" s="59">
         <v>3</v>
       </c>
-      <c r="O14" s="33" t="s">
+      <c r="O14" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="59">
         <v>86</v>
       </c>
       <c r="Q14" s="18" t="s">
         <v>20</v>
       </c>
       <c r="S14" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="T14" s="1">
         <v>4</v>
       </c>
-      <c r="U14" s="38" t="s">
-        <v>126</v>
+      <c r="U14" s="34" t="s">
+        <v>125</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="W14" s="18" t="s">
         <v>20</v>
@@ -4790,61 +4807,61 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="1">
+        <v>62</v>
+      </c>
+      <c r="B15" s="59">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="59">
+        <v>2</v>
+      </c>
+      <c r="G15" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="59" t="s">
+        <v>70</v>
+      </c>
+      <c r="I15" s="59">
+        <v>32</v>
+      </c>
+      <c r="J15" s="59" t="s">
+        <v>151</v>
+      </c>
+      <c r="K15" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="F15" s="1">
+      <c r="M15" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="N15" s="59">
         <v>3</v>
       </c>
-      <c r="G15" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="I15" s="1">
-        <v>65</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K15" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="M15" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="N15" s="1">
-        <v>3</v>
-      </c>
-      <c r="O15" s="33" t="s">
+      <c r="O15" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="59">
         <v>109</v>
       </c>
       <c r="Q15" s="18" t="s">
         <v>58</v>
       </c>
       <c r="S15" s="17" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="T15" s="1">
         <v>4</v>
       </c>
-      <c r="U15" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V15" s="39" t="s">
-        <v>191</v>
+      <c r="U15" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V15" s="35" t="s">
+        <v>186</v>
       </c>
       <c r="W15" s="18" t="s">
         <v>58</v>
@@ -4852,61 +4869,61 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="1">
+        <v>57</v>
+      </c>
+      <c r="B16" s="59">
+        <v>2</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="F16" s="59">
         <v>3</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="1">
-        <v>4</v>
-      </c>
-      <c r="G16" s="37" t="s">
+      <c r="G16" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I16" s="1">
-        <v>52</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>152</v>
+      <c r="H16" s="59" t="s">
+        <v>182</v>
+      </c>
+      <c r="I16" s="59">
+        <v>65</v>
+      </c>
+      <c r="J16" s="59" t="s">
+        <v>151</v>
       </c>
       <c r="K16" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M16" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="N16" s="1">
-        <v>4</v>
-      </c>
-      <c r="O16" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="N16" s="59">
+        <v>3</v>
+      </c>
+      <c r="O16" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="1">
-        <v>67</v>
+      <c r="P16" s="59">
+        <v>120</v>
       </c>
       <c r="Q16" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="S16" s="17" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="T16" s="1">
         <v>4</v>
       </c>
-      <c r="U16" s="38" t="s">
-        <v>126</v>
-      </c>
-      <c r="V16" s="39" t="s">
-        <v>193</v>
+      <c r="U16" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="V16" s="35" t="s">
+        <v>188</v>
       </c>
       <c r="W16" s="18" t="s">
         <v>58</v>
@@ -4914,61 +4931,61 @@
     </row>
     <row r="17" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="B17" s="1">
+        <v>207</v>
+      </c>
+      <c r="B17" s="59">
         <v>3</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17" s="1">
+        <v>93</v>
+      </c>
+      <c r="F17" s="59">
         <v>4</v>
       </c>
-      <c r="G17" s="37" t="s">
+      <c r="G17" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I17" s="1">
-        <v>105</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>152</v>
+      <c r="H17" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="I17" s="59">
+        <v>52</v>
+      </c>
+      <c r="J17" s="59" t="s">
+        <v>151</v>
       </c>
       <c r="K17" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M17" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="N17" s="1">
+        <v>118</v>
+      </c>
+      <c r="N17" s="59">
         <v>4</v>
       </c>
-      <c r="O17" s="33" t="s">
+      <c r="O17" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P17" s="1">
-        <v>103</v>
+      <c r="P17" s="59">
+        <v>67</v>
       </c>
       <c r="Q17" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="S17" s="19" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="T17" s="20">
         <v>5</v>
       </c>
-      <c r="U17" s="31" t="s">
-        <v>126</v>
+      <c r="U17" s="29" t="s">
+        <v>125</v>
       </c>
       <c r="V17" s="20" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="W17" s="21" t="s">
         <v>58</v>
@@ -4976,46 +4993,46 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="B18" s="1">
+        <v>206</v>
+      </c>
+      <c r="B18" s="59">
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" s="1">
-        <v>1</v>
-      </c>
-      <c r="G18" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" s="59">
+        <v>4</v>
+      </c>
+      <c r="G18" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I18" s="1">
-        <v>36</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>153</v>
+      <c r="H18" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="I18" s="59">
+        <v>105</v>
+      </c>
+      <c r="J18" s="59" t="s">
+        <v>151</v>
       </c>
       <c r="K18" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="N18" s="59">
         <v>4</v>
       </c>
-      <c r="M18" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="N18" s="1">
-        <v>4</v>
-      </c>
-      <c r="O18" s="33" t="s">
+      <c r="O18" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P18" s="1">
-        <v>139</v>
+      <c r="P18" s="59">
+        <v>103</v>
       </c>
       <c r="Q18" s="18" t="s">
         <v>20</v>
@@ -5023,285 +5040,300 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>172</v>
-      </c>
-      <c r="B19" s="1">
+        <v>169</v>
+      </c>
+      <c r="B19" s="59">
         <v>3</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="F19" s="1">
-        <v>2</v>
-      </c>
-      <c r="G19" s="37" t="s">
+      <c r="E19" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="F19" s="57">
+        <v>5</v>
+      </c>
+      <c r="G19" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I19" s="1">
-        <v>29</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="K19" s="18" t="s">
+      <c r="H19" s="57" t="s">
+        <v>199</v>
+      </c>
+      <c r="I19" s="57">
+        <v>84</v>
+      </c>
+      <c r="J19" s="57" t="s">
+        <v>151</v>
+      </c>
+      <c r="K19" s="58" t="s">
+        <v>58</v>
+      </c>
+      <c r="M19" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="N19" s="59">
         <v>4</v>
       </c>
-      <c r="M19" s="17" t="s">
-        <v>164</v>
-      </c>
-      <c r="N19" s="1">
-        <v>4</v>
-      </c>
-      <c r="O19" s="33" t="s">
+      <c r="O19" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="P19" s="1">
-        <v>165</v>
+      <c r="P19" s="59">
+        <v>139</v>
       </c>
       <c r="Q19" s="18" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="B20" s="1">
+        <v>170</v>
+      </c>
+      <c r="B20" s="59">
         <v>3</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F20" s="1">
-        <v>3</v>
-      </c>
-      <c r="G20" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="59">
+        <v>1</v>
+      </c>
+      <c r="G20" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I20" s="1">
-        <v>60</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>153</v>
+      <c r="H20" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20" s="59">
+        <v>36</v>
+      </c>
+      <c r="J20" s="59" t="s">
+        <v>152</v>
       </c>
       <c r="K20" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="M20" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="N20" s="20">
+      <c r="M20" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="N20" s="59">
+        <v>4</v>
+      </c>
+      <c r="O20" s="65" t="s">
+        <v>17</v>
+      </c>
+      <c r="P20" s="59">
+        <v>165</v>
+      </c>
+      <c r="Q20" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21" s="59">
+        <v>3</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F21" s="59">
+        <v>2</v>
+      </c>
+      <c r="G21" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="59" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="59">
+        <v>29</v>
+      </c>
+      <c r="J21" s="59" t="s">
+        <v>152</v>
+      </c>
+      <c r="K21" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="N21" s="20">
         <v>5</v>
       </c>
-      <c r="O20" s="29" t="s">
+      <c r="O21" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="P20" s="20">
+      <c r="P21" s="20">
         <v>214</v>
       </c>
-      <c r="Q20" s="21" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
-        <v>174</v>
-      </c>
-      <c r="B21" s="1">
-        <v>3</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>162</v>
-      </c>
-      <c r="F21" s="1">
-        <v>4</v>
-      </c>
-      <c r="G21" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I21" s="1">
-        <v>95</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="K21" s="18" t="s">
+      <c r="Q21" s="21" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="B22" s="1">
+        <v>172</v>
+      </c>
+      <c r="B22" s="59">
         <v>3</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="F22" s="1">
+        <v>87</v>
+      </c>
+      <c r="F22" s="59">
         <v>3</v>
       </c>
-      <c r="G22" s="37" t="s">
+      <c r="G22" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="I22" s="1">
-        <v>98</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>158</v>
+      <c r="H22" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="I22" s="59">
+        <v>60</v>
+      </c>
+      <c r="J22" s="59" t="s">
+        <v>152</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="1">
+        <v>209</v>
+      </c>
+      <c r="B23" s="59">
         <v>3</v>
       </c>
       <c r="C23" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F23" s="1">
+        <v>161</v>
+      </c>
+      <c r="F23" s="59">
         <v>4</v>
       </c>
-      <c r="G23" s="37" t="s">
+      <c r="G23" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="I23" s="1">
-        <v>174</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>158</v>
+      <c r="H23" s="59" t="s">
+        <v>12</v>
+      </c>
+      <c r="I23" s="59">
+        <v>95</v>
+      </c>
+      <c r="J23" s="59" t="s">
+        <v>152</v>
       </c>
       <c r="K23" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" s="1">
+        <v>210</v>
+      </c>
+      <c r="B24" s="59">
         <v>3</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="F24" s="1">
+      <c r="E24" s="56" t="s">
+        <v>196</v>
+      </c>
+      <c r="F24" s="57">
         <v>5</v>
       </c>
-      <c r="G24" s="37" t="s">
+      <c r="G24" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="I24" s="1">
-        <v>269</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K24" s="18" t="s">
+      <c r="H24" s="57" t="s">
+        <v>201</v>
+      </c>
+      <c r="I24" s="57">
+        <v>76</v>
+      </c>
+      <c r="J24" s="57" t="s">
+        <v>152</v>
+      </c>
+      <c r="K24" s="58" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="B25" s="1">
+        <v>211</v>
+      </c>
+      <c r="B25" s="59">
         <v>3</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="F25" s="1">
+        <v>101</v>
+      </c>
+      <c r="F25" s="59">
         <v>3</v>
       </c>
-      <c r="G25" s="37" t="s">
+      <c r="G25" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I25" s="39" t="s">
-        <v>197</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>159</v>
+      <c r="H25" s="59" t="s">
+        <v>102</v>
+      </c>
+      <c r="I25" s="59">
+        <v>98</v>
+      </c>
+      <c r="J25" s="59" t="s">
+        <v>157</v>
       </c>
       <c r="K25" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="B26" s="1">
+        <v>212</v>
+      </c>
+      <c r="B26" s="59">
         <v>3</v>
       </c>
       <c r="C26" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" s="59">
         <v>4</v>
       </c>
-      <c r="E26" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="F26" s="1">
-        <v>4</v>
-      </c>
-      <c r="G26" s="37" t="s">
+      <c r="G26" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I26" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>159</v>
+      <c r="H26" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="I26" s="59">
+        <v>174</v>
+      </c>
+      <c r="J26" s="59" t="s">
+        <v>157</v>
       </c>
       <c r="K26" s="18" t="s">
         <v>20</v>
@@ -5309,31 +5341,31 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="1">
+        <v>167</v>
+      </c>
+      <c r="B27" s="59">
         <v>3</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="F27" s="1">
+        <v>175</v>
+      </c>
+      <c r="F27" s="59">
         <v>5</v>
       </c>
-      <c r="G27" s="37" t="s">
+      <c r="G27" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="I27" s="39" t="s">
-        <v>196</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>159</v>
+      <c r="H27" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="I27" s="59">
+        <v>269</v>
+      </c>
+      <c r="J27" s="59" t="s">
+        <v>157</v>
       </c>
       <c r="K27" s="18" t="s">
         <v>58</v>
@@ -5341,63 +5373,63 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="1">
-        <v>4</v>
+        <v>168</v>
+      </c>
+      <c r="B28" s="59">
+        <v>3</v>
       </c>
       <c r="C28" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="F28" s="1">
-        <v>2</v>
-      </c>
-      <c r="G28" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="F28" s="59">
+        <v>3</v>
+      </c>
+      <c r="G28" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="I28" s="1">
-        <v>29</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>156</v>
+      <c r="H28" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="J28" s="59" t="s">
+        <v>158</v>
       </c>
       <c r="K28" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" s="1">
-        <v>5</v>
+        <v>55</v>
+      </c>
+      <c r="B29" s="59">
+        <v>3</v>
       </c>
       <c r="C29" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="1">
-        <v>3</v>
-      </c>
-      <c r="G29" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="F29" s="59">
+        <v>4</v>
+      </c>
+      <c r="G29" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="I29" s="1">
-        <v>60</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>156</v>
+      <c r="H29" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="I29" s="61" t="s">
+        <v>193</v>
+      </c>
+      <c r="J29" s="59" t="s">
+        <v>158</v>
       </c>
       <c r="K29" s="18" t="s">
         <v>20</v>
@@ -5405,142 +5437,274 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="1">
+        <v>52</v>
+      </c>
+      <c r="B30" s="59">
+        <v>4</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="F30" s="59">
         <v>5</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="G30" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="I30" s="61" t="s">
+        <v>191</v>
+      </c>
+      <c r="J30" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="59">
+        <v>5</v>
+      </c>
+      <c r="C31" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E30" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F30" s="1">
+      <c r="E31" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="F31" s="59">
+        <v>2</v>
+      </c>
+      <c r="G31" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="59" t="s">
+        <v>111</v>
+      </c>
+      <c r="I31" s="59">
+        <v>29</v>
+      </c>
+      <c r="J31" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="59">
+        <v>5</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="F32" s="59">
+        <v>3</v>
+      </c>
+      <c r="G32" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="59" t="s">
+        <v>106</v>
+      </c>
+      <c r="I32" s="59">
+        <v>60</v>
+      </c>
+      <c r="J32" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="20">
+        <v>5</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" s="59">
         <v>4</v>
       </c>
-      <c r="G30" s="37" t="s">
+      <c r="G33" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H33" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I33" s="59">
         <v>95</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="K30" s="18" t="s">
+      <c r="J33" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="K33" s="18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="B31" s="20">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E34" s="56" t="s">
+        <v>195</v>
+      </c>
+      <c r="F34" s="57">
         <v>5</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="G34" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="57" t="s">
+        <v>200</v>
+      </c>
+      <c r="I34" s="57">
+        <v>76</v>
+      </c>
+      <c r="J34" s="57" t="s">
+        <v>155</v>
+      </c>
+      <c r="K34" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="E31" s="17" t="s">
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E35" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F35" s="59">
+        <v>1</v>
+      </c>
+      <c r="G35" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="F31" s="1">
-        <v>1</v>
-      </c>
-      <c r="G31" s="37" t="s">
+      <c r="I35" s="59">
+        <v>36</v>
+      </c>
+      <c r="J35" s="59" t="s">
+        <v>153</v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E36" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F36" s="59">
+        <v>2</v>
+      </c>
+      <c r="G36" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="H36" s="59" t="s">
+        <v>74</v>
+      </c>
+      <c r="I36" s="59">
+        <v>29</v>
+      </c>
+      <c r="J36" s="59" t="s">
+        <v>153</v>
+      </c>
+      <c r="K36" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E37" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="I31" s="1">
-        <v>36</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="K31" s="18" t="s">
+      <c r="F37" s="59">
+        <v>3</v>
+      </c>
+      <c r="G37" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="59" t="s">
+        <v>92</v>
+      </c>
+      <c r="I37" s="59">
+        <v>60</v>
+      </c>
+      <c r="J37" s="59" t="s">
+        <v>153</v>
+      </c>
+      <c r="K37" s="18" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="E32" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="F32" s="1">
-        <v>2</v>
-      </c>
-      <c r="G32" s="37" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E38" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="F38" s="59">
+        <v>4</v>
+      </c>
+      <c r="G38" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="I32" s="1">
-        <v>29</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="K32" s="18" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E33" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="F33" s="1">
-        <v>3</v>
-      </c>
-      <c r="G33" s="37" t="s">
+      <c r="H38" s="59" t="s">
+        <v>160</v>
+      </c>
+      <c r="I38" s="59">
+        <v>95</v>
+      </c>
+      <c r="J38" s="59" t="s">
+        <v>153</v>
+      </c>
+      <c r="K38" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E39" s="62" t="s">
+        <v>198</v>
+      </c>
+      <c r="F39" s="63">
+        <v>5</v>
+      </c>
+      <c r="G39" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I33" s="1">
-        <v>60</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="K33" s="18" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="5:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E34" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="F34" s="20">
-        <v>4</v>
-      </c>
-      <c r="G34" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="H34" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="I34" s="20">
-        <v>95</v>
-      </c>
-      <c r="J34" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="K34" s="21" t="s">
+      <c r="H39" s="63" t="s">
+        <v>203</v>
+      </c>
+      <c r="I39" s="63">
+        <v>76</v>
+      </c>
+      <c r="J39" s="63" t="s">
+        <v>204</v>
+      </c>
+      <c r="K39" s="64" t="s">
         <v>58</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E4:K34">
-    <sortCondition ref="J4:J34"/>
-    <sortCondition ref="F4:F34"/>
-    <sortCondition ref="I4:I34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C33">
+    <sortCondition ref="B4:B33"/>
+    <sortCondition ref="A4:A33"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Added Facility Floor 5 and 6
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0226933-E691-4631-A925-DD786D2DBA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC4424B-F137-4B85-BC85-123438831C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4710" yWindow="1635" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="2400" yWindow="2265" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="216">
   <si>
     <t>Lv</t>
   </si>
@@ -677,6 +677,15 @@
   </si>
   <si>
     <t>Facility F5 Keycard C</t>
+  </si>
+  <si>
+    <t>M6 Gerand</t>
+  </si>
+  <si>
+    <t>Kraber 50-Caliber</t>
+  </si>
+  <si>
+    <t>Mega Bunsen Burner</t>
   </si>
 </sst>
 </file>
@@ -949,7 +958,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1053,6 +1062,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1065,6 +1077,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1074,25 +1089,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1107,34 +1116,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1515,7 +1503,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="40" t="s">
+      <c r="F3" s="41" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1537,7 +1525,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="40"/>
+      <c r="F4" s="41"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1560,7 +1548,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="40"/>
+      <c r="F5" s="41"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1583,7 +1571,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="40"/>
+      <c r="F6" s="41"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1606,7 +1594,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="40"/>
+      <c r="F7" s="41"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1629,7 +1617,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="40"/>
+      <c r="F8" s="41"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1652,7 +1640,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="40"/>
+      <c r="F9" s="41"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1675,7 +1663,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="40"/>
+      <c r="F10" s="41"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1698,7 +1686,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="40"/>
+      <c r="F11" s="41"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1721,7 +1709,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="40"/>
+      <c r="F12" s="41"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1744,7 +1732,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="40"/>
+      <c r="F13" s="41"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1767,7 +1755,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="40"/>
+      <c r="F14" s="41"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1790,7 +1778,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="40"/>
+      <c r="F15" s="41"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1813,7 +1801,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="40"/>
+      <c r="F16" s="41"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1836,7 +1824,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="40"/>
+      <c r="F17" s="41"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1859,7 +1847,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="40"/>
+      <c r="F18" s="41"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1882,7 +1870,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="40"/>
+      <c r="F19" s="41"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1905,7 +1893,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="40"/>
+      <c r="F20" s="41"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1928,9 +1916,9 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="40"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F21" s="41"/>
+    </row>
+    <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <f t="shared" ref="A22:A42" si="6">A21+1</f>
         <v>20</v>
@@ -1951,6 +1939,7 @@
         <f t="shared" si="5"/>
         <v>17639</v>
       </c>
+      <c r="F22" s="41"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -3692,7 +3681,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F3:F21"/>
+    <mergeCell ref="F3:F22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3721,10 +3710,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="55"/>
+      <c r="B3" s="42"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3739,214 +3728,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="41">
+      <c r="D4" s="43">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="44" t="s">
+      <c r="F4" s="55" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="42"/>
+      <c r="A5" s="44"/>
       <c r="B5" s="51"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="42"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="40"/>
+      <c r="F5" s="41"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="42"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="51"/>
-      <c r="C6" s="50"/>
-      <c r="D6" s="42"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="44"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="40"/>
+      <c r="F6" s="41"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
-      <c r="B7" s="49"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="43"/>
+      <c r="A7" s="45"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="45"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="45"/>
+      <c r="F7" s="56"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="44" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="44" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="41" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="42"/>
-      <c r="B9" s="42"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="44"/>
       <c r="C9" s="53"/>
-      <c r="D9" s="42"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="40"/>
+      <c r="F9" s="41"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="43"/>
-      <c r="B10" s="43"/>
+      <c r="A10" s="45"/>
+      <c r="B10" s="45"/>
       <c r="C10" s="54"/>
-      <c r="D10" s="43"/>
+      <c r="D10" s="45"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="45"/>
+      <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="42">
+      <c r="D11" s="44">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="41" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="42"/>
-      <c r="B12" s="42"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="42"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="44"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="40"/>
+      <c r="F12" s="41"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="43"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="47"/>
-      <c r="D13" s="43"/>
+      <c r="A13" s="45"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="45"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="45"/>
+      <c r="F13" s="56"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
+      <c r="A14" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="43" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="44" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="40" t="s">
+      <c r="F14" s="41" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="42"/>
-      <c r="B15" s="42"/>
+      <c r="A15" s="44"/>
+      <c r="B15" s="44"/>
       <c r="C15" s="53"/>
-      <c r="D15" s="42"/>
+      <c r="D15" s="44"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="40"/>
+      <c r="F15" s="41"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="43"/>
-      <c r="B16" s="43"/>
+      <c r="A16" s="45"/>
+      <c r="B16" s="45"/>
       <c r="C16" s="54"/>
-      <c r="D16" s="43"/>
+      <c r="D16" s="45"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="45"/>
+      <c r="F16" s="56"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B17" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="42">
+      <c r="D17" s="44">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="F17" s="41" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="42"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="50"/>
-      <c r="D18" s="42"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="44"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="40"/>
+      <c r="F18" s="41"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="43"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="43"/>
+      <c r="A19" s="45"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="45"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="45"/>
+      <c r="F19" s="56"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3969,55 +3958,37 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="41" t="s">
+      <c r="A21" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="48" t="s">
+      <c r="B21" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="46" t="s">
+      <c r="C21" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="41">
+      <c r="D21" s="43">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="44" t="s">
+      <c r="F21" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="43"/>
-      <c r="B22" s="49"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="43"/>
+      <c r="A22" s="45"/>
+      <c r="B22" s="47"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="45"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="45"/>
+      <c r="F22" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -4031,6 +4002,24 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4063,24 +4052,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="37"/>
+      <c r="B1" s="38"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="39"/>
+      <c r="B3" s="40"/>
       <c r="C3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="39"/>
+      <c r="F3" s="40"/>
       <c r="G3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4096,10 +4085,10 @@
       <c r="K3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="M3" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="39"/>
+      <c r="N3" s="40"/>
       <c r="O3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4109,10 +4098,10 @@
       <c r="Q3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="S3" s="38" t="s">
+      <c r="S3" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="39"/>
+      <c r="T3" s="40"/>
       <c r="U3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4189,7 +4178,7 @@
       <c r="A5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="59">
+      <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
@@ -4198,19 +4187,19 @@
       <c r="E5" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="F5" s="59">
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="60" t="s">
+      <c r="G5" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="59" t="s">
+      <c r="H5" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I5" s="59">
+      <c r="I5" s="1">
         <v>70</v>
       </c>
-      <c r="J5" s="59" t="s">
+      <c r="J5" s="1" t="s">
         <v>150</v>
       </c>
       <c r="K5" s="18" t="s">
@@ -4219,13 +4208,13 @@
       <c r="M5" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="N5" s="59">
+      <c r="N5" s="57">
         <v>1</v>
       </c>
-      <c r="O5" s="65" t="s">
+      <c r="O5" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="59">
+      <c r="P5" s="57">
         <v>13</v>
       </c>
       <c r="Q5" s="18" t="s">
@@ -4251,7 +4240,7 @@
       <c r="A6" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="59">
+      <c r="B6" s="1">
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
@@ -4260,19 +4249,19 @@
       <c r="E6" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F6" s="59">
+      <c r="F6" s="1">
         <v>1</v>
       </c>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I6" s="59">
+      <c r="I6" s="1">
         <v>44</v>
       </c>
-      <c r="J6" s="59" t="s">
+      <c r="J6" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K6" s="18" t="s">
@@ -4281,13 +4270,13 @@
       <c r="M6" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="N6" s="59">
+      <c r="N6" s="57">
         <v>1</v>
       </c>
-      <c r="O6" s="65" t="s">
+      <c r="O6" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="59">
+      <c r="P6" s="57">
         <v>39</v>
       </c>
       <c r="Q6" s="18" t="s">
@@ -4313,7 +4302,7 @@
       <c r="A7" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B7" s="59">
+      <c r="B7" s="1">
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -4322,19 +4311,19 @@
       <c r="E7" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="F7" s="59">
+      <c r="F7" s="1">
         <v>2</v>
       </c>
-      <c r="G7" s="60" t="s">
+      <c r="G7" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="59" t="s">
+      <c r="H7" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I7" s="59">
+      <c r="I7" s="1">
         <v>35</v>
       </c>
-      <c r="J7" s="59" t="s">
+      <c r="J7" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K7" s="18" t="s">
@@ -4343,13 +4332,13 @@
       <c r="M7" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N7" s="59">
+      <c r="N7" s="57">
         <v>2</v>
       </c>
-      <c r="O7" s="65" t="s">
+      <c r="O7" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="59">
+      <c r="P7" s="57">
         <v>21</v>
       </c>
       <c r="Q7" s="18" t="s">
@@ -4375,7 +4364,7 @@
       <c r="A8" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="59">
+      <c r="B8" s="1">
         <v>1</v>
       </c>
       <c r="C8" s="18" t="s">
@@ -4384,19 +4373,19 @@
       <c r="E8" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="F8" s="59">
+      <c r="F8" s="1">
         <v>4</v>
       </c>
-      <c r="G8" s="60" t="s">
+      <c r="G8" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="59" t="s">
+      <c r="H8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I8" s="59">
+      <c r="I8" s="1">
         <v>56</v>
       </c>
-      <c r="J8" s="59" t="s">
+      <c r="J8" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K8" s="18" t="s">
@@ -4405,13 +4394,13 @@
       <c r="M8" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="N8" s="59">
+      <c r="N8" s="57">
         <v>2</v>
       </c>
-      <c r="O8" s="65" t="s">
+      <c r="O8" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="59">
+      <c r="P8" s="57">
         <v>56</v>
       </c>
       <c r="Q8" s="18" t="s">
@@ -4437,7 +4426,7 @@
       <c r="A9" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="59">
+      <c r="B9" s="1">
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
@@ -4446,19 +4435,19 @@
       <c r="E9" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="59">
+      <c r="F9" s="1">
         <v>2</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="59" t="s">
+      <c r="H9" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I9" s="59">
+      <c r="I9" s="1">
         <v>32</v>
       </c>
-      <c r="J9" s="59" t="s">
+      <c r="J9" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K9" s="18" t="s">
@@ -4467,13 +4456,13 @@
       <c r="M9" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="N9" s="59">
+      <c r="N9" s="57">
         <v>2</v>
       </c>
-      <c r="O9" s="65" t="s">
+      <c r="O9" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="59">
+      <c r="P9" s="57">
         <v>73</v>
       </c>
       <c r="Q9" s="18" t="s">
@@ -4499,7 +4488,7 @@
       <c r="A10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="59">
+      <c r="B10" s="1">
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
@@ -4508,19 +4497,19 @@
       <c r="E10" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="59">
+      <c r="F10" s="1">
         <v>3</v>
       </c>
-      <c r="G10" s="60" t="s">
+      <c r="G10" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="59" t="s">
+      <c r="H10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="I10" s="59">
+      <c r="I10" s="1">
         <v>65</v>
       </c>
-      <c r="J10" s="59" t="s">
+      <c r="J10" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K10" s="18" t="s">
@@ -4529,13 +4518,13 @@
       <c r="M10" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="N10" s="59">
+      <c r="N10" s="57">
         <v>3</v>
       </c>
-      <c r="O10" s="65" t="s">
+      <c r="O10" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="59">
+      <c r="P10" s="57">
         <v>36</v>
       </c>
       <c r="Q10" s="18" t="s">
@@ -4561,7 +4550,7 @@
       <c r="A11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="59">
+      <c r="B11" s="1">
         <v>2</v>
       </c>
       <c r="C11" s="18" t="s">
@@ -4570,19 +4559,19 @@
       <c r="E11" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="F11" s="59">
+      <c r="F11" s="1">
         <v>4</v>
       </c>
-      <c r="G11" s="60" t="s">
+      <c r="G11" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="59" t="s">
+      <c r="H11" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I11" s="59">
+      <c r="I11" s="1">
         <v>52</v>
       </c>
-      <c r="J11" s="59" t="s">
+      <c r="J11" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K11" s="18" t="s">
@@ -4591,13 +4580,13 @@
       <c r="M11" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="N11" s="59">
+      <c r="N11" s="57">
         <v>3</v>
       </c>
-      <c r="O11" s="65" t="s">
+      <c r="O11" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="59">
+      <c r="P11" s="57">
         <v>46</v>
       </c>
       <c r="Q11" s="18" t="s">
@@ -4623,7 +4612,7 @@
       <c r="A12" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="59">
+      <c r="B12" s="1">
         <v>2</v>
       </c>
       <c r="C12" s="18" t="s">
@@ -4632,19 +4621,19 @@
       <c r="E12" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="59">
+      <c r="F12" s="1">
         <v>4</v>
       </c>
-      <c r="G12" s="60" t="s">
+      <c r="G12" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="59" t="s">
+      <c r="H12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I12" s="59">
+      <c r="I12" s="1">
         <v>105</v>
       </c>
-      <c r="J12" s="59" t="s">
+      <c r="J12" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K12" s="18" t="s">
@@ -4653,13 +4642,13 @@
       <c r="M12" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="N12" s="59">
+      <c r="N12" s="57">
         <v>3</v>
       </c>
-      <c r="O12" s="65" t="s">
+      <c r="O12" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P12" s="59">
+      <c r="P12" s="57">
         <v>71</v>
       </c>
       <c r="Q12" s="18" t="s">
@@ -4685,43 +4674,43 @@
       <c r="A13" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="59">
+      <c r="B13" s="1">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="56" t="s">
+      <c r="E13" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="F13" s="57">
+      <c r="F13" s="1">
         <v>5</v>
       </c>
-      <c r="G13" s="60" t="s">
+      <c r="G13" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="57" t="s">
+      <c r="H13" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="I13" s="57">
+      <c r="I13" s="1">
         <v>84</v>
       </c>
-      <c r="J13" s="57" t="s">
+      <c r="J13" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="K13" s="58" t="s">
+      <c r="K13" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M13" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="N13" s="59">
+      <c r="N13" s="57">
         <v>3</v>
       </c>
-      <c r="O13" s="65" t="s">
+      <c r="O13" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="59">
+      <c r="P13" s="57">
         <v>78</v>
       </c>
       <c r="Q13" s="18" t="s">
@@ -4747,7 +4736,7 @@
       <c r="A14" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="B14" s="59">
+      <c r="B14" s="1">
         <v>2</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -4756,19 +4745,19 @@
       <c r="E14" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F14" s="59">
+      <c r="F14" s="1">
         <v>1</v>
       </c>
-      <c r="G14" s="60" t="s">
+      <c r="G14" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="59" t="s">
+      <c r="H14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I14" s="59">
+      <c r="I14" s="1">
         <v>40</v>
       </c>
-      <c r="J14" s="59" t="s">
+      <c r="J14" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K14" s="18" t="s">
@@ -4777,13 +4766,13 @@
       <c r="M14" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="N14" s="59">
+      <c r="N14" s="57">
         <v>3</v>
       </c>
-      <c r="O14" s="65" t="s">
+      <c r="O14" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P14" s="59">
+      <c r="P14" s="57">
         <v>86</v>
       </c>
       <c r="Q14" s="18" t="s">
@@ -4809,7 +4798,7 @@
       <c r="A15" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="59">
+      <c r="B15" s="1">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -4818,35 +4807,35 @@
       <c r="E15" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="59">
+      <c r="F15" s="1">
         <v>2</v>
       </c>
-      <c r="G15" s="60" t="s">
+      <c r="G15" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="59" t="s">
+      <c r="H15" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="I15" s="59">
+      <c r="I15" s="1">
         <v>32</v>
       </c>
-      <c r="J15" s="59" t="s">
+      <c r="J15" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K15" s="18" t="s">
         <v>4</v>
       </c>
       <c r="M15" s="17" t="s">
-        <v>162</v>
-      </c>
-      <c r="N15" s="59">
+        <v>215</v>
+      </c>
+      <c r="N15" s="57">
         <v>3</v>
       </c>
-      <c r="O15" s="65" t="s">
+      <c r="O15" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P15" s="59">
-        <v>109</v>
+      <c r="P15" s="57">
+        <v>108</v>
       </c>
       <c r="Q15" s="18" t="s">
         <v>58</v>
@@ -4871,7 +4860,7 @@
       <c r="A16" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="59">
+      <c r="B16" s="1">
         <v>2</v>
       </c>
       <c r="C16" s="18" t="s">
@@ -4880,35 +4869,35 @@
       <c r="E16" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="F16" s="59">
+      <c r="F16" s="1">
         <v>3</v>
       </c>
-      <c r="G16" s="60" t="s">
+      <c r="G16" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="59" t="s">
+      <c r="H16" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I16" s="59">
+      <c r="I16" s="1">
         <v>65</v>
       </c>
-      <c r="J16" s="59" t="s">
+      <c r="J16" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K16" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M16" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="N16" s="59">
+        <v>162</v>
+      </c>
+      <c r="N16" s="57">
         <v>3</v>
       </c>
-      <c r="O16" s="65" t="s">
+      <c r="O16" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="59">
-        <v>120</v>
+      <c r="P16" s="57">
+        <v>109</v>
       </c>
       <c r="Q16" s="18" t="s">
         <v>58</v>
@@ -4933,7 +4922,7 @@
       <c r="A17" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="B17" s="59">
+      <c r="B17" s="1">
         <v>3</v>
       </c>
       <c r="C17" s="18" t="s">
@@ -4942,38 +4931,38 @@
       <c r="E17" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="59">
+      <c r="F17" s="1">
         <v>4</v>
       </c>
-      <c r="G17" s="60" t="s">
+      <c r="G17" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="59" t="s">
+      <c r="H17" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="I17" s="59">
+      <c r="I17" s="1">
         <v>52</v>
       </c>
-      <c r="J17" s="59" t="s">
+      <c r="J17" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K17" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M17" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="N17" s="59">
-        <v>4</v>
-      </c>
-      <c r="O17" s="65" t="s">
+        <v>205</v>
+      </c>
+      <c r="N17" s="57">
+        <v>3</v>
+      </c>
+      <c r="O17" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P17" s="59">
-        <v>67</v>
+      <c r="P17" s="57">
+        <v>120</v>
       </c>
       <c r="Q17" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="S17" s="19" t="s">
         <v>189</v>
@@ -4995,7 +4984,7 @@
       <c r="A18" s="17" t="s">
         <v>206</v>
       </c>
-      <c r="B18" s="59">
+      <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
@@ -5004,82 +4993,82 @@
       <c r="E18" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="59">
+      <c r="F18" s="1">
         <v>4</v>
       </c>
-      <c r="G18" s="60" t="s">
+      <c r="G18" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="59" t="s">
+      <c r="H18" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="59">
+      <c r="I18" s="1">
         <v>105</v>
       </c>
-      <c r="J18" s="59" t="s">
+      <c r="J18" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K18" s="18" t="s">
         <v>20</v>
       </c>
       <c r="M18" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="N18" s="59">
+        <v>118</v>
+      </c>
+      <c r="N18" s="57">
         <v>4</v>
       </c>
-      <c r="O18" s="65" t="s">
+      <c r="O18" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P18" s="59">
-        <v>103</v>
+      <c r="P18" s="57">
+        <v>67</v>
       </c>
       <c r="Q18" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="B19" s="59">
+      <c r="B19" s="1">
         <v>3</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="56" t="s">
+      <c r="E19" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="F19" s="57">
+      <c r="F19" s="1">
         <v>5</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="57" t="s">
+      <c r="H19" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="I19" s="57">
+      <c r="I19" s="1">
         <v>84</v>
       </c>
-      <c r="J19" s="57" t="s">
+      <c r="J19" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="K19" s="58" t="s">
+      <c r="K19" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M19" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="N19" s="59">
+        <v>123</v>
+      </c>
+      <c r="N19" s="57">
         <v>4</v>
       </c>
-      <c r="O19" s="65" t="s">
+      <c r="O19" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P19" s="59">
-        <v>139</v>
+      <c r="P19" s="57">
+        <v>103</v>
       </c>
       <c r="Q19" s="18" t="s">
         <v>20</v>
@@ -5089,7 +5078,7 @@
       <c r="A20" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="B20" s="59">
+      <c r="B20" s="1">
         <v>3</v>
       </c>
       <c r="C20" s="18" t="s">
@@ -5098,45 +5087,45 @@
       <c r="E20" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="59">
+      <c r="F20" s="1">
         <v>1</v>
       </c>
-      <c r="G20" s="60" t="s">
+      <c r="G20" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="59" t="s">
+      <c r="H20" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I20" s="59">
+      <c r="I20" s="1">
         <v>36</v>
       </c>
-      <c r="J20" s="59" t="s">
+      <c r="J20" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K20" s="18" t="s">
         <v>4</v>
       </c>
       <c r="M20" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="N20" s="59">
+        <v>124</v>
+      </c>
+      <c r="N20" s="57">
         <v>4</v>
       </c>
-      <c r="O20" s="65" t="s">
+      <c r="O20" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P20" s="59">
-        <v>165</v>
+      <c r="P20" s="57">
+        <v>139</v>
       </c>
       <c r="Q20" s="18" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="B21" s="59">
+      <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="C21" s="18" t="s">
@@ -5145,37 +5134,37 @@
       <c r="E21" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="59">
+      <c r="F21" s="1">
         <v>2</v>
       </c>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="59" t="s">
+      <c r="H21" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="I21" s="59">
+      <c r="I21" s="1">
         <v>29</v>
       </c>
-      <c r="J21" s="59" t="s">
+      <c r="J21" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K21" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="M21" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="N21" s="20">
-        <v>5</v>
-      </c>
-      <c r="O21" s="27" t="s">
+      <c r="M21" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="N21" s="57">
+        <v>4</v>
+      </c>
+      <c r="O21" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="P21" s="20">
-        <v>214</v>
-      </c>
-      <c r="Q21" s="21" t="s">
+      <c r="P21" s="57">
+        <v>165</v>
+      </c>
+      <c r="Q21" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5183,7 +5172,7 @@
       <c r="A22" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="B22" s="59">
+      <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="18" t="s">
@@ -5192,30 +5181,45 @@
       <c r="E22" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="59">
+      <c r="F22" s="1">
         <v>3</v>
       </c>
-      <c r="G22" s="60" t="s">
+      <c r="G22" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="59" t="s">
+      <c r="H22" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="I22" s="59">
+      <c r="I22" s="1">
         <v>60</v>
       </c>
-      <c r="J22" s="59" t="s">
+      <c r="J22" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K22" s="18" t="s">
         <v>4</v>
+      </c>
+      <c r="M22" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="N22" s="57">
+        <v>5</v>
+      </c>
+      <c r="O22" s="58" t="s">
+        <v>17</v>
+      </c>
+      <c r="P22" s="57">
+        <v>194</v>
+      </c>
+      <c r="Q22" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="B23" s="59">
+      <c r="B23" s="1">
         <v>3</v>
       </c>
       <c r="C23" s="18" t="s">
@@ -5224,54 +5228,84 @@
       <c r="E23" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="F23" s="59">
+      <c r="F23" s="1">
         <v>4</v>
       </c>
-      <c r="G23" s="60" t="s">
+      <c r="G23" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="59" t="s">
+      <c r="H23" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="59">
+      <c r="I23" s="1">
         <v>95</v>
       </c>
-      <c r="J23" s="59" t="s">
+      <c r="J23" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K23" s="18" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="M23" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="N23" s="57">
+        <v>5</v>
+      </c>
+      <c r="O23" s="58" t="s">
+        <v>17</v>
+      </c>
+      <c r="P23" s="57">
+        <v>210</v>
+      </c>
+      <c r="Q23" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="B24" s="59">
+      <c r="B24" s="1">
         <v>3</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="56" t="s">
+      <c r="E24" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="F24" s="57">
+      <c r="F24" s="1">
         <v>5</v>
       </c>
-      <c r="G24" s="60" t="s">
+      <c r="G24" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="57" t="s">
+      <c r="H24" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="I24" s="57">
+      <c r="I24" s="1">
         <v>76</v>
       </c>
-      <c r="J24" s="57" t="s">
+      <c r="J24" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="K24" s="58" t="s">
+      <c r="K24" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="M24" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="N24" s="20">
+        <v>5</v>
+      </c>
+      <c r="O24" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="P24" s="20">
+        <v>214</v>
+      </c>
+      <c r="Q24" s="21" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5279,7 +5313,7 @@
       <c r="A25" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="B25" s="59">
+      <c r="B25" s="1">
         <v>3</v>
       </c>
       <c r="C25" s="18" t="s">
@@ -5288,19 +5322,19 @@
       <c r="E25" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="59">
+      <c r="F25" s="1">
         <v>3</v>
       </c>
-      <c r="G25" s="60" t="s">
+      <c r="G25" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="59" t="s">
+      <c r="H25" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="I25" s="59">
+      <c r="I25" s="1">
         <v>98</v>
       </c>
-      <c r="J25" s="59" t="s">
+      <c r="J25" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K25" s="18" t="s">
@@ -5311,7 +5345,7 @@
       <c r="A26" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="B26" s="59">
+      <c r="B26" s="1">
         <v>3</v>
       </c>
       <c r="C26" s="18" t="s">
@@ -5320,19 +5354,19 @@
       <c r="E26" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="59">
+      <c r="F26" s="1">
         <v>4</v>
       </c>
-      <c r="G26" s="60" t="s">
+      <c r="G26" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="59" t="s">
+      <c r="H26" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="I26" s="59">
+      <c r="I26" s="1">
         <v>174</v>
       </c>
-      <c r="J26" s="59" t="s">
+      <c r="J26" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K26" s="18" t="s">
@@ -5343,7 +5377,7 @@
       <c r="A27" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="B27" s="59">
+      <c r="B27" s="1">
         <v>3</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -5352,19 +5386,19 @@
       <c r="E27" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="F27" s="59">
+      <c r="F27" s="1">
         <v>5</v>
       </c>
-      <c r="G27" s="60" t="s">
+      <c r="G27" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="59" t="s">
+      <c r="H27" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="I27" s="59">
+      <c r="I27" s="1">
         <v>269</v>
       </c>
-      <c r="J27" s="59" t="s">
+      <c r="J27" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K27" s="18" t="s">
@@ -5375,7 +5409,7 @@
       <c r="A28" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="B28" s="59">
+      <c r="B28" s="1">
         <v>3</v>
       </c>
       <c r="C28" s="18" t="s">
@@ -5384,19 +5418,19 @@
       <c r="E28" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="59">
+      <c r="F28" s="1">
         <v>3</v>
       </c>
-      <c r="G28" s="60" t="s">
+      <c r="G28" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="59" t="s">
+      <c r="H28" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I28" s="61" t="s">
+      <c r="I28" s="35" t="s">
         <v>192</v>
       </c>
-      <c r="J28" s="59" t="s">
+      <c r="J28" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K28" s="18" t="s">
@@ -5407,7 +5441,7 @@
       <c r="A29" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="59">
+      <c r="B29" s="1">
         <v>3</v>
       </c>
       <c r="C29" s="18" t="s">
@@ -5416,19 +5450,19 @@
       <c r="E29" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="F29" s="59">
+      <c r="F29" s="1">
         <v>4</v>
       </c>
-      <c r="G29" s="60" t="s">
+      <c r="G29" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="59" t="s">
+      <c r="H29" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="I29" s="61" t="s">
+      <c r="I29" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="J29" s="59" t="s">
+      <c r="J29" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K29" s="18" t="s">
@@ -5439,7 +5473,7 @@
       <c r="A30" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="59">
+      <c r="B30" s="1">
         <v>4</v>
       </c>
       <c r="C30" s="18" t="s">
@@ -5448,19 +5482,19 @@
       <c r="E30" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="F30" s="59">
+      <c r="F30" s="1">
         <v>5</v>
       </c>
-      <c r="G30" s="60" t="s">
+      <c r="G30" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="59" t="s">
+      <c r="H30" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I30" s="61" t="s">
+      <c r="I30" s="35" t="s">
         <v>191</v>
       </c>
-      <c r="J30" s="59" t="s">
+      <c r="J30" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K30" s="18" t="s">
@@ -5471,7 +5505,7 @@
       <c r="A31" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="59">
+      <c r="B31" s="1">
         <v>5</v>
       </c>
       <c r="C31" s="18" t="s">
@@ -5480,19 +5514,19 @@
       <c r="E31" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F31" s="59">
+      <c r="F31" s="1">
         <v>2</v>
       </c>
-      <c r="G31" s="60" t="s">
+      <c r="G31" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="59" t="s">
+      <c r="H31" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="I31" s="59">
+      <c r="I31" s="1">
         <v>29</v>
       </c>
-      <c r="J31" s="59" t="s">
+      <c r="J31" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K31" s="18" t="s">
@@ -5503,7 +5537,7 @@
       <c r="A32" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="59">
+      <c r="B32" s="1">
         <v>5</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -5512,19 +5546,19 @@
       <c r="E32" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="F32" s="59">
+      <c r="F32" s="1">
         <v>3</v>
       </c>
-      <c r="G32" s="60" t="s">
+      <c r="G32" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="59" t="s">
+      <c r="H32" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="I32" s="59">
+      <c r="I32" s="1">
         <v>60</v>
       </c>
-      <c r="J32" s="59" t="s">
+      <c r="J32" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K32" s="18" t="s">
@@ -5544,19 +5578,19 @@
       <c r="E33" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F33" s="59">
+      <c r="F33" s="1">
         <v>4</v>
       </c>
-      <c r="G33" s="60" t="s">
+      <c r="G33" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="59" t="s">
+      <c r="H33" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I33" s="59">
+      <c r="I33" s="1">
         <v>95</v>
       </c>
-      <c r="J33" s="59" t="s">
+      <c r="J33" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K33" s="18" t="s">
@@ -5564,25 +5598,25 @@
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E34" s="56" t="s">
+      <c r="E34" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="F34" s="57">
+      <c r="F34" s="1">
         <v>5</v>
       </c>
-      <c r="G34" s="60" t="s">
+      <c r="G34" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H34" s="57" t="s">
+      <c r="H34" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="I34" s="57">
+      <c r="I34" s="1">
         <v>76</v>
       </c>
-      <c r="J34" s="57" t="s">
+      <c r="J34" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="K34" s="58" t="s">
+      <c r="K34" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5590,19 +5624,19 @@
       <c r="E35" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="F35" s="59">
+      <c r="F35" s="1">
         <v>1</v>
       </c>
-      <c r="G35" s="60" t="s">
+      <c r="G35" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="59" t="s">
+      <c r="H35" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="I35" s="59">
+      <c r="I35" s="1">
         <v>36</v>
       </c>
-      <c r="J35" s="59" t="s">
+      <c r="J35" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K35" s="18" t="s">
@@ -5613,19 +5647,19 @@
       <c r="E36" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="F36" s="59">
+      <c r="F36" s="1">
         <v>2</v>
       </c>
-      <c r="G36" s="60" t="s">
+      <c r="G36" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H36" s="59" t="s">
+      <c r="H36" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I36" s="59">
+      <c r="I36" s="1">
         <v>29</v>
       </c>
-      <c r="J36" s="59" t="s">
+      <c r="J36" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K36" s="18" t="s">
@@ -5636,19 +5670,19 @@
       <c r="E37" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="F37" s="59">
+      <c r="F37" s="1">
         <v>3</v>
       </c>
-      <c r="G37" s="60" t="s">
+      <c r="G37" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H37" s="59" t="s">
+      <c r="H37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I37" s="59">
+      <c r="I37" s="1">
         <v>60</v>
       </c>
-      <c r="J37" s="59" t="s">
+      <c r="J37" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K37" s="18" t="s">
@@ -5659,19 +5693,19 @@
       <c r="E38" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="F38" s="59">
+      <c r="F38" s="1">
         <v>4</v>
       </c>
-      <c r="G38" s="60" t="s">
+      <c r="G38" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="59" t="s">
+      <c r="H38" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I38" s="59">
+      <c r="I38" s="1">
         <v>95</v>
       </c>
-      <c r="J38" s="59" t="s">
+      <c r="J38" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K38" s="18" t="s">
@@ -5679,32 +5713,32 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E39" s="62" t="s">
+      <c r="E39" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="F39" s="63">
+      <c r="F39" s="20">
         <v>5</v>
       </c>
       <c r="G39" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="H39" s="63" t="s">
+      <c r="H39" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="I39" s="63">
+      <c r="I39" s="20">
         <v>76</v>
       </c>
-      <c r="J39" s="63" t="s">
+      <c r="J39" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="K39" s="64" t="s">
+      <c r="K39" s="21" t="s">
         <v>58</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C33">
-    <sortCondition ref="B4:B33"/>
-    <sortCondition ref="A4:A33"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M4:Q24">
+    <sortCondition ref="N4:N24"/>
+    <sortCondition ref="P4:P24"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Added Magma Floor 1 and Absorb/Repel ailments
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC4424B-F137-4B85-BC85-123438831C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EEA00EE-D6E9-4299-86AB-BCA0ED283714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="2265" windowWidth="21585" windowHeight="13440" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="235">
   <si>
     <t>Lv</t>
   </si>
@@ -676,9 +676,6 @@
     <t>Facility F5 Keycard B</t>
   </si>
   <si>
-    <t>Facility F5 Keycard C</t>
-  </si>
-  <si>
     <t>M6 Gerand</t>
   </si>
   <si>
@@ -686,6 +683,66 @@
   </si>
   <si>
     <t>Mega Bunsen Burner</t>
+  </si>
+  <si>
+    <t>Paquette Pylon</t>
+  </si>
+  <si>
+    <t>Eye of the Spark</t>
+  </si>
+  <si>
+    <t>Fitzroy Motherload</t>
+  </si>
+  <si>
+    <t>Eye of the Sun</t>
+  </si>
+  <si>
+    <t>F5 Twister in a Barrel</t>
+  </si>
+  <si>
+    <t>Eye of the Storm</t>
+  </si>
+  <si>
+    <t>Book of God - 2049 Edition</t>
+  </si>
+  <si>
+    <t>Blightaon</t>
+  </si>
+  <si>
+    <t>Orb of Dark Matter</t>
+  </si>
+  <si>
+    <t>Hexaon</t>
+  </si>
+  <si>
+    <t>Facility F6 Keycard</t>
+  </si>
+  <si>
+    <t>10 Dollar Coin</t>
+  </si>
+  <si>
+    <t>Chemical Pipette</t>
+  </si>
+  <si>
+    <t>x7 Melee</t>
+  </si>
+  <si>
+    <t>x7 Skill</t>
+  </si>
+  <si>
+    <t>Power Supplements 50mg</t>
+  </si>
+  <si>
+    <t>Concentration Pills 50mg</t>
+  </si>
+  <si>
+    <t>Enhanced Flask</t>
+  </si>
+  <si>
+    <t>+999 STA</t>
+  </si>
+  <si>
+    <t>Emergency Defibrilator</t>
   </si>
 </sst>
 </file>
@@ -958,7 +1015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1053,18 +1110,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1127,6 +1172,42 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1503,7 +1584,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="37" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1525,7 +1606,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="41"/>
+      <c r="F4" s="37"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1548,7 +1629,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="41"/>
+      <c r="F5" s="37"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1571,7 +1652,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="41"/>
+      <c r="F6" s="37"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1594,7 +1675,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="41"/>
+      <c r="F7" s="37"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1617,7 +1698,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="41"/>
+      <c r="F8" s="37"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1640,7 +1721,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="41"/>
+      <c r="F9" s="37"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1663,7 +1744,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="41"/>
+      <c r="F10" s="37"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1686,7 +1767,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="41"/>
+      <c r="F11" s="37"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1709,7 +1790,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="41"/>
+      <c r="F12" s="37"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1732,7 +1813,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="41"/>
+      <c r="F13" s="37"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1755,7 +1836,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="41"/>
+      <c r="F14" s="37"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1778,7 +1859,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="41"/>
+      <c r="F15" s="37"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1801,7 +1882,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="41"/>
+      <c r="F16" s="37"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1824,7 +1905,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="41"/>
+      <c r="F17" s="37"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1847,7 +1928,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="41"/>
+      <c r="F18" s="37"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1870,7 +1951,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="41"/>
+      <c r="F19" s="37"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1893,7 +1974,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="41"/>
+      <c r="F20" s="37"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1916,7 +1997,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="41"/>
+      <c r="F21" s="37"/>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -1939,7 +2020,7 @@
         <f t="shared" si="5"/>
         <v>17639</v>
       </c>
-      <c r="F22" s="41"/>
+      <c r="F22" s="37"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -1962,6 +2043,9 @@
         <f t="shared" ref="E23:E45" si="7">D23+E22</f>
         <v>23827</v>
       </c>
+      <c r="F23" s="66" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
@@ -1984,6 +2068,7 @@
         <f t="shared" si="7"/>
         <v>30479</v>
       </c>
+      <c r="F24" s="66"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -2006,6 +2091,7 @@
         <f t="shared" si="7"/>
         <v>37629</v>
       </c>
+      <c r="F25" s="66"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -2028,6 +2114,7 @@
         <f t="shared" si="7"/>
         <v>45315</v>
       </c>
+      <c r="F26" s="66"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -2050,6 +2137,7 @@
         <f t="shared" si="7"/>
         <v>53577</v>
       </c>
+      <c r="F27" s="66"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -2072,6 +2160,7 @@
         <f t="shared" si="7"/>
         <v>62458</v>
       </c>
+      <c r="F28" s="66"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -2094,6 +2183,7 @@
         <f t="shared" si="7"/>
         <v>72005</v>
       </c>
+      <c r="F29" s="66"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -2116,6 +2206,7 @@
         <f t="shared" si="7"/>
         <v>82268</v>
       </c>
+      <c r="F30" s="66"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -2138,6 +2229,7 @@
         <f t="shared" si="7"/>
         <v>93300</v>
       </c>
+      <c r="F31" s="66"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -2160,8 +2252,9 @@
         <f t="shared" si="7"/>
         <v>105159</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="66"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <f t="shared" si="6"/>
         <v>31</v>
@@ -2182,8 +2275,9 @@
         <f t="shared" si="7"/>
         <v>117907</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="66"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <f t="shared" si="6"/>
         <v>32</v>
@@ -2204,8 +2298,9 @@
         <f t="shared" si="7"/>
         <v>131611</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="66"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <f t="shared" si="6"/>
         <v>33</v>
@@ -2226,8 +2321,9 @@
         <f t="shared" si="7"/>
         <v>146342</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="66"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <f t="shared" si="6"/>
         <v>34</v>
@@ -2248,8 +2344,9 @@
         <f t="shared" si="7"/>
         <v>162177</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="66"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <f t="shared" si="6"/>
         <v>35</v>
@@ -2270,8 +2367,9 @@
         <f t="shared" si="7"/>
         <v>179199</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="66"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <f t="shared" si="6"/>
         <v>36</v>
@@ -2292,8 +2390,9 @@
         <f t="shared" si="7"/>
         <v>197497</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="66"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <f t="shared" si="6"/>
         <v>37</v>
@@ -2314,8 +2413,9 @@
         <f t="shared" si="7"/>
         <v>217167</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="66"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <f t="shared" si="6"/>
         <v>38</v>
@@ -2336,8 +2436,9 @@
         <f t="shared" si="7"/>
         <v>238312</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="66"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <f t="shared" si="6"/>
         <v>39</v>
@@ -2358,8 +2459,9 @@
         <f t="shared" si="7"/>
         <v>261042</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="66"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <f t="shared" si="6"/>
         <v>40</v>
@@ -2380,8 +2482,9 @@
         <f t="shared" si="7"/>
         <v>285476</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="66"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <f>A42+1</f>
         <v>41</v>
@@ -2402,8 +2505,9 @@
         <f t="shared" si="7"/>
         <v>311742</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="66"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <f>A43+1</f>
         <v>42</v>
@@ -2424,8 +2528,9 @@
         <f t="shared" si="7"/>
         <v>339977</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="66"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <f t="shared" ref="A45:A62" si="9">A44+1</f>
         <v>43</v>
@@ -2446,8 +2551,9 @@
         <f t="shared" si="7"/>
         <v>370329</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="66"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <f t="shared" si="9"/>
         <v>44</v>
@@ -2468,8 +2574,11 @@
         <f t="shared" ref="E46:E88" si="10">D46+E45</f>
         <v>402957</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="40" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <f t="shared" si="9"/>
         <v>45</v>
@@ -2490,8 +2599,9 @@
         <f t="shared" si="10"/>
         <v>438032</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="40"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <f t="shared" si="9"/>
         <v>46</v>
@@ -2512,8 +2622,9 @@
         <f t="shared" si="10"/>
         <v>475737</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="40"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <f t="shared" si="9"/>
         <v>47</v>
@@ -2534,8 +2645,9 @@
         <f t="shared" si="10"/>
         <v>516269</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="40"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <f t="shared" si="9"/>
         <v>48</v>
@@ -2556,8 +2668,9 @@
         <f t="shared" si="10"/>
         <v>559840</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" s="40"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <f t="shared" si="9"/>
         <v>49</v>
@@ -2578,8 +2691,9 @@
         <f t="shared" si="10"/>
         <v>606678</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" s="40"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <f t="shared" si="9"/>
         <v>50</v>
@@ -2600,8 +2714,9 @@
         <f t="shared" si="10"/>
         <v>657028</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" s="40"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <f t="shared" si="9"/>
         <v>51</v>
@@ -2622,8 +2737,9 @@
         <f t="shared" si="10"/>
         <v>708888</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" s="40"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <f t="shared" si="9"/>
         <v>52</v>
@@ -2644,8 +2760,9 @@
         <f t="shared" si="10"/>
         <v>762303</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" s="40"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <f t="shared" si="9"/>
         <v>53</v>
@@ -2666,8 +2783,9 @@
         <f t="shared" si="10"/>
         <v>817320</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" s="40"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <f t="shared" si="9"/>
         <v>54</v>
@@ -2689,7 +2807,7 @@
         <v>873987</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <f t="shared" si="9"/>
         <v>55</v>
@@ -2711,7 +2829,7 @@
         <v>932354</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <f t="shared" si="9"/>
         <v>56</v>
@@ -2733,7 +2851,7 @@
         <v>992472</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <f t="shared" si="9"/>
         <v>57</v>
@@ -2755,7 +2873,7 @@
         <v>1054393</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <f t="shared" si="9"/>
         <v>58</v>
@@ -2777,7 +2895,7 @@
         <v>1118171</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <f t="shared" si="9"/>
         <v>59</v>
@@ -2799,7 +2917,7 @@
         <v>1183862</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <f t="shared" si="9"/>
         <v>60</v>
@@ -2821,7 +2939,7 @@
         <v>1251523</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <f>A62+1</f>
         <v>61</v>
@@ -2843,7 +2961,7 @@
         <v>1321213</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <f>A63+1</f>
         <v>62</v>
@@ -3680,8 +3798,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="F3:F22"/>
+    <mergeCell ref="F23:F45"/>
+    <mergeCell ref="F46:F55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3710,10 +3830,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="42"/>
+      <c r="B3" s="38"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3728,214 +3848,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="43">
+      <c r="D4" s="39">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="55" t="s">
+      <c r="F4" s="51" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="44"/>
-      <c r="B5" s="51"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="44"/>
+      <c r="A5" s="40"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="40"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="41"/>
+      <c r="F5" s="37"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="44"/>
-      <c r="B6" s="51"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="44"/>
+      <c r="A6" s="40"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="40"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="41"/>
+      <c r="F6" s="37"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="45"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="45"/>
+      <c r="A7" s="41"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="41"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="56"/>
+      <c r="F7" s="52"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="53" t="s">
+      <c r="C8" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D8" s="40" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="41" t="s">
+      <c r="F8" s="37" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44"/>
-      <c r="B9" s="44"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="44"/>
+      <c r="A9" s="40"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="40"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="41"/>
+      <c r="F9" s="37"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="45"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="45"/>
+      <c r="A10" s="41"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="41"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="56"/>
+      <c r="F10" s="52"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="44">
+      <c r="D11" s="40">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="41" t="s">
+      <c r="F11" s="37" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="44"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="44"/>
+      <c r="A12" s="40"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="40"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="41"/>
+      <c r="F12" s="37"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="45"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="45"/>
+      <c r="A13" s="41"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="41"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="56"/>
+      <c r="F13" s="52"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="52" t="s">
+      <c r="C14" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="44" t="s">
+      <c r="D14" s="40" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="41" t="s">
+      <c r="F14" s="37" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
-      <c r="B15" s="44"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="44"/>
+      <c r="A15" s="40"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="40"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="41"/>
+      <c r="F15" s="37"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="45"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="45"/>
+      <c r="A16" s="41"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="41"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="56"/>
+      <c r="F16" s="52"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="44">
+      <c r="D17" s="40">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="41" t="s">
+      <c r="F17" s="37" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="44"/>
-      <c r="B18" s="44"/>
-      <c r="C18" s="49"/>
-      <c r="D18" s="44"/>
+      <c r="A18" s="40"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="40"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="41"/>
+      <c r="F18" s="37"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="45"/>
-      <c r="B19" s="45"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="45"/>
+      <c r="A19" s="41"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="41"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="56"/>
+      <c r="F19" s="52"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -3958,34 +4078,34 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="46" t="s">
+      <c r="B21" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="43">
+      <c r="D21" s="39">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="55" t="s">
+      <c r="F21" s="51" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="45"/>
-      <c r="B22" s="47"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="45"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="41"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="56"/>
+      <c r="F22" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -4028,7 +4148,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E36AA0E8-4612-49A3-9CD4-2D5734B3DCEA}">
-  <dimension ref="A1:W39"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -4036,7 +4156,7 @@
     <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
     <col min="5" max="5" width="25.140625" customWidth="1"/>
     <col min="6" max="6" width="3.140625" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" customWidth="1"/>
     <col min="9" max="9" width="9.42578125" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="22.5703125" customWidth="1"/>
@@ -4052,24 +4172,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="38"/>
+      <c r="B1" s="34"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="40"/>
+      <c r="B3" s="36"/>
       <c r="C3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="40"/>
+      <c r="F3" s="36"/>
       <c r="G3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4085,10 +4205,10 @@
       <c r="K3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="39" t="s">
+      <c r="M3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="40"/>
+      <c r="N3" s="36"/>
       <c r="O3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4098,10 +4218,10 @@
       <c r="Q3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="S3" s="39" t="s">
+      <c r="S3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="40"/>
+      <c r="T3" s="36"/>
       <c r="U3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4114,13 +4234,13 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>177</v>
+        <v>54</v>
       </c>
       <c r="B4" s="23">
         <v>1</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>65</v>
@@ -4176,9 +4296,9 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="1">
+        <v>53</v>
+      </c>
+      <c r="B5" s="53">
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
@@ -4187,19 +4307,19 @@
       <c r="E5" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="53">
         <v>3</v>
       </c>
-      <c r="G5" s="37" t="s">
+      <c r="G5" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="53" t="s">
         <v>179</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="53">
         <v>70</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="53" t="s">
         <v>150</v>
       </c>
       <c r="K5" s="18" t="s">
@@ -4208,13 +4328,13 @@
       <c r="M5" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="N5" s="57">
+      <c r="N5" s="53">
         <v>1</v>
       </c>
-      <c r="O5" s="58" t="s">
+      <c r="O5" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="57">
+      <c r="P5" s="53">
         <v>13</v>
       </c>
       <c r="Q5" s="18" t="s">
@@ -4223,13 +4343,13 @@
       <c r="S5" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="T5" s="1">
+      <c r="T5" s="53">
         <v>1</v>
       </c>
-      <c r="U5" s="34" t="s">
+      <c r="U5" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="35" t="s">
+      <c r="V5" s="59" t="s">
         <v>130</v>
       </c>
       <c r="W5" s="18" t="s">
@@ -4238,45 +4358,45 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="1">
+        <v>60</v>
+      </c>
+      <c r="B6" s="53">
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="37" t="s">
+      <c r="E6" s="55" t="s">
+        <v>221</v>
+      </c>
+      <c r="F6" s="56">
+        <v>4</v>
+      </c>
+      <c r="G6" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I6" s="1">
-        <v>44</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="K6" s="18" t="s">
-        <v>20</v>
+      <c r="H6" s="56" t="s">
+        <v>222</v>
+      </c>
+      <c r="I6" s="56">
+        <v>120</v>
+      </c>
+      <c r="J6" s="56" t="s">
+        <v>150</v>
+      </c>
+      <c r="K6" s="58" t="s">
+        <v>58</v>
       </c>
       <c r="M6" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="N6" s="57">
+      <c r="N6" s="53">
         <v>1</v>
       </c>
-      <c r="O6" s="58" t="s">
+      <c r="O6" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="57">
+      <c r="P6" s="53">
         <v>39</v>
       </c>
       <c r="Q6" s="18" t="s">
@@ -4285,13 +4405,13 @@
       <c r="S6" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="T6" s="1">
+      <c r="T6" s="53">
         <v>2</v>
       </c>
-      <c r="U6" s="34" t="s">
+      <c r="U6" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V6" s="35" t="s">
+      <c r="V6" s="59" t="s">
         <v>132</v>
       </c>
       <c r="W6" s="18" t="s">
@@ -4300,30 +4420,30 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="1">
+        <v>177</v>
+      </c>
+      <c r="B7" s="53">
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="F7" s="1">
-        <v>2</v>
-      </c>
-      <c r="G7" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="53">
+        <v>1</v>
+      </c>
+      <c r="G7" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I7" s="1">
-        <v>35</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="H7" s="53" t="s">
+        <v>78</v>
+      </c>
+      <c r="I7" s="53">
+        <v>44</v>
+      </c>
+      <c r="J7" s="53" t="s">
         <v>154</v>
       </c>
       <c r="K7" s="18" t="s">
@@ -4332,13 +4452,13 @@
       <c r="M7" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N7" s="57">
+      <c r="N7" s="53">
         <v>2</v>
       </c>
-      <c r="O7" s="58" t="s">
+      <c r="O7" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="57">
+      <c r="P7" s="53">
         <v>21</v>
       </c>
       <c r="Q7" s="18" t="s">
@@ -4347,13 +4467,13 @@
       <c r="S7" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="T7" s="1">
+      <c r="T7" s="53">
         <v>2</v>
       </c>
-      <c r="U7" s="34" t="s">
+      <c r="U7" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V7" s="35" t="s">
+      <c r="V7" s="59" t="s">
         <v>134</v>
       </c>
       <c r="W7" s="18" t="s">
@@ -4362,30 +4482,30 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="1">
+        <v>56</v>
+      </c>
+      <c r="B8" s="53">
         <v>1</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="F8" s="1">
-        <v>4</v>
-      </c>
-      <c r="G8" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8" s="53">
+        <v>2</v>
+      </c>
+      <c r="G8" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I8" s="1">
-        <v>56</v>
-      </c>
-      <c r="J8" s="1" t="s">
+      <c r="H8" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="53">
+        <v>35</v>
+      </c>
+      <c r="J8" s="53" t="s">
         <v>154</v>
       </c>
       <c r="K8" s="18" t="s">
@@ -4394,13 +4514,13 @@
       <c r="M8" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="N8" s="57">
+      <c r="N8" s="53">
         <v>2</v>
       </c>
-      <c r="O8" s="58" t="s">
+      <c r="O8" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="57">
+      <c r="P8" s="53">
         <v>56</v>
       </c>
       <c r="Q8" s="18" t="s">
@@ -4409,13 +4529,13 @@
       <c r="S8" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="T8" s="1">
+      <c r="T8" s="53">
         <v>3</v>
       </c>
-      <c r="U8" s="34" t="s">
+      <c r="U8" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V8" s="35" t="s">
+      <c r="V8" s="59" t="s">
         <v>136</v>
       </c>
       <c r="W8" s="18" t="s">
@@ -4424,31 +4544,31 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="1">
+        <v>50</v>
+      </c>
+      <c r="B9" s="53">
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" s="1">
-        <v>2</v>
-      </c>
-      <c r="G9" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="F9" s="53">
+        <v>4</v>
+      </c>
+      <c r="G9" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="I9" s="1">
-        <v>32</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>156</v>
+      <c r="H9" s="53" t="s">
+        <v>100</v>
+      </c>
+      <c r="I9" s="53">
+        <v>56</v>
+      </c>
+      <c r="J9" s="53" t="s">
+        <v>154</v>
       </c>
       <c r="K9" s="18" t="s">
         <v>20</v>
@@ -4456,13 +4576,13 @@
       <c r="M9" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="N9" s="57">
+      <c r="N9" s="53">
         <v>2</v>
       </c>
-      <c r="O9" s="58" t="s">
+      <c r="O9" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="57">
+      <c r="P9" s="53">
         <v>73</v>
       </c>
       <c r="Q9" s="18" t="s">
@@ -4471,13 +4591,13 @@
       <c r="S9" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="T9" s="1">
+      <c r="T9" s="53">
         <v>3</v>
       </c>
-      <c r="U9" s="34" t="s">
+      <c r="U9" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V9" s="35" t="s">
+      <c r="V9" s="59" t="s">
         <v>138</v>
       </c>
       <c r="W9" s="18" t="s">
@@ -4486,45 +4606,45 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="1">
+        <v>48</v>
+      </c>
+      <c r="B10" s="53">
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="55" t="s">
+        <v>223</v>
+      </c>
+      <c r="F10" s="56">
+        <v>4</v>
+      </c>
+      <c r="G10" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="I10" s="56">
+        <v>120</v>
+      </c>
+      <c r="J10" s="56" t="s">
+        <v>154</v>
+      </c>
+      <c r="K10" s="58" t="s">
         <v>58</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="F10" s="1">
-        <v>3</v>
-      </c>
-      <c r="G10" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I10" s="1">
-        <v>65</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="K10" s="18" t="s">
-        <v>4</v>
       </c>
       <c r="M10" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="N10" s="57">
+      <c r="N10" s="53">
         <v>3</v>
       </c>
-      <c r="O10" s="58" t="s">
+      <c r="O10" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="57">
+      <c r="P10" s="53">
         <v>36</v>
       </c>
       <c r="Q10" s="18" t="s">
@@ -4533,13 +4653,13 @@
       <c r="S10" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="T10" s="1">
+      <c r="T10" s="53">
         <v>3</v>
       </c>
-      <c r="U10" s="34" t="s">
+      <c r="U10" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="V10" s="53" t="s">
         <v>140</v>
       </c>
       <c r="W10" s="18" t="s">
@@ -4550,43 +4670,43 @@
       <c r="A11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="53">
         <v>2</v>
       </c>
       <c r="C11" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="F11" s="1">
-        <v>4</v>
-      </c>
-      <c r="G11" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="53">
+        <v>2</v>
+      </c>
+      <c r="G11" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="I11" s="1">
-        <v>52</v>
-      </c>
-      <c r="J11" s="1" t="s">
+      <c r="H11" s="53" t="s">
+        <v>109</v>
+      </c>
+      <c r="I11" s="53">
+        <v>32</v>
+      </c>
+      <c r="J11" s="53" t="s">
         <v>156</v>
       </c>
       <c r="K11" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="M11" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="N11" s="57">
+      <c r="N11" s="53">
         <v>3</v>
       </c>
-      <c r="O11" s="58" t="s">
+      <c r="O11" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="57">
+      <c r="P11" s="53">
         <v>46</v>
       </c>
       <c r="Q11" s="18" t="s">
@@ -4595,13 +4715,13 @@
       <c r="S11" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="T11" s="1">
+      <c r="T11" s="53">
         <v>3</v>
       </c>
-      <c r="U11" s="34" t="s">
+      <c r="U11" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V11" s="1" t="s">
+      <c r="V11" s="53" t="s">
         <v>142</v>
       </c>
       <c r="W11" s="18" t="s">
@@ -4610,45 +4730,45 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" s="1">
+        <v>62</v>
+      </c>
+      <c r="B12" s="53">
         <v>2</v>
       </c>
       <c r="C12" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="53">
+        <v>3</v>
+      </c>
+      <c r="G12" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="53" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" s="53">
+        <v>65</v>
+      </c>
+      <c r="J12" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="K12" s="18" t="s">
         <v>4</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="F12" s="1">
-        <v>4</v>
-      </c>
-      <c r="G12" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="I12" s="1">
-        <v>105</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="K12" s="18" t="s">
-        <v>20</v>
       </c>
       <c r="M12" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="N12" s="57">
+      <c r="N12" s="53">
         <v>3</v>
       </c>
-      <c r="O12" s="58" t="s">
+      <c r="O12" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P12" s="57">
+      <c r="P12" s="53">
         <v>71</v>
       </c>
       <c r="Q12" s="18" t="s">
@@ -4657,13 +4777,13 @@
       <c r="S12" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="T12" s="1">
+      <c r="T12" s="53">
         <v>4</v>
       </c>
-      <c r="U12" s="34" t="s">
+      <c r="U12" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V12" s="36" t="s">
+      <c r="V12" s="64" t="s">
         <v>144</v>
       </c>
       <c r="W12" s="18" t="s">
@@ -4672,45 +4792,45 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="1">
+        <v>208</v>
+      </c>
+      <c r="B13" s="53">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="F13" s="53">
         <v>4</v>
       </c>
-      <c r="E13" s="17" t="s">
-        <v>197</v>
-      </c>
-      <c r="F13" s="1">
-        <v>5</v>
-      </c>
-      <c r="G13" s="37" t="s">
+      <c r="G13" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="I13" s="1">
-        <v>84</v>
-      </c>
-      <c r="J13" s="1" t="s">
+      <c r="H13" s="53" t="s">
+        <v>174</v>
+      </c>
+      <c r="I13" s="53">
+        <v>52</v>
+      </c>
+      <c r="J13" s="53" t="s">
         <v>156</v>
       </c>
       <c r="K13" s="18" t="s">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="M13" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="N13" s="57">
+      <c r="N13" s="53">
         <v>3</v>
       </c>
-      <c r="O13" s="58" t="s">
+      <c r="O13" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="57">
+      <c r="P13" s="53">
         <v>78</v>
       </c>
       <c r="Q13" s="18" t="s">
@@ -4719,13 +4839,13 @@
       <c r="S13" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="53">
         <v>4</v>
       </c>
-      <c r="U13" s="34" t="s">
+      <c r="U13" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V13" s="1" t="s">
+      <c r="V13" s="53" t="s">
         <v>145</v>
       </c>
       <c r="W13" s="18" t="s">
@@ -4734,45 +4854,45 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="B14" s="1">
+        <v>51</v>
+      </c>
+      <c r="B14" s="53">
         <v>2</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="1">
-        <v>1</v>
-      </c>
-      <c r="G14" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F14" s="53">
+        <v>4</v>
+      </c>
+      <c r="G14" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I14" s="1">
-        <v>40</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>151</v>
+      <c r="H14" s="53" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="53">
+        <v>105</v>
+      </c>
+      <c r="J14" s="53" t="s">
+        <v>156</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="M14" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="N14" s="57">
+      <c r="N14" s="53">
         <v>3</v>
       </c>
-      <c r="O14" s="58" t="s">
+      <c r="O14" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P14" s="57">
+      <c r="P14" s="53">
         <v>86</v>
       </c>
       <c r="Q14" s="18" t="s">
@@ -4781,13 +4901,13 @@
       <c r="S14" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="53">
         <v>4</v>
       </c>
-      <c r="U14" s="34" t="s">
+      <c r="U14" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V14" s="1" t="s">
+      <c r="V14" s="53" t="s">
         <v>146</v>
       </c>
       <c r="W14" s="18" t="s">
@@ -4796,45 +4916,45 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="1">
+        <v>59</v>
+      </c>
+      <c r="B15" s="53">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" s="1">
-        <v>2</v>
-      </c>
-      <c r="G15" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="F15" s="53">
+        <v>5</v>
+      </c>
+      <c r="G15" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="I15" s="1">
-        <v>32</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>151</v>
+      <c r="H15" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="I15" s="53">
+        <v>84</v>
+      </c>
+      <c r="J15" s="53" t="s">
+        <v>156</v>
       </c>
       <c r="K15" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="M15" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="N15" s="57">
+        <v>214</v>
+      </c>
+      <c r="N15" s="53">
         <v>3</v>
       </c>
-      <c r="O15" s="58" t="s">
+      <c r="O15" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P15" s="57">
+      <c r="P15" s="53">
         <v>108</v>
       </c>
       <c r="Q15" s="18" t="s">
@@ -4843,13 +4963,13 @@
       <c r="S15" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="53">
         <v>4</v>
       </c>
-      <c r="U15" s="34" t="s">
+      <c r="U15" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V15" s="35" t="s">
+      <c r="V15" s="59" t="s">
         <v>186</v>
       </c>
       <c r="W15" s="18" t="s">
@@ -4860,43 +4980,43 @@
       <c r="A16" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="53">
         <v>2</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="F16" s="1">
-        <v>3</v>
-      </c>
-      <c r="G16" s="37" t="s">
+      <c r="E16" s="55" t="s">
+        <v>215</v>
+      </c>
+      <c r="F16" s="56">
+        <v>5</v>
+      </c>
+      <c r="G16" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I16" s="1">
-        <v>65</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="K16" s="18" t="s">
-        <v>20</v>
+      <c r="H16" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="I16" s="56">
+        <v>445</v>
+      </c>
+      <c r="J16" s="56" t="s">
+        <v>156</v>
+      </c>
+      <c r="K16" s="58" t="s">
+        <v>58</v>
       </c>
       <c r="M16" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="N16" s="57">
+      <c r="N16" s="53">
         <v>3</v>
       </c>
-      <c r="O16" s="58" t="s">
+      <c r="O16" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="57">
+      <c r="P16" s="53">
         <v>109</v>
       </c>
       <c r="Q16" s="18" t="s">
@@ -4905,310 +5025,370 @@
       <c r="S16" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="T16" s="1">
+      <c r="T16" s="53">
         <v>4</v>
       </c>
-      <c r="U16" s="34" t="s">
+      <c r="U16" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V16" s="35" t="s">
+      <c r="V16" s="59" t="s">
         <v>188</v>
       </c>
       <c r="W16" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>207</v>
-      </c>
-      <c r="B17" s="1">
+        <v>206</v>
+      </c>
+      <c r="B17" s="53">
         <v>3</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="F17" s="1">
+        <v>67</v>
+      </c>
+      <c r="F17" s="53">
+        <v>1</v>
+      </c>
+      <c r="G17" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="I17" s="53">
+        <v>40</v>
+      </c>
+      <c r="J17" s="53" t="s">
+        <v>151</v>
+      </c>
+      <c r="K17" s="18" t="s">
         <v>4</v>
-      </c>
-      <c r="G17" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="I17" s="1">
-        <v>52</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="K17" s="18" t="s">
-        <v>20</v>
       </c>
       <c r="M17" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="N17" s="57">
+      <c r="N17" s="53">
         <v>3</v>
       </c>
-      <c r="O17" s="58" t="s">
+      <c r="O17" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P17" s="57">
+      <c r="P17" s="53">
         <v>120</v>
       </c>
       <c r="Q17" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="S17" s="19" t="s">
+      <c r="S17" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="T17" s="20">
+      <c r="T17" s="53">
         <v>5</v>
       </c>
-      <c r="U17" s="29" t="s">
+      <c r="U17" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V17" s="20" t="s">
+      <c r="V17" s="53" t="s">
         <v>190</v>
       </c>
-      <c r="W17" s="21" t="s">
+      <c r="W17" s="18" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="1">
+        <v>169</v>
+      </c>
+      <c r="B18" s="53">
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="F18" s="1">
+        <v>69</v>
+      </c>
+      <c r="F18" s="53">
+        <v>2</v>
+      </c>
+      <c r="G18" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="I18" s="53">
+        <v>32</v>
+      </c>
+      <c r="J18" s="53" t="s">
+        <v>151</v>
+      </c>
+      <c r="K18" s="18" t="s">
         <v>4</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I18" s="1">
-        <v>105</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="K18" s="18" t="s">
-        <v>20</v>
       </c>
       <c r="M18" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="N18" s="57">
+      <c r="N18" s="53">
         <v>4</v>
       </c>
-      <c r="O18" s="58" t="s">
+      <c r="O18" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P18" s="57">
+      <c r="P18" s="53">
         <v>67</v>
       </c>
       <c r="Q18" s="18" t="s">
         <v>4</v>
       </c>
+      <c r="S18" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="T18" s="53">
+        <v>5</v>
+      </c>
+      <c r="U18" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="V18" s="53" t="s">
+        <v>228</v>
+      </c>
+      <c r="W18" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="B19" s="1">
+        <v>170</v>
+      </c>
+      <c r="B19" s="53">
         <v>3</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>194</v>
-      </c>
-      <c r="F19" s="1">
-        <v>5</v>
-      </c>
-      <c r="G19" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="F19" s="53">
+        <v>3</v>
+      </c>
+      <c r="G19" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="I19" s="1">
-        <v>84</v>
-      </c>
-      <c r="J19" s="1" t="s">
+      <c r="H19" s="53" t="s">
+        <v>182</v>
+      </c>
+      <c r="I19" s="53">
+        <v>65</v>
+      </c>
+      <c r="J19" s="53" t="s">
         <v>151</v>
       </c>
       <c r="K19" s="18" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="M19" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="N19" s="57">
+      <c r="N19" s="53">
         <v>4</v>
       </c>
-      <c r="O19" s="58" t="s">
+      <c r="O19" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P19" s="57">
+      <c r="P19" s="53">
         <v>103</v>
       </c>
       <c r="Q19" s="18" t="s">
         <v>20</v>
       </c>
+      <c r="S19" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="T19" s="53">
+        <v>5</v>
+      </c>
+      <c r="U19" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="V19" s="53" t="s">
+        <v>229</v>
+      </c>
+      <c r="W19" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="B20" s="1">
+        <v>171</v>
+      </c>
+      <c r="B20" s="53">
         <v>3</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="F20" s="1">
-        <v>1</v>
-      </c>
-      <c r="G20" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="53">
+        <v>4</v>
+      </c>
+      <c r="G20" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="I20" s="1">
-        <v>36</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>152</v>
+      <c r="H20" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="I20" s="53">
+        <v>52</v>
+      </c>
+      <c r="J20" s="53" t="s">
+        <v>151</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="M20" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="N20" s="57">
+      <c r="N20" s="53">
         <v>4</v>
       </c>
-      <c r="O20" s="58" t="s">
+      <c r="O20" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P20" s="57">
+      <c r="P20" s="53">
         <v>139</v>
       </c>
       <c r="Q20" s="18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S20" s="55" t="s">
+        <v>232</v>
+      </c>
+      <c r="T20" s="53">
+        <v>5</v>
+      </c>
+      <c r="U20" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="V20" s="59" t="s">
+        <v>233</v>
+      </c>
+      <c r="W20" s="58" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="B21" s="1">
+        <v>172</v>
+      </c>
+      <c r="B21" s="53">
         <v>3</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="F21" s="1">
-        <v>2</v>
-      </c>
-      <c r="G21" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="53">
+        <v>4</v>
+      </c>
+      <c r="G21" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="I21" s="1">
-        <v>29</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>152</v>
+      <c r="H21" s="53" t="s">
+        <v>82</v>
+      </c>
+      <c r="I21" s="53">
+        <v>105</v>
+      </c>
+      <c r="J21" s="53" t="s">
+        <v>151</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="M21" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="N21" s="57">
+      <c r="N21" s="53">
         <v>4</v>
       </c>
-      <c r="O21" s="58" t="s">
+      <c r="O21" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P21" s="57">
+      <c r="P21" s="53">
         <v>165</v>
       </c>
       <c r="Q21" s="18" t="s">
         <v>58</v>
       </c>
+      <c r="S21" s="60" t="s">
+        <v>234</v>
+      </c>
+      <c r="T21" s="20">
+        <v>5</v>
+      </c>
+      <c r="U21" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="V21" s="65" t="s">
+        <v>191</v>
+      </c>
+      <c r="W21" s="62" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>172</v>
-      </c>
-      <c r="B22" s="1">
+        <v>55</v>
+      </c>
+      <c r="B22" s="53">
         <v>3</v>
       </c>
       <c r="C22" s="18" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="F22" s="1">
-        <v>3</v>
-      </c>
-      <c r="G22" s="37" t="s">
+        <v>194</v>
+      </c>
+      <c r="F22" s="53">
+        <v>5</v>
+      </c>
+      <c r="G22" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="I22" s="1">
-        <v>60</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>152</v>
+      <c r="H22" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="I22" s="53">
+        <v>84</v>
+      </c>
+      <c r="J22" s="53" t="s">
+        <v>151</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="M22" s="17" t="s">
-        <v>213</v>
-      </c>
-      <c r="N22" s="57">
+        <v>212</v>
+      </c>
+      <c r="N22" s="53">
         <v>5</v>
       </c>
-      <c r="O22" s="58" t="s">
+      <c r="O22" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P22" s="57">
+      <c r="P22" s="53">
         <v>194</v>
       </c>
       <c r="Q22" s="18" t="s">
@@ -5217,45 +5397,45 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="B23" s="1">
+        <v>226</v>
+      </c>
+      <c r="B23" s="53">
         <v>3</v>
       </c>
       <c r="C23" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E23" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="F23" s="1">
-        <v>4</v>
-      </c>
-      <c r="G23" s="37" t="s">
+      <c r="E23" s="55" t="s">
+        <v>217</v>
+      </c>
+      <c r="F23" s="56">
+        <v>5</v>
+      </c>
+      <c r="G23" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" s="1">
-        <v>95</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K23" s="18" t="s">
+      <c r="H23" s="56" t="s">
+        <v>218</v>
+      </c>
+      <c r="I23" s="56">
+        <v>445</v>
+      </c>
+      <c r="J23" s="56" t="s">
+        <v>151</v>
+      </c>
+      <c r="K23" s="58" t="s">
         <v>58</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>214</v>
-      </c>
-      <c r="N23" s="57">
+        <v>213</v>
+      </c>
+      <c r="N23" s="53">
         <v>5</v>
       </c>
-      <c r="O23" s="58" t="s">
+      <c r="O23" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="P23" s="57">
+      <c r="P23" s="53">
         <v>210</v>
       </c>
       <c r="Q23" s="18" t="s">
@@ -5264,34 +5444,34 @@
     </row>
     <row r="24" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="B24" s="1">
+        <v>207</v>
+      </c>
+      <c r="B24" s="53">
         <v>3</v>
       </c>
       <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="F24" s="1">
-        <v>5</v>
-      </c>
-      <c r="G24" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="53">
+        <v>1</v>
+      </c>
+      <c r="G24" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="I24" s="1">
-        <v>76</v>
-      </c>
-      <c r="J24" s="1" t="s">
+      <c r="H24" s="53" t="s">
+        <v>84</v>
+      </c>
+      <c r="I24" s="53">
+        <v>36</v>
+      </c>
+      <c r="J24" s="53" t="s">
         <v>152</v>
       </c>
       <c r="K24" s="18" t="s">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="M24" s="19" t="s">
         <v>166</v>
@@ -5311,95 +5491,95 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>211</v>
-      </c>
-      <c r="B25" s="1">
+        <v>227</v>
+      </c>
+      <c r="B25" s="53">
         <v>3</v>
       </c>
       <c r="C25" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>101</v>
-      </c>
-      <c r="F25" s="1">
-        <v>3</v>
-      </c>
-      <c r="G25" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="53">
+        <v>2</v>
+      </c>
+      <c r="G25" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="I25" s="1">
-        <v>98</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>157</v>
+      <c r="H25" s="53" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="53">
+        <v>29</v>
+      </c>
+      <c r="J25" s="53" t="s">
+        <v>152</v>
       </c>
       <c r="K25" s="18" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>212</v>
-      </c>
-      <c r="B26" s="1">
+        <v>209</v>
+      </c>
+      <c r="B26" s="53">
         <v>3</v>
       </c>
       <c r="C26" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="F26" s="1">
+        <v>87</v>
+      </c>
+      <c r="F26" s="53">
+        <v>3</v>
+      </c>
+      <c r="G26" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="53" t="s">
+        <v>88</v>
+      </c>
+      <c r="I26" s="53">
+        <v>60</v>
+      </c>
+      <c r="J26" s="53" t="s">
+        <v>152</v>
+      </c>
+      <c r="K26" s="18" t="s">
         <v>4</v>
-      </c>
-      <c r="G26" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="I26" s="1">
-        <v>174</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="K26" s="18" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="B27" s="1">
+        <v>210</v>
+      </c>
+      <c r="B27" s="53">
         <v>3</v>
       </c>
       <c r="C27" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="F27" s="53">
         <v>4</v>
       </c>
-      <c r="E27" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="F27" s="1">
-        <v>5</v>
-      </c>
-      <c r="G27" s="37" t="s">
+      <c r="G27" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="I27" s="1">
-        <v>269</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>157</v>
+      <c r="H27" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" s="53">
+        <v>95</v>
+      </c>
+      <c r="J27" s="53" t="s">
+        <v>152</v>
       </c>
       <c r="K27" s="18" t="s">
         <v>58</v>
@@ -5407,63 +5587,63 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="B28" s="1">
+        <v>211</v>
+      </c>
+      <c r="B28" s="53">
         <v>3</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="F28" s="1">
-        <v>3</v>
-      </c>
-      <c r="G28" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="F28" s="53">
+        <v>5</v>
+      </c>
+      <c r="G28" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H28" s="53" t="s">
+        <v>201</v>
+      </c>
+      <c r="I28" s="53">
         <v>76</v>
       </c>
-      <c r="I28" s="35" t="s">
-        <v>192</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>158</v>
+      <c r="J28" s="53" t="s">
+        <v>152</v>
       </c>
       <c r="K28" s="18" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="1">
+        <v>225</v>
+      </c>
+      <c r="B29" s="53">
         <v>3</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="F29" s="1">
-        <v>4</v>
-      </c>
-      <c r="G29" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="F29" s="53">
+        <v>3</v>
+      </c>
+      <c r="G29" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I29" s="35" t="s">
-        <v>193</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>158</v>
+      <c r="H29" s="53" t="s">
+        <v>102</v>
+      </c>
+      <c r="I29" s="53">
+        <v>98</v>
+      </c>
+      <c r="J29" s="53" t="s">
+        <v>157</v>
       </c>
       <c r="K29" s="18" t="s">
         <v>20</v>
@@ -5471,274 +5651,406 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" s="1">
-        <v>4</v>
+        <v>167</v>
+      </c>
+      <c r="B30" s="53">
+        <v>3</v>
       </c>
       <c r="C30" s="18" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="F30" s="1">
-        <v>5</v>
-      </c>
-      <c r="G30" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="F30" s="53">
+        <v>4</v>
+      </c>
+      <c r="G30" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="I30" s="35" t="s">
-        <v>191</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>158</v>
+      <c r="H30" s="53" t="s">
+        <v>104</v>
+      </c>
+      <c r="I30" s="53">
+        <v>174</v>
+      </c>
+      <c r="J30" s="53" t="s">
+        <v>157</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" s="1">
+        <v>168</v>
+      </c>
+      <c r="B31" s="53">
+        <v>3</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="F31" s="53">
         <v>5</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="F31" s="1">
-        <v>2</v>
-      </c>
-      <c r="G31" s="37" t="s">
+      <c r="G31" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="I31" s="1">
-        <v>29</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>155</v>
+      <c r="H31" s="53" t="s">
+        <v>176</v>
+      </c>
+      <c r="I31" s="53">
+        <v>269</v>
+      </c>
+      <c r="J31" s="53" t="s">
+        <v>157</v>
       </c>
       <c r="K31" s="18" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="1">
+        <v>52</v>
+      </c>
+      <c r="B32" s="53">
+        <v>4</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F32" s="53">
+        <v>3</v>
+      </c>
+      <c r="G32" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="I32" s="59" t="s">
+        <v>192</v>
+      </c>
+      <c r="J32" s="53" t="s">
+        <v>158</v>
+      </c>
+      <c r="K32" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="53">
         <v>5</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C33" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E32" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="F32" s="1">
-        <v>3</v>
-      </c>
-      <c r="G32" s="37" t="s">
+      <c r="E33" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F33" s="53">
+        <v>4</v>
+      </c>
+      <c r="G33" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="I32" s="1">
-        <v>60</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="K32" s="18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="B33" s="20">
-        <v>5</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="E33" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="F33" s="1">
-        <v>4</v>
-      </c>
-      <c r="G33" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I33" s="1">
-        <v>95</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>155</v>
+      <c r="H33" s="53" t="s">
+        <v>80</v>
+      </c>
+      <c r="I33" s="59" t="s">
+        <v>193</v>
+      </c>
+      <c r="J33" s="53" t="s">
+        <v>158</v>
       </c>
       <c r="K33" s="18" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="53">
+        <v>5</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>20</v>
+      </c>
       <c r="E34" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="F34" s="1">
+        <v>183</v>
+      </c>
+      <c r="F34" s="53">
         <v>5</v>
       </c>
-      <c r="G34" s="37" t="s">
+      <c r="G34" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="I34" s="1">
-        <v>76</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>155</v>
+      <c r="H34" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" s="59" t="s">
+        <v>191</v>
+      </c>
+      <c r="J34" s="53" t="s">
+        <v>158</v>
       </c>
       <c r="K34" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="B35" s="20">
+        <v>5</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>58</v>
+      </c>
       <c r="E35" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="F35" s="1">
-        <v>1</v>
-      </c>
-      <c r="G35" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="F35" s="53">
+        <v>2</v>
+      </c>
+      <c r="G35" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="I35" s="1">
-        <v>36</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>153</v>
+      <c r="H35" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="I35" s="53">
+        <v>29</v>
+      </c>
+      <c r="J35" s="53" t="s">
+        <v>155</v>
       </c>
       <c r="K35" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="E36" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="F36" s="1">
-        <v>2</v>
-      </c>
-      <c r="G36" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="F36" s="53">
+        <v>3</v>
+      </c>
+      <c r="G36" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H36" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I36" s="1">
-        <v>29</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>153</v>
+      <c r="H36" s="53" t="s">
+        <v>106</v>
+      </c>
+      <c r="I36" s="53">
+        <v>60</v>
+      </c>
+      <c r="J36" s="53" t="s">
+        <v>155</v>
       </c>
       <c r="K36" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="E37" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="F37" s="1">
-        <v>3</v>
-      </c>
-      <c r="G37" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="F37" s="53">
+        <v>4</v>
+      </c>
+      <c r="G37" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H37" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="I37" s="1">
-        <v>60</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>153</v>
+      <c r="H37" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="I37" s="53">
+        <v>95</v>
+      </c>
+      <c r="J37" s="53" t="s">
+        <v>155</v>
       </c>
       <c r="K37" s="18" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="E38" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="F38" s="1">
-        <v>4</v>
-      </c>
-      <c r="G38" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="F38" s="53">
+        <v>5</v>
+      </c>
+      <c r="G38" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="I38" s="1">
-        <v>95</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>153</v>
+      <c r="H38" s="53" t="s">
+        <v>200</v>
+      </c>
+      <c r="I38" s="53">
+        <v>76</v>
+      </c>
+      <c r="J38" s="53" t="s">
+        <v>155</v>
       </c>
       <c r="K38" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E39" s="19" t="s">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E39" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F39" s="53">
+        <v>1</v>
+      </c>
+      <c r="G39" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H39" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="I39" s="53">
+        <v>36</v>
+      </c>
+      <c r="J39" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="K39" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E40" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F40" s="53">
+        <v>2</v>
+      </c>
+      <c r="G40" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H40" s="53" t="s">
+        <v>74</v>
+      </c>
+      <c r="I40" s="53">
+        <v>29</v>
+      </c>
+      <c r="J40" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="K40" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E41" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F41" s="53">
+        <v>3</v>
+      </c>
+      <c r="G41" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="I41" s="53">
+        <v>60</v>
+      </c>
+      <c r="J41" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="K41" s="18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E42" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="F42" s="53">
+        <v>4</v>
+      </c>
+      <c r="G42" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="53" t="s">
+        <v>160</v>
+      </c>
+      <c r="I42" s="53">
+        <v>95</v>
+      </c>
+      <c r="J42" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="K42" s="18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="E43" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="F39" s="20">
+      <c r="F43" s="53">
         <v>5</v>
       </c>
-      <c r="G39" s="25" t="s">
+      <c r="G43" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="H39" s="20" t="s">
+      <c r="H43" s="53" t="s">
         <v>203</v>
       </c>
-      <c r="I39" s="20">
+      <c r="I43" s="53">
         <v>76</v>
       </c>
-      <c r="J39" s="20" t="s">
+      <c r="J43" s="53" t="s">
         <v>204</v>
       </c>
-      <c r="K39" s="21" t="s">
+      <c r="K43" s="18" t="s">
         <v>58</v>
       </c>
     </row>
+    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E44" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="F44" s="61">
+        <v>5</v>
+      </c>
+      <c r="G44" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H44" s="61" t="s">
+        <v>220</v>
+      </c>
+      <c r="I44" s="61">
+        <v>445</v>
+      </c>
+      <c r="J44" s="61" t="s">
+        <v>153</v>
+      </c>
+      <c r="K44" s="62" t="s">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="M4:Q24">
-    <sortCondition ref="N4:N24"/>
-    <sortCondition ref="P4:P24"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="S4:W21">
+    <sortCondition ref="T4:T21"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Added Magma Floor 3 and Floor 4, Magma boss fight with gimmick
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EEA00EE-D6E9-4299-86AB-BCA0ED283714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0097926B-CAD3-42AC-8A2E-DE8D9DEB8F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-26175" yWindow="1095" windowWidth="21585" windowHeight="13515" activeTab="2" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="236">
   <si>
     <t>Lv</t>
   </si>
@@ -743,6 +743,9 @@
   </si>
   <si>
     <t>Emergency Defibrilator</t>
+  </si>
+  <si>
+    <t>Blunt Kunai</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1018,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1110,28 +1113,49 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1140,13 +1164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1161,53 +1179,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1584,7 +1566,7 @@
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="37" t="s">
+      <c r="F3" s="40" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1606,7 +1588,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="37"/>
+      <c r="F4" s="40"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1629,7 +1611,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="37"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1652,7 +1634,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="37"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1675,7 +1657,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="37"/>
+      <c r="F7" s="40"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1698,7 +1680,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="37"/>
+      <c r="F8" s="40"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1721,7 +1703,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="37"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1744,7 +1726,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="40"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1767,7 +1749,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="40"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1790,7 +1772,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="37"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1813,7 +1795,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="37"/>
+      <c r="F13" s="40"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1836,7 +1818,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="37"/>
+      <c r="F14" s="40"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1859,7 +1841,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="37"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1882,7 +1864,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="37"/>
+      <c r="F16" s="40"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1905,7 +1887,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="37"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1928,7 +1910,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="37"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1951,7 +1933,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="37"/>
+      <c r="F19" s="40"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1974,7 +1956,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="37"/>
+      <c r="F20" s="40"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1997,7 +1979,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="37"/>
+      <c r="F21" s="40"/>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -2020,7 +2002,7 @@
         <f t="shared" si="5"/>
         <v>17639</v>
       </c>
-      <c r="F22" s="37"/>
+      <c r="F22" s="40"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -2043,7 +2025,7 @@
         <f t="shared" ref="E23:E45" si="7">D23+E22</f>
         <v>23827</v>
       </c>
-      <c r="F23" s="66" t="s">
+      <c r="F23" s="41" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2068,7 +2050,7 @@
         <f t="shared" si="7"/>
         <v>30479</v>
       </c>
-      <c r="F24" s="66"/>
+      <c r="F24" s="41"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -2091,7 +2073,7 @@
         <f t="shared" si="7"/>
         <v>37629</v>
       </c>
-      <c r="F25" s="66"/>
+      <c r="F25" s="41"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -2114,7 +2096,7 @@
         <f t="shared" si="7"/>
         <v>45315</v>
       </c>
-      <c r="F26" s="66"/>
+      <c r="F26" s="41"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -2137,7 +2119,7 @@
         <f t="shared" si="7"/>
         <v>53577</v>
       </c>
-      <c r="F27" s="66"/>
+      <c r="F27" s="41"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -2160,7 +2142,7 @@
         <f t="shared" si="7"/>
         <v>62458</v>
       </c>
-      <c r="F28" s="66"/>
+      <c r="F28" s="41"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -2183,7 +2165,7 @@
         <f t="shared" si="7"/>
         <v>72005</v>
       </c>
-      <c r="F29" s="66"/>
+      <c r="F29" s="41"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -2206,7 +2188,7 @@
         <f t="shared" si="7"/>
         <v>82268</v>
       </c>
-      <c r="F30" s="66"/>
+      <c r="F30" s="41"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -2229,7 +2211,7 @@
         <f t="shared" si="7"/>
         <v>93300</v>
       </c>
-      <c r="F31" s="66"/>
+      <c r="F31" s="41"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -2252,7 +2234,7 @@
         <f t="shared" si="7"/>
         <v>105159</v>
       </c>
-      <c r="F32" s="66"/>
+      <c r="F32" s="41"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -2275,7 +2257,7 @@
         <f t="shared" si="7"/>
         <v>117907</v>
       </c>
-      <c r="F33" s="66"/>
+      <c r="F33" s="41"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -2298,7 +2280,7 @@
         <f t="shared" si="7"/>
         <v>131611</v>
       </c>
-      <c r="F34" s="66"/>
+      <c r="F34" s="41"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -2321,7 +2303,7 @@
         <f t="shared" si="7"/>
         <v>146342</v>
       </c>
-      <c r="F35" s="66"/>
+      <c r="F35" s="41"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -2344,7 +2326,7 @@
         <f t="shared" si="7"/>
         <v>162177</v>
       </c>
-      <c r="F36" s="66"/>
+      <c r="F36" s="41"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -2367,7 +2349,7 @@
         <f t="shared" si="7"/>
         <v>179199</v>
       </c>
-      <c r="F37" s="66"/>
+      <c r="F37" s="41"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -2390,7 +2372,7 @@
         <f t="shared" si="7"/>
         <v>197497</v>
       </c>
-      <c r="F38" s="66"/>
+      <c r="F38" s="41"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
@@ -2413,7 +2395,7 @@
         <f t="shared" si="7"/>
         <v>217167</v>
       </c>
-      <c r="F39" s="66"/>
+      <c r="F39" s="41"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
@@ -2436,7 +2418,7 @@
         <f t="shared" si="7"/>
         <v>238312</v>
       </c>
-      <c r="F40" s="66"/>
+      <c r="F40" s="41"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
@@ -2459,7 +2441,7 @@
         <f t="shared" si="7"/>
         <v>261042</v>
       </c>
-      <c r="F41" s="66"/>
+      <c r="F41" s="41"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
@@ -2482,7 +2464,7 @@
         <f t="shared" si="7"/>
         <v>285476</v>
       </c>
-      <c r="F42" s="66"/>
+      <c r="F42" s="41"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
@@ -2505,7 +2487,7 @@
         <f t="shared" si="7"/>
         <v>311742</v>
       </c>
-      <c r="F43" s="66"/>
+      <c r="F43" s="41"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
@@ -2528,7 +2510,7 @@
         <f t="shared" si="7"/>
         <v>339977</v>
       </c>
-      <c r="F44" s="66"/>
+      <c r="F44" s="41"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
@@ -2551,7 +2533,7 @@
         <f t="shared" si="7"/>
         <v>370329</v>
       </c>
-      <c r="F45" s="66"/>
+      <c r="F45" s="41"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
@@ -2574,7 +2556,7 @@
         <f t="shared" ref="E46:E88" si="10">D46+E45</f>
         <v>402957</v>
       </c>
-      <c r="F46" s="40" t="s">
+      <c r="F46" s="42" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2599,7 +2581,7 @@
         <f t="shared" si="10"/>
         <v>438032</v>
       </c>
-      <c r="F47" s="40"/>
+      <c r="F47" s="42"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
@@ -2622,7 +2604,7 @@
         <f t="shared" si="10"/>
         <v>475737</v>
       </c>
-      <c r="F48" s="40"/>
+      <c r="F48" s="42"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
@@ -2645,7 +2627,7 @@
         <f t="shared" si="10"/>
         <v>516269</v>
       </c>
-      <c r="F49" s="40"/>
+      <c r="F49" s="42"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
@@ -2668,7 +2650,7 @@
         <f t="shared" si="10"/>
         <v>559840</v>
       </c>
-      <c r="F50" s="40"/>
+      <c r="F50" s="42"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
@@ -2691,7 +2673,7 @@
         <f t="shared" si="10"/>
         <v>606678</v>
       </c>
-      <c r="F51" s="40"/>
+      <c r="F51" s="42"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
@@ -2714,7 +2696,7 @@
         <f t="shared" si="10"/>
         <v>657028</v>
       </c>
-      <c r="F52" s="40"/>
+      <c r="F52" s="42"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
@@ -2737,7 +2719,7 @@
         <f t="shared" si="10"/>
         <v>708888</v>
       </c>
-      <c r="F53" s="40"/>
+      <c r="F53" s="42"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
@@ -2760,7 +2742,7 @@
         <f t="shared" si="10"/>
         <v>762303</v>
       </c>
-      <c r="F54" s="40"/>
+      <c r="F54" s="42"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
@@ -2783,7 +2765,7 @@
         <f t="shared" si="10"/>
         <v>817320</v>
       </c>
-      <c r="F55" s="40"/>
+      <c r="F55" s="42"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
@@ -3830,10 +3812,10 @@
       <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="38"/>
+      <c r="B3" s="56"/>
       <c r="C3" s="12" t="s">
         <v>8</v>
       </c>
@@ -3848,214 +3830,214 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="39">
+      <c r="D4" s="43">
         <v>52</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="51" t="s">
+      <c r="F4" s="45" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="40"/>
-      <c r="B5" s="47"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="40"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="42"/>
       <c r="E5" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="37"/>
+      <c r="F5" s="40"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="40"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="40"/>
+      <c r="A6" s="42"/>
+      <c r="B6" s="52"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="42"/>
       <c r="E6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="37"/>
+      <c r="F6" s="40"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="41"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="41"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="44"/>
       <c r="E7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="52"/>
+      <c r="F7" s="46"/>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="42" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="40" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="40"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="42"/>
       <c r="E9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="37"/>
+      <c r="F9" s="40"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="41"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="41"/>
+      <c r="A10" s="44"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="44"/>
       <c r="E10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="52"/>
+      <c r="F10" s="46"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="44" t="s">
+      <c r="C11" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="40">
+      <c r="D11" s="42">
         <v>96</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="40" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="40"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="40"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="42"/>
       <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="37"/>
+      <c r="F12" s="40"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="41"/>
-      <c r="B13" s="41"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="41"/>
+      <c r="A13" s="44"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="44"/>
       <c r="E13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="52"/>
+      <c r="F13" s="46"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="42" t="s">
         <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="40" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="40"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="37"/>
+      <c r="F15" s="40"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="41"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="41"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="44"/>
       <c r="E16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="52"/>
+      <c r="F16" s="46"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="39" t="s">
+      <c r="A17" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="44" t="s">
+      <c r="C17" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="40">
+      <c r="D17" s="42">
         <v>137</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="40" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="40"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="42"/>
       <c r="E18" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="37"/>
+      <c r="F18" s="40"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="41"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="41"/>
+      <c r="A19" s="44"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="44"/>
       <c r="E19" t="s">
         <v>19</v>
       </c>
-      <c r="F19" s="52"/>
+      <c r="F19" s="46"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
@@ -4078,37 +4060,55 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="C21" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="39">
+      <c r="D21" s="43">
         <v>209</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="51" t="s">
+      <c r="F21" s="45" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="41"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="41"/>
+      <c r="A22" s="44"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="44"/>
       <c r="E22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F22" s="52"/>
+      <c r="F22" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C4:C7"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="C11:C13"/>
     <mergeCell ref="D4:D7"/>
     <mergeCell ref="F4:F7"/>
     <mergeCell ref="F21:F22"/>
@@ -4122,24 +4122,6 @@
     <mergeCell ref="D8:D10"/>
     <mergeCell ref="F17:F19"/>
     <mergeCell ref="D17:D19"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="A4:A7"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A17:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4172,24 +4154,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="34"/>
+      <c r="B1" s="57"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="36"/>
+      <c r="B3" s="59"/>
       <c r="C3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="36"/>
+      <c r="F3" s="59"/>
       <c r="G3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4205,10 +4187,10 @@
       <c r="K3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="M3" s="35" t="s">
+      <c r="M3" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="36"/>
+      <c r="N3" s="59"/>
       <c r="O3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4218,10 +4200,10 @@
       <c r="Q3" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="S3" s="35" t="s">
+      <c r="S3" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="36"/>
+      <c r="T3" s="59"/>
       <c r="U3" s="31" t="s">
         <v>8</v>
       </c>
@@ -4298,7 +4280,7 @@
       <c r="A5" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="53">
+      <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
@@ -4307,19 +4289,19 @@
       <c r="E5" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="F5" s="53">
+      <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="57" t="s">
+      <c r="G5" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="53" t="s">
+      <c r="H5" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="I5" s="53">
+      <c r="I5" s="1">
         <v>70</v>
       </c>
-      <c r="J5" s="53" t="s">
+      <c r="J5" s="1" t="s">
         <v>150</v>
       </c>
       <c r="K5" s="18" t="s">
@@ -4328,13 +4310,13 @@
       <c r="M5" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="N5" s="53">
+      <c r="N5" s="1">
         <v>1</v>
       </c>
-      <c r="O5" s="54" t="s">
+      <c r="O5" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="53">
+      <c r="P5" s="1">
         <v>13</v>
       </c>
       <c r="Q5" s="18" t="s">
@@ -4343,13 +4325,13 @@
       <c r="S5" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="T5" s="53">
+      <c r="T5" s="1">
         <v>1</v>
       </c>
-      <c r="U5" s="63" t="s">
+      <c r="U5" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="59" t="s">
+      <c r="V5" s="36" t="s">
         <v>130</v>
       </c>
       <c r="W5" s="18" t="s">
@@ -4360,43 +4342,43 @@
       <c r="A6" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="53">
+      <c r="B6" s="1">
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="F6" s="56">
+      <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="57" t="s">
+      <c r="G6" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="56" t="s">
+      <c r="H6" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="I6" s="56">
+      <c r="I6" s="1">
         <v>120</v>
       </c>
-      <c r="J6" s="56" t="s">
+      <c r="J6" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K6" s="58" t="s">
+      <c r="K6" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M6" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="N6" s="53">
+      <c r="N6" s="1">
         <v>1</v>
       </c>
-      <c r="O6" s="54" t="s">
+      <c r="O6" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="53">
+      <c r="P6" s="1">
         <v>39</v>
       </c>
       <c r="Q6" s="18" t="s">
@@ -4405,13 +4387,13 @@
       <c r="S6" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="T6" s="53">
+      <c r="T6" s="1">
         <v>2</v>
       </c>
-      <c r="U6" s="63" t="s">
+      <c r="U6" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V6" s="59" t="s">
+      <c r="V6" s="36" t="s">
         <v>132</v>
       </c>
       <c r="W6" s="18" t="s">
@@ -4422,7 +4404,7 @@
       <c r="A7" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="53">
+      <c r="B7" s="1">
         <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -4431,19 +4413,19 @@
       <c r="E7" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="53">
+      <c r="F7" s="1">
         <v>1</v>
       </c>
-      <c r="G7" s="57" t="s">
+      <c r="G7" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="53" t="s">
+      <c r="H7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I7" s="53">
+      <c r="I7" s="1">
         <v>44</v>
       </c>
-      <c r="J7" s="53" t="s">
+      <c r="J7" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K7" s="18" t="s">
@@ -4452,13 +4434,13 @@
       <c r="M7" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N7" s="53">
+      <c r="N7" s="1">
         <v>2</v>
       </c>
-      <c r="O7" s="54" t="s">
+      <c r="O7" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="53">
+      <c r="P7" s="1">
         <v>21</v>
       </c>
       <c r="Q7" s="18" t="s">
@@ -4467,13 +4449,13 @@
       <c r="S7" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="T7" s="53">
+      <c r="T7" s="1">
         <v>2</v>
       </c>
-      <c r="U7" s="63" t="s">
+      <c r="U7" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V7" s="59" t="s">
+      <c r="V7" s="36" t="s">
         <v>134</v>
       </c>
       <c r="W7" s="18" t="s">
@@ -4484,7 +4466,7 @@
       <c r="A8" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="1">
         <v>1</v>
       </c>
       <c r="C8" s="18" t="s">
@@ -4493,19 +4475,19 @@
       <c r="E8" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="F8" s="53">
+      <c r="F8" s="1">
         <v>2</v>
       </c>
-      <c r="G8" s="57" t="s">
+      <c r="G8" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="53" t="s">
+      <c r="H8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I8" s="53">
+      <c r="I8" s="1">
         <v>35</v>
       </c>
-      <c r="J8" s="53" t="s">
+      <c r="J8" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K8" s="18" t="s">
@@ -4514,13 +4496,13 @@
       <c r="M8" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="N8" s="53">
+      <c r="N8" s="1">
         <v>2</v>
       </c>
-      <c r="O8" s="54" t="s">
+      <c r="O8" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="53">
+      <c r="P8" s="1">
         <v>56</v>
       </c>
       <c r="Q8" s="18" t="s">
@@ -4529,13 +4511,13 @@
       <c r="S8" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="T8" s="53">
+      <c r="T8" s="1">
         <v>3</v>
       </c>
-      <c r="U8" s="63" t="s">
+      <c r="U8" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V8" s="59" t="s">
+      <c r="V8" s="36" t="s">
         <v>136</v>
       </c>
       <c r="W8" s="18" t="s">
@@ -4546,7 +4528,7 @@
       <c r="A9" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="1">
         <v>1</v>
       </c>
       <c r="C9" s="18" t="s">
@@ -4555,19 +4537,19 @@
       <c r="E9" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="1">
         <v>4</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="53" t="s">
+      <c r="H9" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I9" s="53">
+      <c r="I9" s="1">
         <v>56</v>
       </c>
-      <c r="J9" s="53" t="s">
+      <c r="J9" s="1" t="s">
         <v>154</v>
       </c>
       <c r="K9" s="18" t="s">
@@ -4576,13 +4558,13 @@
       <c r="M9" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="N9" s="53">
+      <c r="N9" s="1">
         <v>2</v>
       </c>
-      <c r="O9" s="54" t="s">
+      <c r="O9" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="53">
+      <c r="P9" s="1">
         <v>73</v>
       </c>
       <c r="Q9" s="18" t="s">
@@ -4591,13 +4573,13 @@
       <c r="S9" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="T9" s="53">
+      <c r="T9" s="1">
         <v>3</v>
       </c>
-      <c r="U9" s="63" t="s">
+      <c r="U9" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V9" s="59" t="s">
+      <c r="V9" s="36" t="s">
         <v>138</v>
       </c>
       <c r="W9" s="18" t="s">
@@ -4608,43 +4590,43 @@
       <c r="A10" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="53">
+      <c r="B10" s="1">
         <v>1</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="55" t="s">
+      <c r="E10" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="F10" s="56">
+      <c r="F10" s="1">
         <v>4</v>
       </c>
-      <c r="G10" s="57" t="s">
+      <c r="G10" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="56" t="s">
+      <c r="H10" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="I10" s="56">
+      <c r="I10" s="1">
         <v>120</v>
       </c>
-      <c r="J10" s="56" t="s">
+      <c r="J10" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="K10" s="58" t="s">
+      <c r="K10" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M10" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="N10" s="53">
+      <c r="N10" s="1">
         <v>3</v>
       </c>
-      <c r="O10" s="54" t="s">
+      <c r="O10" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="53">
+      <c r="P10" s="1">
         <v>36</v>
       </c>
       <c r="Q10" s="18" t="s">
@@ -4653,13 +4635,13 @@
       <c r="S10" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="T10" s="53">
+      <c r="T10" s="1">
         <v>3</v>
       </c>
-      <c r="U10" s="63" t="s">
+      <c r="U10" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V10" s="53" t="s">
+      <c r="V10" s="1" t="s">
         <v>140</v>
       </c>
       <c r="W10" s="18" t="s">
@@ -4670,7 +4652,7 @@
       <c r="A11" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="53">
+      <c r="B11" s="1">
         <v>2</v>
       </c>
       <c r="C11" s="18" t="s">
@@ -4679,19 +4661,19 @@
       <c r="E11" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="1">
         <v>2</v>
       </c>
-      <c r="G11" s="57" t="s">
+      <c r="G11" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="53" t="s">
+      <c r="H11" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I11" s="53">
+      <c r="I11" s="1">
         <v>32</v>
       </c>
-      <c r="J11" s="53" t="s">
+      <c r="J11" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K11" s="18" t="s">
@@ -4700,13 +4682,13 @@
       <c r="M11" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="N11" s="53">
+      <c r="N11" s="1">
         <v>3</v>
       </c>
-      <c r="O11" s="54" t="s">
+      <c r="O11" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="53">
+      <c r="P11" s="1">
         <v>46</v>
       </c>
       <c r="Q11" s="18" t="s">
@@ -4715,13 +4697,13 @@
       <c r="S11" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="T11" s="53">
+      <c r="T11" s="1">
         <v>3</v>
       </c>
-      <c r="U11" s="63" t="s">
+      <c r="U11" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V11" s="53" t="s">
+      <c r="V11" s="1" t="s">
         <v>142</v>
       </c>
       <c r="W11" s="18" t="s">
@@ -4732,7 +4714,7 @@
       <c r="A12" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="53">
+      <c r="B12" s="1">
         <v>2</v>
       </c>
       <c r="C12" s="18" t="s">
@@ -4741,19 +4723,19 @@
       <c r="E12" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="1">
         <v>3</v>
       </c>
-      <c r="G12" s="57" t="s">
+      <c r="G12" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="53" t="s">
+      <c r="H12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="I12" s="53">
+      <c r="I12" s="1">
         <v>65</v>
       </c>
-      <c r="J12" s="53" t="s">
+      <c r="J12" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K12" s="18" t="s">
@@ -4762,13 +4744,13 @@
       <c r="M12" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="N12" s="53">
+      <c r="N12" s="1">
         <v>3</v>
       </c>
-      <c r="O12" s="54" t="s">
+      <c r="O12" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P12" s="53">
+      <c r="P12" s="1">
         <v>71</v>
       </c>
       <c r="Q12" s="18" t="s">
@@ -4777,13 +4759,13 @@
       <c r="S12" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="T12" s="53">
+      <c r="T12" s="1">
         <v>4</v>
       </c>
-      <c r="U12" s="63" t="s">
+      <c r="U12" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V12" s="64" t="s">
+      <c r="V12" s="38" t="s">
         <v>144</v>
       </c>
       <c r="W12" s="18" t="s">
@@ -4794,7 +4776,7 @@
       <c r="A13" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="B13" s="53">
+      <c r="B13" s="1">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="s">
@@ -4803,19 +4785,19 @@
       <c r="E13" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="F13" s="53">
+      <c r="F13" s="1">
         <v>4</v>
       </c>
-      <c r="G13" s="57" t="s">
+      <c r="G13" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="53" t="s">
+      <c r="H13" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I13" s="53">
+      <c r="I13" s="1">
         <v>52</v>
       </c>
-      <c r="J13" s="53" t="s">
+      <c r="J13" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K13" s="18" t="s">
@@ -4824,13 +4806,13 @@
       <c r="M13" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="N13" s="53">
+      <c r="N13" s="1">
         <v>3</v>
       </c>
-      <c r="O13" s="54" t="s">
+      <c r="O13" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="53">
+      <c r="P13" s="1">
         <v>78</v>
       </c>
       <c r="Q13" s="18" t="s">
@@ -4839,13 +4821,13 @@
       <c r="S13" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="T13" s="53">
+      <c r="T13" s="1">
         <v>4</v>
       </c>
-      <c r="U13" s="63" t="s">
+      <c r="U13" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V13" s="53" t="s">
+      <c r="V13" s="1" t="s">
         <v>145</v>
       </c>
       <c r="W13" s="18" t="s">
@@ -4856,7 +4838,7 @@
       <c r="A14" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="53">
+      <c r="B14" s="1">
         <v>2</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -4865,19 +4847,19 @@
       <c r="E14" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="53">
+      <c r="F14" s="1">
         <v>4</v>
       </c>
-      <c r="G14" s="57" t="s">
+      <c r="G14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="53" t="s">
+      <c r="H14" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I14" s="53">
+      <c r="I14" s="1">
         <v>105</v>
       </c>
-      <c r="J14" s="53" t="s">
+      <c r="J14" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K14" s="18" t="s">
@@ -4886,13 +4868,13 @@
       <c r="M14" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="N14" s="53">
+      <c r="N14" s="1">
         <v>3</v>
       </c>
-      <c r="O14" s="54" t="s">
+      <c r="O14" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P14" s="53">
+      <c r="P14" s="1">
         <v>86</v>
       </c>
       <c r="Q14" s="18" t="s">
@@ -4901,13 +4883,13 @@
       <c r="S14" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="T14" s="53">
+      <c r="T14" s="1">
         <v>4</v>
       </c>
-      <c r="U14" s="63" t="s">
+      <c r="U14" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V14" s="53" t="s">
+      <c r="V14" s="1" t="s">
         <v>146</v>
       </c>
       <c r="W14" s="18" t="s">
@@ -4918,7 +4900,7 @@
       <c r="A15" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="53">
+      <c r="B15" s="1">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -4927,19 +4909,19 @@
       <c r="E15" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="1">
         <v>5</v>
       </c>
-      <c r="G15" s="57" t="s">
+      <c r="G15" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="53" t="s">
+      <c r="H15" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="I15" s="53">
+      <c r="I15" s="1">
         <v>84</v>
       </c>
-      <c r="J15" s="53" t="s">
+      <c r="J15" s="1" t="s">
         <v>156</v>
       </c>
       <c r="K15" s="18" t="s">
@@ -4948,13 +4930,13 @@
       <c r="M15" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="N15" s="53">
+      <c r="N15" s="1">
         <v>3</v>
       </c>
-      <c r="O15" s="54" t="s">
+      <c r="O15" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P15" s="53">
+      <c r="P15" s="1">
         <v>108</v>
       </c>
       <c r="Q15" s="18" t="s">
@@ -4963,13 +4945,13 @@
       <c r="S15" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="T15" s="53">
+      <c r="T15" s="1">
         <v>4</v>
       </c>
-      <c r="U15" s="63" t="s">
+      <c r="U15" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V15" s="59" t="s">
+      <c r="V15" s="36" t="s">
         <v>186</v>
       </c>
       <c r="W15" s="18" t="s">
@@ -4980,43 +4962,43 @@
       <c r="A16" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="53">
+      <c r="B16" s="1">
         <v>2</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="55" t="s">
+      <c r="E16" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="F16" s="56">
+      <c r="F16" s="1">
         <v>5</v>
       </c>
-      <c r="G16" s="57" t="s">
+      <c r="G16" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="56" t="s">
+      <c r="H16" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="1">
         <v>445</v>
       </c>
-      <c r="J16" s="56" t="s">
+      <c r="J16" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="K16" s="58" t="s">
+      <c r="K16" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M16" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="N16" s="53">
+      <c r="N16" s="1">
         <v>3</v>
       </c>
-      <c r="O16" s="54" t="s">
+      <c r="O16" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="53">
+      <c r="P16" s="1">
         <v>109</v>
       </c>
       <c r="Q16" s="18" t="s">
@@ -5025,13 +5007,13 @@
       <c r="S16" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="T16" s="53">
+      <c r="T16" s="1">
         <v>4</v>
       </c>
-      <c r="U16" s="63" t="s">
+      <c r="U16" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V16" s="59" t="s">
+      <c r="V16" s="36" t="s">
         <v>188</v>
       </c>
       <c r="W16" s="18" t="s">
@@ -5042,7 +5024,7 @@
       <c r="A17" s="17" t="s">
         <v>206</v>
       </c>
-      <c r="B17" s="53">
+      <c r="B17" s="1">
         <v>3</v>
       </c>
       <c r="C17" s="18" t="s">
@@ -5051,19 +5033,19 @@
       <c r="E17" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F17" s="53">
+      <c r="F17" s="1">
         <v>1</v>
       </c>
-      <c r="G17" s="57" t="s">
+      <c r="G17" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I17" s="53">
+      <c r="I17" s="1">
         <v>40</v>
       </c>
-      <c r="J17" s="53" t="s">
+      <c r="J17" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K17" s="18" t="s">
@@ -5072,13 +5054,13 @@
       <c r="M17" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="N17" s="53">
+      <c r="N17" s="1">
         <v>3</v>
       </c>
-      <c r="O17" s="54" t="s">
+      <c r="O17" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P17" s="53">
+      <c r="P17" s="1">
         <v>120</v>
       </c>
       <c r="Q17" s="18" t="s">
@@ -5087,13 +5069,13 @@
       <c r="S17" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="T17" s="53">
+      <c r="T17" s="1">
         <v>5</v>
       </c>
-      <c r="U17" s="63" t="s">
+      <c r="U17" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V17" s="53" t="s">
+      <c r="V17" s="1" t="s">
         <v>190</v>
       </c>
       <c r="W17" s="18" t="s">
@@ -5104,7 +5086,7 @@
       <c r="A18" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="B18" s="53">
+      <c r="B18" s="1">
         <v>3</v>
       </c>
       <c r="C18" s="18" t="s">
@@ -5113,19 +5095,19 @@
       <c r="E18" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="53">
+      <c r="F18" s="1">
         <v>2</v>
       </c>
-      <c r="G18" s="57" t="s">
+      <c r="G18" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H18" s="53" t="s">
+      <c r="H18" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="I18" s="53">
+      <c r="I18" s="1">
         <v>32</v>
       </c>
-      <c r="J18" s="53" t="s">
+      <c r="J18" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K18" s="18" t="s">
@@ -5134,13 +5116,13 @@
       <c r="M18" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="N18" s="53">
+      <c r="N18" s="1">
         <v>4</v>
       </c>
-      <c r="O18" s="54" t="s">
+      <c r="O18" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P18" s="53">
+      <c r="P18" s="1">
         <v>67</v>
       </c>
       <c r="Q18" s="18" t="s">
@@ -5149,13 +5131,13 @@
       <c r="S18" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="T18" s="53">
+      <c r="T18" s="1">
         <v>5</v>
       </c>
-      <c r="U18" s="63" t="s">
+      <c r="U18" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V18" s="53" t="s">
+      <c r="V18" s="1" t="s">
         <v>228</v>
       </c>
       <c r="W18" s="18" t="s">
@@ -5166,7 +5148,7 @@
       <c r="A19" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="B19" s="53">
+      <c r="B19" s="1">
         <v>3</v>
       </c>
       <c r="C19" s="18" t="s">
@@ -5175,19 +5157,19 @@
       <c r="E19" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="F19" s="53">
+      <c r="F19" s="1">
         <v>3</v>
       </c>
-      <c r="G19" s="57" t="s">
+      <c r="G19" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="53" t="s">
+      <c r="H19" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="I19" s="53">
+      <c r="I19" s="1">
         <v>65</v>
       </c>
-      <c r="J19" s="53" t="s">
+      <c r="J19" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K19" s="18" t="s">
@@ -5196,13 +5178,13 @@
       <c r="M19" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="N19" s="53">
+      <c r="N19" s="1">
         <v>4</v>
       </c>
-      <c r="O19" s="54" t="s">
+      <c r="O19" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P19" s="53">
+      <c r="P19" s="1">
         <v>103</v>
       </c>
       <c r="Q19" s="18" t="s">
@@ -5211,13 +5193,13 @@
       <c r="S19" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="T19" s="53">
+      <c r="T19" s="1">
         <v>5</v>
       </c>
-      <c r="U19" s="63" t="s">
+      <c r="U19" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V19" s="53" t="s">
+      <c r="V19" s="1" t="s">
         <v>229</v>
       </c>
       <c r="W19" s="18" t="s">
@@ -5228,7 +5210,7 @@
       <c r="A20" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="B20" s="53">
+      <c r="B20" s="1">
         <v>3</v>
       </c>
       <c r="C20" s="18" t="s">
@@ -5237,19 +5219,19 @@
       <c r="E20" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="F20" s="53">
+      <c r="F20" s="1">
         <v>4</v>
       </c>
-      <c r="G20" s="57" t="s">
+      <c r="G20" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="53" t="s">
+      <c r="H20" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="I20" s="53">
+      <c r="I20" s="1">
         <v>52</v>
       </c>
-      <c r="J20" s="53" t="s">
+      <c r="J20" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K20" s="18" t="s">
@@ -5258,31 +5240,31 @@
       <c r="M20" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="N20" s="53">
+      <c r="N20" s="1">
         <v>4</v>
       </c>
-      <c r="O20" s="54" t="s">
+      <c r="O20" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P20" s="53">
+      <c r="P20" s="1">
         <v>139</v>
       </c>
       <c r="Q20" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="S20" s="55" t="s">
+      <c r="S20" s="17" t="s">
         <v>232</v>
       </c>
-      <c r="T20" s="53">
+      <c r="T20" s="1">
         <v>5</v>
       </c>
-      <c r="U20" s="63" t="s">
+      <c r="U20" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="V20" s="59" t="s">
+      <c r="V20" s="36" t="s">
         <v>233</v>
       </c>
-      <c r="W20" s="58" t="s">
+      <c r="W20" s="18" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5290,7 +5272,7 @@
       <c r="A21" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="53">
+      <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="C21" s="18" t="s">
@@ -5299,19 +5281,19 @@
       <c r="E21" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="F21" s="53">
+      <c r="F21" s="1">
         <v>4</v>
       </c>
-      <c r="G21" s="57" t="s">
+      <c r="G21" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="53" t="s">
+      <c r="H21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I21" s="53">
+      <c r="I21" s="1">
         <v>105</v>
       </c>
-      <c r="J21" s="53" t="s">
+      <c r="J21" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K21" s="18" t="s">
@@ -5320,19 +5302,19 @@
       <c r="M21" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="N21" s="53">
+      <c r="N21" s="1">
         <v>4</v>
       </c>
-      <c r="O21" s="54" t="s">
+      <c r="O21" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P21" s="53">
+      <c r="P21" s="1">
         <v>165</v>
       </c>
       <c r="Q21" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="S21" s="60" t="s">
+      <c r="S21" s="19" t="s">
         <v>234</v>
       </c>
       <c r="T21" s="20">
@@ -5341,10 +5323,10 @@
       <c r="U21" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="V21" s="65" t="s">
+      <c r="V21" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="W21" s="62" t="s">
+      <c r="W21" s="21" t="s">
         <v>58</v>
       </c>
     </row>
@@ -5352,7 +5334,7 @@
       <c r="A22" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="53">
+      <c r="B22" s="1">
         <v>3</v>
       </c>
       <c r="C22" s="18" t="s">
@@ -5361,19 +5343,19 @@
       <c r="E22" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="F22" s="53">
+      <c r="F22" s="1">
         <v>5</v>
       </c>
-      <c r="G22" s="57" t="s">
+      <c r="G22" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="53" t="s">
+      <c r="H22" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="I22" s="53">
+      <c r="I22" s="1">
         <v>84</v>
       </c>
-      <c r="J22" s="53" t="s">
+      <c r="J22" s="1" t="s">
         <v>151</v>
       </c>
       <c r="K22" s="18" t="s">
@@ -5382,13 +5364,13 @@
       <c r="M22" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="N22" s="53">
+      <c r="N22" s="1">
         <v>5</v>
       </c>
-      <c r="O22" s="54" t="s">
+      <c r="O22" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P22" s="53">
+      <c r="P22" s="1">
         <v>194</v>
       </c>
       <c r="Q22" s="18" t="s">
@@ -5399,43 +5381,43 @@
       <c r="A23" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="B23" s="53">
+      <c r="B23" s="1">
         <v>3</v>
       </c>
       <c r="C23" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E23" s="55" t="s">
+      <c r="E23" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="F23" s="56">
+      <c r="F23" s="1">
         <v>5</v>
       </c>
-      <c r="G23" s="57" t="s">
+      <c r="G23" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H23" s="56" t="s">
+      <c r="H23" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="I23" s="56">
+      <c r="I23" s="1">
         <v>445</v>
       </c>
-      <c r="J23" s="56" t="s">
+      <c r="J23" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="K23" s="58" t="s">
+      <c r="K23" s="18" t="s">
         <v>58</v>
       </c>
       <c r="M23" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="N23" s="53">
+      <c r="N23" s="1">
         <v>5</v>
       </c>
-      <c r="O23" s="54" t="s">
+      <c r="O23" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="P23" s="53">
+      <c r="P23" s="1">
         <v>210</v>
       </c>
       <c r="Q23" s="18" t="s">
@@ -5446,7 +5428,7 @@
       <c r="A24" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="B24" s="53">
+      <c r="B24" s="1">
         <v>3</v>
       </c>
       <c r="C24" s="18" t="s">
@@ -5455,19 +5437,19 @@
       <c r="E24" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="F24" s="53">
+      <c r="F24" s="1">
         <v>1</v>
       </c>
-      <c r="G24" s="57" t="s">
+      <c r="G24" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H24" s="53" t="s">
+      <c r="H24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I24" s="53">
+      <c r="I24" s="1">
         <v>36</v>
       </c>
-      <c r="J24" s="53" t="s">
+      <c r="J24" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K24" s="18" t="s">
@@ -5493,7 +5475,7 @@
       <c r="A25" s="17" t="s">
         <v>227</v>
       </c>
-      <c r="B25" s="53">
+      <c r="B25" s="1">
         <v>3</v>
       </c>
       <c r="C25" s="18" t="s">
@@ -5502,30 +5484,45 @@
       <c r="E25" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="F25" s="53">
+      <c r="F25" s="1">
         <v>2</v>
       </c>
-      <c r="G25" s="57" t="s">
+      <c r="G25" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="53" t="s">
+      <c r="H25" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="I25" s="53">
+      <c r="I25" s="1">
         <v>29</v>
       </c>
-      <c r="J25" s="53" t="s">
+      <c r="J25" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K25" s="18" t="s">
         <v>4</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="N25" s="1">
+        <v>5</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P25" s="1">
+        <v>224</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="B26" s="53">
+      <c r="B26" s="1">
         <v>3</v>
       </c>
       <c r="C26" s="18" t="s">
@@ -5534,19 +5531,19 @@
       <c r="E26" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="F26" s="53">
+      <c r="F26" s="1">
         <v>3</v>
       </c>
-      <c r="G26" s="57" t="s">
+      <c r="G26" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="53" t="s">
+      <c r="H26" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="I26" s="53">
+      <c r="I26" s="1">
         <v>60</v>
       </c>
-      <c r="J26" s="53" t="s">
+      <c r="J26" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K26" s="18" t="s">
@@ -5557,7 +5554,7 @@
       <c r="A27" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="B27" s="53">
+      <c r="B27" s="1">
         <v>3</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -5566,19 +5563,19 @@
       <c r="E27" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="F27" s="53">
+      <c r="F27" s="1">
         <v>4</v>
       </c>
-      <c r="G27" s="57" t="s">
+      <c r="G27" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="53" t="s">
+      <c r="H27" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I27" s="53">
+      <c r="I27" s="1">
         <v>95</v>
       </c>
-      <c r="J27" s="53" t="s">
+      <c r="J27" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K27" s="18" t="s">
@@ -5589,7 +5586,7 @@
       <c r="A28" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="B28" s="53">
+      <c r="B28" s="1">
         <v>3</v>
       </c>
       <c r="C28" s="18" t="s">
@@ -5598,19 +5595,19 @@
       <c r="E28" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="F28" s="53">
+      <c r="F28" s="1">
         <v>5</v>
       </c>
-      <c r="G28" s="57" t="s">
+      <c r="G28" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="53" t="s">
+      <c r="H28" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="I28" s="53">
+      <c r="I28" s="1">
         <v>76</v>
       </c>
-      <c r="J28" s="53" t="s">
+      <c r="J28" s="1" t="s">
         <v>152</v>
       </c>
       <c r="K28" s="18" t="s">
@@ -5621,7 +5618,7 @@
       <c r="A29" s="17" t="s">
         <v>225</v>
       </c>
-      <c r="B29" s="53">
+      <c r="B29" s="1">
         <v>3</v>
       </c>
       <c r="C29" s="18" t="s">
@@ -5630,19 +5627,19 @@
       <c r="E29" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F29" s="53">
+      <c r="F29" s="1">
         <v>3</v>
       </c>
-      <c r="G29" s="57" t="s">
+      <c r="G29" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="53" t="s">
+      <c r="H29" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="I29" s="53">
+      <c r="I29" s="1">
         <v>98</v>
       </c>
-      <c r="J29" s="53" t="s">
+      <c r="J29" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K29" s="18" t="s">
@@ -5653,7 +5650,7 @@
       <c r="A30" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="B30" s="53">
+      <c r="B30" s="1">
         <v>3</v>
       </c>
       <c r="C30" s="18" t="s">
@@ -5662,19 +5659,19 @@
       <c r="E30" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="F30" s="53">
+      <c r="F30" s="1">
         <v>4</v>
       </c>
-      <c r="G30" s="57" t="s">
+      <c r="G30" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="53" t="s">
+      <c r="H30" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="I30" s="53">
+      <c r="I30" s="1">
         <v>174</v>
       </c>
-      <c r="J30" s="53" t="s">
+      <c r="J30" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K30" s="18" t="s">
@@ -5685,7 +5682,7 @@
       <c r="A31" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="B31" s="53">
+      <c r="B31" s="1">
         <v>3</v>
       </c>
       <c r="C31" s="18" t="s">
@@ -5694,19 +5691,19 @@
       <c r="E31" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="F31" s="53">
+      <c r="F31" s="1">
         <v>5</v>
       </c>
-      <c r="G31" s="57" t="s">
+      <c r="G31" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="53" t="s">
+      <c r="H31" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="I31" s="53">
+      <c r="I31" s="1">
         <v>269</v>
       </c>
-      <c r="J31" s="53" t="s">
+      <c r="J31" s="1" t="s">
         <v>157</v>
       </c>
       <c r="K31" s="18" t="s">
@@ -5717,7 +5714,7 @@
       <c r="A32" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="53">
+      <c r="B32" s="1">
         <v>4</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -5726,19 +5723,19 @@
       <c r="E32" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="F32" s="53">
+      <c r="F32" s="1">
         <v>3</v>
       </c>
-      <c r="G32" s="57" t="s">
+      <c r="G32" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="53" t="s">
+      <c r="H32" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I32" s="59" t="s">
+      <c r="I32" s="36" t="s">
         <v>192</v>
       </c>
-      <c r="J32" s="53" t="s">
+      <c r="J32" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K32" s="18" t="s">
@@ -5749,7 +5746,7 @@
       <c r="A33" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="53">
+      <c r="B33" s="1">
         <v>5</v>
       </c>
       <c r="C33" s="18" t="s">
@@ -5758,19 +5755,19 @@
       <c r="E33" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="F33" s="53">
+      <c r="F33" s="1">
         <v>4</v>
       </c>
-      <c r="G33" s="57" t="s">
+      <c r="G33" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="53" t="s">
+      <c r="H33" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="I33" s="59" t="s">
+      <c r="I33" s="36" t="s">
         <v>193</v>
       </c>
-      <c r="J33" s="53" t="s">
+      <c r="J33" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K33" s="18" t="s">
@@ -5781,7 +5778,7 @@
       <c r="A34" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="53">
+      <c r="B34" s="1">
         <v>5</v>
       </c>
       <c r="C34" s="18" t="s">
@@ -5790,19 +5787,19 @@
       <c r="E34" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="F34" s="53">
+      <c r="F34" s="1">
         <v>5</v>
       </c>
-      <c r="G34" s="57" t="s">
+      <c r="G34" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H34" s="53" t="s">
+      <c r="H34" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="I34" s="59" t="s">
+      <c r="I34" s="36" t="s">
         <v>191</v>
       </c>
-      <c r="J34" s="53" t="s">
+      <c r="J34" s="1" t="s">
         <v>158</v>
       </c>
       <c r="K34" s="18" t="s">
@@ -5822,19 +5819,19 @@
       <c r="E35" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F35" s="53">
+      <c r="F35" s="1">
         <v>2</v>
       </c>
-      <c r="G35" s="57" t="s">
+      <c r="G35" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="53" t="s">
+      <c r="H35" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="I35" s="53">
+      <c r="I35" s="1">
         <v>29</v>
       </c>
-      <c r="J35" s="53" t="s">
+      <c r="J35" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K35" s="18" t="s">
@@ -5845,19 +5842,19 @@
       <c r="E36" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="F36" s="53">
+      <c r="F36" s="1">
         <v>3</v>
       </c>
-      <c r="G36" s="57" t="s">
+      <c r="G36" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H36" s="53" t="s">
+      <c r="H36" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="I36" s="53">
+      <c r="I36" s="1">
         <v>60</v>
       </c>
-      <c r="J36" s="53" t="s">
+      <c r="J36" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K36" s="18" t="s">
@@ -5868,19 +5865,19 @@
       <c r="E37" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="F37" s="53">
+      <c r="F37" s="1">
         <v>4</v>
       </c>
-      <c r="G37" s="57" t="s">
+      <c r="G37" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H37" s="53" t="s">
+      <c r="H37" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I37" s="53">
+      <c r="I37" s="1">
         <v>95</v>
       </c>
-      <c r="J37" s="53" t="s">
+      <c r="J37" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K37" s="18" t="s">
@@ -5891,19 +5888,19 @@
       <c r="E38" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="F38" s="53">
+      <c r="F38" s="1">
         <v>5</v>
       </c>
-      <c r="G38" s="57" t="s">
+      <c r="G38" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="53" t="s">
+      <c r="H38" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="I38" s="53">
+      <c r="I38" s="1">
         <v>76</v>
       </c>
-      <c r="J38" s="53" t="s">
+      <c r="J38" s="1" t="s">
         <v>155</v>
       </c>
       <c r="K38" s="18" t="s">
@@ -5914,19 +5911,19 @@
       <c r="E39" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="F39" s="53">
+      <c r="F39" s="1">
         <v>1</v>
       </c>
-      <c r="G39" s="57" t="s">
+      <c r="G39" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H39" s="53" t="s">
+      <c r="H39" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="I39" s="53">
+      <c r="I39" s="1">
         <v>36</v>
       </c>
-      <c r="J39" s="53" t="s">
+      <c r="J39" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K39" s="18" t="s">
@@ -5937,19 +5934,19 @@
       <c r="E40" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="F40" s="53">
+      <c r="F40" s="1">
         <v>2</v>
       </c>
-      <c r="G40" s="57" t="s">
+      <c r="G40" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H40" s="53" t="s">
+      <c r="H40" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I40" s="53">
+      <c r="I40" s="1">
         <v>29</v>
       </c>
-      <c r="J40" s="53" t="s">
+      <c r="J40" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K40" s="18" t="s">
@@ -5960,19 +5957,19 @@
       <c r="E41" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="F41" s="53">
+      <c r="F41" s="1">
         <v>3</v>
       </c>
-      <c r="G41" s="57" t="s">
+      <c r="G41" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H41" s="53" t="s">
+      <c r="H41" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I41" s="53">
+      <c r="I41" s="1">
         <v>60</v>
       </c>
-      <c r="J41" s="53" t="s">
+      <c r="J41" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K41" s="18" t="s">
@@ -5983,19 +5980,19 @@
       <c r="E42" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="F42" s="53">
+      <c r="F42" s="1">
         <v>4</v>
       </c>
-      <c r="G42" s="57" t="s">
+      <c r="G42" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H42" s="53" t="s">
+      <c r="H42" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="I42" s="53">
+      <c r="I42" s="1">
         <v>95</v>
       </c>
-      <c r="J42" s="53" t="s">
+      <c r="J42" s="1" t="s">
         <v>153</v>
       </c>
       <c r="K42" s="18" t="s">
@@ -6006,19 +6003,19 @@
       <c r="E43" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="F43" s="53">
+      <c r="F43" s="1">
         <v>5</v>
       </c>
-      <c r="G43" s="57" t="s">
+      <c r="G43" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H43" s="53" t="s">
+      <c r="H43" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="I43" s="53">
+      <c r="I43" s="1">
         <v>76</v>
       </c>
-      <c r="J43" s="53" t="s">
+      <c r="J43" s="1" t="s">
         <v>204</v>
       </c>
       <c r="K43" s="18" t="s">
@@ -6026,25 +6023,25 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E44" s="60" t="s">
+      <c r="E44" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="F44" s="61">
+      <c r="F44" s="20">
         <v>5</v>
       </c>
       <c r="G44" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="H44" s="61" t="s">
+      <c r="H44" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="I44" s="61">
+      <c r="I44" s="20">
         <v>445</v>
       </c>
-      <c r="J44" s="61" t="s">
+      <c r="J44" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="K44" s="62" t="s">
+      <c r="K44" s="21" t="s">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v05_26.05 - Added Dungeon 6 + Optimisation
Read the patch notes included
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B93B57-139A-4EFA-BB2E-AD6BA0C7DF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D552AF-58F7-46ED-8AA7-A5B96110258B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24645" yWindow="1890" windowWidth="21585" windowHeight="13515" activeTab="1" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="1590" yWindow="1875" windowWidth="21585" windowHeight="13515" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -891,6 +891,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -908,9 +911,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1247,7 +1247,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C80B310D-5657-4E61-A0DA-301A4716D270}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A2:F101"/>
+  <dimension ref="A2:F102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="1"/>
@@ -1285,9 +1285,9 @@
       <c r="C3" s="1">
         <v>62</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="29" t="s">
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="30" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="29"/>
+      <c r="F4" s="30"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1332,7 +1332,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="29"/>
+      <c r="F5" s="30"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1355,7 +1355,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="29"/>
+      <c r="F6" s="30"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1378,7 +1378,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="29"/>
+      <c r="F7" s="30"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1401,7 +1401,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="29"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1424,7 +1424,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="29"/>
+      <c r="F9" s="30"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1447,7 +1447,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="29"/>
+      <c r="F10" s="30"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1470,7 +1470,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="29"/>
+      <c r="F11" s="30"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1493,7 +1493,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="29"/>
+      <c r="F12" s="30"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1516,7 +1516,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="29"/>
+      <c r="F13" s="30"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1539,7 +1539,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="29"/>
+      <c r="F14" s="30"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1562,7 +1562,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="29"/>
+      <c r="F15" s="30"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1585,7 +1585,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="29"/>
+      <c r="F16" s="30"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1608,7 +1608,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="29"/>
+      <c r="F17" s="30"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1631,7 +1631,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="29"/>
+      <c r="F18" s="30"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1654,7 +1654,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="29"/>
+      <c r="F19" s="30"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1677,7 +1677,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="29"/>
+      <c r="F20" s="30"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1700,7 +1700,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="29"/>
+      <c r="F21" s="30"/>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -1723,7 +1723,7 @@
         <f t="shared" si="5"/>
         <v>17639</v>
       </c>
-      <c r="F22" s="29"/>
+      <c r="F22" s="30"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -1746,7 +1746,7 @@
         <f t="shared" ref="E23:E45" si="7">D23+E22</f>
         <v>23827</v>
       </c>
-      <c r="F23" s="30" t="s">
+      <c r="F23" s="31" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
         <f t="shared" si="7"/>
         <v>30479</v>
       </c>
-      <c r="F24" s="30"/>
+      <c r="F24" s="31"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -1794,7 +1794,7 @@
         <f t="shared" si="7"/>
         <v>37629</v>
       </c>
-      <c r="F25" s="30"/>
+      <c r="F25" s="31"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -1817,7 +1817,7 @@
         <f t="shared" si="7"/>
         <v>45315</v>
       </c>
-      <c r="F26" s="30"/>
+      <c r="F26" s="31"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -1840,7 +1840,7 @@
         <f t="shared" si="7"/>
         <v>53577</v>
       </c>
-      <c r="F27" s="30"/>
+      <c r="F27" s="31"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -1863,7 +1863,7 @@
         <f t="shared" si="7"/>
         <v>62458</v>
       </c>
-      <c r="F28" s="30"/>
+      <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -1886,7 +1886,7 @@
         <f t="shared" si="7"/>
         <v>72005</v>
       </c>
-      <c r="F29" s="30"/>
+      <c r="F29" s="31"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -1909,7 +1909,7 @@
         <f t="shared" si="7"/>
         <v>82268</v>
       </c>
-      <c r="F30" s="30"/>
+      <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -1932,7 +1932,7 @@
         <f t="shared" si="7"/>
         <v>93300</v>
       </c>
-      <c r="F31" s="30"/>
+      <c r="F31" s="31"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -1955,7 +1955,7 @@
         <f t="shared" si="7"/>
         <v>105159</v>
       </c>
-      <c r="F32" s="30"/>
+      <c r="F32" s="31"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -1978,7 +1978,7 @@
         <f t="shared" si="7"/>
         <v>117907</v>
       </c>
-      <c r="F33" s="30"/>
+      <c r="F33" s="31"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -2001,7 +2001,7 @@
         <f t="shared" si="7"/>
         <v>131611</v>
       </c>
-      <c r="F34" s="30"/>
+      <c r="F34" s="31"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -2024,7 +2024,7 @@
         <f t="shared" si="7"/>
         <v>146342</v>
       </c>
-      <c r="F35" s="30"/>
+      <c r="F35" s="31"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -2047,7 +2047,7 @@
         <f t="shared" si="7"/>
         <v>162177</v>
       </c>
-      <c r="F36" s="30"/>
+      <c r="F36" s="31"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -2070,7 +2070,7 @@
         <f t="shared" si="7"/>
         <v>179199</v>
       </c>
-      <c r="F37" s="30"/>
+      <c r="F37" s="31"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -2093,7 +2093,7 @@
         <f t="shared" si="7"/>
         <v>197497</v>
       </c>
-      <c r="F38" s="30"/>
+      <c r="F38" s="31"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
@@ -2116,7 +2116,7 @@
         <f t="shared" si="7"/>
         <v>217167</v>
       </c>
-      <c r="F39" s="30"/>
+      <c r="F39" s="31"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
@@ -2139,7 +2139,7 @@
         <f t="shared" si="7"/>
         <v>238312</v>
       </c>
-      <c r="F40" s="30"/>
+      <c r="F40" s="31"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
@@ -2162,7 +2162,7 @@
         <f t="shared" si="7"/>
         <v>261042</v>
       </c>
-      <c r="F41" s="30"/>
+      <c r="F41" s="31"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
@@ -2185,7 +2185,7 @@
         <f t="shared" si="7"/>
         <v>285476</v>
       </c>
-      <c r="F42" s="30"/>
+      <c r="F42" s="31"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
@@ -2208,7 +2208,7 @@
         <f t="shared" si="7"/>
         <v>311742</v>
       </c>
-      <c r="F43" s="30"/>
+      <c r="F43" s="31"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
@@ -2231,7 +2231,7 @@
         <f t="shared" si="7"/>
         <v>339977</v>
       </c>
-      <c r="F44" s="30"/>
+      <c r="F44" s="31"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
@@ -2254,7 +2254,7 @@
         <f t="shared" si="7"/>
         <v>370329</v>
       </c>
-      <c r="F45" s="30"/>
+      <c r="F45" s="31"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
@@ -2277,7 +2277,7 @@
         <f t="shared" ref="E46:E88" si="10">D46+E45</f>
         <v>402957</v>
       </c>
-      <c r="F46" s="31" t="s">
+      <c r="F46" s="32" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
         <f t="shared" si="10"/>
         <v>438032</v>
       </c>
-      <c r="F47" s="31"/>
+      <c r="F47" s="32"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
@@ -2325,7 +2325,7 @@
         <f t="shared" si="10"/>
         <v>475737</v>
       </c>
-      <c r="F48" s="31"/>
+      <c r="F48" s="32"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
@@ -2348,7 +2348,7 @@
         <f t="shared" si="10"/>
         <v>516269</v>
       </c>
-      <c r="F49" s="31"/>
+      <c r="F49" s="32"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
@@ -2371,7 +2371,7 @@
         <f t="shared" si="10"/>
         <v>559840</v>
       </c>
-      <c r="F50" s="31"/>
+      <c r="F50" s="32"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
@@ -2394,7 +2394,7 @@
         <f t="shared" si="10"/>
         <v>606678</v>
       </c>
-      <c r="F51" s="31"/>
+      <c r="F51" s="32"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
@@ -2417,7 +2417,7 @@
         <f t="shared" si="10"/>
         <v>657028</v>
       </c>
-      <c r="F52" s="31"/>
+      <c r="F52" s="32"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
@@ -2440,7 +2440,7 @@
         <f t="shared" si="10"/>
         <v>708888</v>
       </c>
-      <c r="F53" s="31"/>
+      <c r="F53" s="32"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
@@ -2456,14 +2456,14 @@
         <v>266</v>
       </c>
       <c r="D54" s="1">
-        <f t="shared" ref="D54:D101" si="11">INT(D53*1.03)</f>
+        <f t="shared" ref="D54:D102" si="11">INT(D53*1.03)</f>
         <v>53415</v>
       </c>
       <c r="E54" s="1">
         <f t="shared" si="10"/>
         <v>762303</v>
       </c>
-      <c r="F54" s="31"/>
+      <c r="F54" s="32"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
@@ -2486,7 +2486,7 @@
         <f t="shared" si="10"/>
         <v>817320</v>
       </c>
-      <c r="F55" s="31"/>
+      <c r="F55" s="32"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
@@ -2509,7 +2509,7 @@
         <f t="shared" si="10"/>
         <v>873987</v>
       </c>
-      <c r="F56" s="31"/>
+      <c r="F56" s="32"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
@@ -2532,7 +2532,7 @@
         <f t="shared" si="10"/>
         <v>932354</v>
       </c>
-      <c r="F57" s="31"/>
+      <c r="F57" s="32"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
@@ -2555,7 +2555,7 @@
         <f t="shared" si="10"/>
         <v>992472</v>
       </c>
-      <c r="F58" s="31"/>
+      <c r="F58" s="32"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
@@ -2578,7 +2578,7 @@
         <f t="shared" si="10"/>
         <v>1054393</v>
       </c>
-      <c r="F59" s="31"/>
+      <c r="F59" s="32"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
@@ -2601,7 +2601,7 @@
         <f t="shared" si="10"/>
         <v>1118171</v>
       </c>
-      <c r="F60" s="31"/>
+      <c r="F60" s="32"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
@@ -2624,7 +2624,7 @@
         <f t="shared" si="10"/>
         <v>1183862</v>
       </c>
-      <c r="F61" s="31"/>
+      <c r="F61" s="32"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
@@ -2647,7 +2647,7 @@
         <f t="shared" si="10"/>
         <v>1251523</v>
       </c>
-      <c r="F62" s="31"/>
+      <c r="F62" s="32"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
@@ -2670,7 +2670,7 @@
         <f t="shared" si="10"/>
         <v>1321213</v>
       </c>
-      <c r="F63" s="30" t="s">
+      <c r="F63" s="31" t="s">
         <v>204</v>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
         <f t="shared" si="10"/>
         <v>1392993</v>
       </c>
-      <c r="F64" s="30"/>
+      <c r="F64" s="31"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
@@ -2718,7 +2718,7 @@
         <f t="shared" si="10"/>
         <v>1466926</v>
       </c>
-      <c r="F65" s="30"/>
+      <c r="F65" s="31"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
@@ -2741,7 +2741,7 @@
         <f t="shared" si="10"/>
         <v>1543076</v>
       </c>
-      <c r="F66" s="30"/>
+      <c r="F66" s="31"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
@@ -2764,7 +2764,7 @@
         <f t="shared" si="10"/>
         <v>1621510</v>
       </c>
-      <c r="F67" s="30"/>
+      <c r="F67" s="31"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
@@ -2787,7 +2787,7 @@
         <f t="shared" si="10"/>
         <v>1702297</v>
       </c>
-      <c r="F68" s="30"/>
+      <c r="F68" s="31"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
@@ -2795,11 +2795,11 @@
         <v>67</v>
       </c>
       <c r="B69" s="1">
-        <f t="shared" ref="B69:B101" si="13">(B68+7)</f>
+        <f t="shared" ref="B69:B102" si="13">(B68+7)</f>
         <v>602</v>
       </c>
       <c r="C69" s="1">
-        <f t="shared" ref="C69:C101" si="14">(C68+4)</f>
+        <f t="shared" ref="C69:C102" si="14">(C68+4)</f>
         <v>326</v>
       </c>
       <c r="D69" s="1">
@@ -2810,7 +2810,7 @@
         <f t="shared" si="10"/>
         <v>1785507</v>
       </c>
-      <c r="F69" s="30"/>
+      <c r="F69" s="31"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
@@ -2833,7 +2833,7 @@
         <f t="shared" si="10"/>
         <v>1871213</v>
       </c>
-      <c r="F70" s="30"/>
+      <c r="F70" s="31"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
@@ -2856,7 +2856,7 @@
         <f t="shared" si="10"/>
         <v>1959490</v>
       </c>
-      <c r="F71" s="30"/>
+      <c r="F71" s="31"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
@@ -2879,7 +2879,7 @@
         <f t="shared" si="10"/>
         <v>2050415</v>
       </c>
-      <c r="F72" s="30"/>
+      <c r="F72" s="31"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
@@ -2902,7 +2902,7 @@
         <f t="shared" si="10"/>
         <v>2144067</v>
       </c>
-      <c r="F73" s="30"/>
+      <c r="F73" s="31"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
@@ -2925,7 +2925,7 @@
         <f t="shared" si="10"/>
         <v>2240528</v>
       </c>
-      <c r="F74" s="30"/>
+      <c r="F74" s="31"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
@@ -2948,7 +2948,7 @@
         <f t="shared" si="10"/>
         <v>2339882</v>
       </c>
-      <c r="F75" s="30"/>
+      <c r="F75" s="31"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
@@ -2971,7 +2971,7 @@
         <f t="shared" si="10"/>
         <v>2442216</v>
       </c>
-      <c r="F76" s="30"/>
+      <c r="F76" s="31"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
@@ -2994,7 +2994,7 @@
         <f t="shared" si="10"/>
         <v>2547620</v>
       </c>
-      <c r="F77" s="30"/>
+      <c r="F77" s="31"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
@@ -3017,7 +3017,7 @@
         <f t="shared" si="10"/>
         <v>2656186</v>
       </c>
-      <c r="F78" s="30"/>
+      <c r="F78" s="31"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
@@ -3040,7 +3040,7 @@
         <f t="shared" si="10"/>
         <v>2768008</v>
       </c>
-      <c r="F79" s="30"/>
+      <c r="F79" s="31"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
@@ -3063,7 +3063,7 @@
         <f t="shared" si="10"/>
         <v>2883184</v>
       </c>
-      <c r="F80" s="30"/>
+      <c r="F80" s="31"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
@@ -3086,7 +3086,7 @@
         <f t="shared" si="10"/>
         <v>3001815</v>
       </c>
-      <c r="F81" s="30"/>
+      <c r="F81" s="31"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
@@ -3109,7 +3109,7 @@
         <f t="shared" si="10"/>
         <v>3124004</v>
       </c>
-      <c r="F82" s="30"/>
+      <c r="F82" s="31"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
@@ -3132,7 +3132,7 @@
         <f t="shared" si="10"/>
         <v>3249858</v>
       </c>
-      <c r="F83" s="30"/>
+      <c r="F83" s="31"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
@@ -3155,7 +3155,7 @@
         <f t="shared" si="10"/>
         <v>3379487</v>
       </c>
-      <c r="F84" s="30"/>
+      <c r="F84" s="31"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
@@ -3178,7 +3178,7 @@
         <f t="shared" si="10"/>
         <v>3513004</v>
       </c>
-      <c r="F85" s="30"/>
+      <c r="F85" s="31"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
@@ -3201,7 +3201,7 @@
         <f t="shared" si="10"/>
         <v>3650526</v>
       </c>
-      <c r="F86" s="30"/>
+      <c r="F86" s="31"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
@@ -3224,11 +3224,11 @@
         <f t="shared" si="10"/>
         <v>3792173</v>
       </c>
-      <c r="F87" s="30"/>
+      <c r="F87" s="31"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <f t="shared" ref="A88:A101" si="15">A87+1</f>
+        <f t="shared" ref="A88:A102" si="15">A87+1</f>
         <v>86</v>
       </c>
       <c r="B88" s="1">
@@ -3247,7 +3247,7 @@
         <f t="shared" si="10"/>
         <v>3938069</v>
       </c>
-      <c r="F88" s="30"/>
+      <c r="F88" s="31"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
@@ -3267,10 +3267,10 @@
         <v>150272</v>
       </c>
       <c r="E89" s="1">
-        <f t="shared" ref="E89:E101" si="16">D89+E88</f>
+        <f t="shared" ref="E89:E102" si="16">D89+E88</f>
         <v>4088341</v>
       </c>
-      <c r="F89" s="30"/>
+      <c r="F89" s="31"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
@@ -3293,7 +3293,7 @@
         <f t="shared" si="16"/>
         <v>4243121</v>
       </c>
-      <c r="F90" s="30"/>
+      <c r="F90" s="31"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
@@ -3316,7 +3316,7 @@
         <f t="shared" si="16"/>
         <v>4402544</v>
       </c>
-      <c r="F91" s="30"/>
+      <c r="F91" s="31"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
@@ -3339,7 +3339,7 @@
         <f t="shared" si="16"/>
         <v>4566749</v>
       </c>
-      <c r="F92" s="30"/>
+      <c r="F92" s="31"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
@@ -3362,7 +3362,7 @@
         <f t="shared" si="16"/>
         <v>4735880</v>
       </c>
-      <c r="F93" s="30"/>
+      <c r="F93" s="31"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
@@ -3385,7 +3385,7 @@
         <f t="shared" si="16"/>
         <v>4910084</v>
       </c>
-      <c r="F94" s="30"/>
+      <c r="F94" s="31"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
@@ -3408,7 +3408,7 @@
         <f t="shared" si="16"/>
         <v>5089514</v>
       </c>
-      <c r="F95" s="30"/>
+      <c r="F95" s="31"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
@@ -3431,7 +3431,7 @@
         <f t="shared" si="16"/>
         <v>5274326</v>
       </c>
-      <c r="F96" s="30"/>
+      <c r="F96" s="31"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
@@ -3454,7 +3454,7 @@
         <f t="shared" si="16"/>
         <v>5464682</v>
       </c>
-      <c r="F97" s="30"/>
+      <c r="F97" s="31"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
@@ -3477,7 +3477,7 @@
         <f t="shared" si="16"/>
         <v>5660748</v>
       </c>
-      <c r="F98" s="30"/>
+      <c r="F98" s="31"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
@@ -3500,7 +3500,7 @@
         <f t="shared" si="16"/>
         <v>5862695</v>
       </c>
-      <c r="F99" s="30"/>
+      <c r="F99" s="31"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
@@ -3523,7 +3523,7 @@
         <f t="shared" si="16"/>
         <v>6070700</v>
       </c>
-      <c r="F100" s="30"/>
+      <c r="F100" s="31"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
@@ -3546,7 +3546,29 @@
         <f t="shared" si="16"/>
         <v>6284945</v>
       </c>
-      <c r="F101" s="30"/>
+      <c r="F101" s="31"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <f t="shared" si="15"/>
+        <v>100</v>
+      </c>
+      <c r="B102" s="1">
+        <f t="shared" si="13"/>
+        <v>833</v>
+      </c>
+      <c r="C102" s="1">
+        <f t="shared" si="14"/>
+        <v>458</v>
+      </c>
+      <c r="D102" s="1">
+        <f t="shared" si="11"/>
+        <v>220672</v>
+      </c>
+      <c r="E102" s="1">
+        <f t="shared" si="16"/>
+        <v>6505617</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3585,24 +3607,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="27"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="28"/>
+      <c r="F3" s="29"/>
       <c r="G3" s="17" t="s">
         <v>8</v>
       </c>
@@ -3618,10 +3640,10 @@
       <c r="K3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="27" t="s">
+      <c r="M3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="28"/>
+      <c r="N3" s="29"/>
       <c r="O3" s="17" t="s">
         <v>8</v>
       </c>
@@ -3631,10 +3653,10 @@
       <c r="Q3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S3" s="27" t="s">
+      <c r="S3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="28"/>
+      <c r="T3" s="29"/>
       <c r="U3" s="17" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
v05_26.06 - Added Physical Element
</commit_message>
<xml_diff>
--- a/Lost Histories/stats.xlsx
+++ b/Lost Histories/stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Macko Games WIP\Lost Histories\Lost-Histories\Lost Histories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D552AF-58F7-46ED-8AA7-A5B96110258B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F5A6C9-5CB7-455F-98B7-81F709B7CAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1590" yWindow="1875" windowWidth="21585" windowHeight="13515" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6EE75E54-00C6-466F-BA17-D4DCF0C1D8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Levels" sheetId="1" r:id="rId1"/>
@@ -894,6 +894,15 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -902,15 +911,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1247,7 +1247,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C80B310D-5657-4E61-A0DA-301A4716D270}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A2:F102"/>
+  <dimension ref="A2:F101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="1"/>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="D3" s="26"/>
       <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="27" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="F4" s="30"/>
+      <c r="F4" s="27"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1317,11 +1317,11 @@
         <v>3</v>
       </c>
       <c r="B5" s="1">
-        <f t="shared" ref="B5:B68" si="0">(B4+7)</f>
+        <f t="shared" ref="B5:B21" si="0">(B4+7)</f>
         <v>154</v>
       </c>
       <c r="C5" s="1">
-        <f t="shared" ref="C5:C68" si="1">(C4+4)</f>
+        <f t="shared" ref="C5:C21" si="1">(C4+4)</f>
         <v>70</v>
       </c>
       <c r="D5" s="1">
@@ -1332,7 +1332,7 @@
         <f>D5+E4</f>
         <v>49</v>
       </c>
-      <c r="F5" s="30"/>
+      <c r="F5" s="27"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1355,7 +1355,7 @@
         <f>D6+E5</f>
         <v>88</v>
       </c>
-      <c r="F6" s="30"/>
+      <c r="F6" s="27"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1378,7 +1378,7 @@
         <f t="shared" ref="E7:E20" si="4">D7+E6</f>
         <v>140</v>
       </c>
-      <c r="F7" s="30"/>
+      <c r="F7" s="27"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1401,7 +1401,7 @@
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
-      <c r="F8" s="30"/>
+      <c r="F8" s="27"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -1424,7 +1424,7 @@
         <f t="shared" si="4"/>
         <v>304</v>
       </c>
-      <c r="F9" s="30"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -1447,7 +1447,7 @@
         <f t="shared" si="4"/>
         <v>430</v>
       </c>
-      <c r="F10" s="30"/>
+      <c r="F10" s="27"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -1470,7 +1470,7 @@
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="F11" s="30"/>
+      <c r="F11" s="27"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1493,7 +1493,7 @@
         <f t="shared" si="4"/>
         <v>829</v>
       </c>
-      <c r="F12" s="30"/>
+      <c r="F12" s="27"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -1516,7 +1516,7 @@
         <f t="shared" si="4"/>
         <v>1138</v>
       </c>
-      <c r="F13" s="30"/>
+      <c r="F13" s="27"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -1539,7 +1539,7 @@
         <f t="shared" si="4"/>
         <v>1555</v>
       </c>
-      <c r="F14" s="30"/>
+      <c r="F14" s="27"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1562,7 +1562,7 @@
         <f t="shared" si="4"/>
         <v>2117</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="27"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -1585,7 +1585,7 @@
         <f t="shared" si="4"/>
         <v>2875</v>
       </c>
-      <c r="F16" s="30"/>
+      <c r="F16" s="27"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
@@ -1608,7 +1608,7 @@
         <f t="shared" si="4"/>
         <v>3898</v>
       </c>
-      <c r="F17" s="30"/>
+      <c r="F17" s="27"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -1631,7 +1631,7 @@
         <f t="shared" si="4"/>
         <v>5279</v>
       </c>
-      <c r="F18" s="30"/>
+      <c r="F18" s="27"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
@@ -1654,7 +1654,7 @@
         <f t="shared" si="4"/>
         <v>7143</v>
       </c>
-      <c r="F19" s="30"/>
+      <c r="F19" s="27"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -1677,7 +1677,7 @@
         <f t="shared" si="4"/>
         <v>9659</v>
       </c>
-      <c r="F20" s="30"/>
+      <c r="F20" s="27"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1700,7 +1700,7 @@
         <f t="shared" ref="E21:E22" si="5">D21+E20</f>
         <v>13055</v>
       </c>
-      <c r="F21" s="30"/>
+      <c r="F21" s="27"/>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -1708,12 +1708,12 @@
         <v>20</v>
       </c>
       <c r="B22" s="1">
-        <f t="shared" si="0"/>
-        <v>273</v>
+        <f>(B21+8)</f>
+        <v>274</v>
       </c>
       <c r="C22" s="1">
-        <f t="shared" si="1"/>
-        <v>138</v>
+        <f>(C21+5)</f>
+        <v>139</v>
       </c>
       <c r="D22" s="1">
         <f t="shared" si="3"/>
@@ -1723,7 +1723,7 @@
         <f t="shared" si="5"/>
         <v>17639</v>
       </c>
-      <c r="F22" s="30"/>
+      <c r="F22" s="27"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -1731,22 +1731,22 @@
         <v>21</v>
       </c>
       <c r="B23" s="1">
-        <f t="shared" si="0"/>
-        <v>280</v>
+        <f t="shared" ref="B23:B51" si="7">(B22+8)</f>
+        <v>282</v>
       </c>
       <c r="C23" s="1">
-        <f t="shared" si="1"/>
-        <v>142</v>
+        <f t="shared" ref="C23:C51" si="8">(C22+5)</f>
+        <v>144</v>
       </c>
       <c r="D23" s="1">
         <f t="shared" si="3"/>
         <v>6188</v>
       </c>
       <c r="E23" s="1">
-        <f t="shared" ref="E23:E45" si="7">D23+E22</f>
+        <f t="shared" ref="E23:E45" si="9">D23+E22</f>
         <v>23827</v>
       </c>
-      <c r="F23" s="31" t="s">
+      <c r="F23" s="28" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1756,22 +1756,22 @@
         <v>22</v>
       </c>
       <c r="B24" s="1">
-        <f t="shared" si="0"/>
-        <v>287</v>
+        <f t="shared" si="7"/>
+        <v>290</v>
       </c>
       <c r="C24" s="1">
-        <f t="shared" si="1"/>
-        <v>146</v>
+        <f t="shared" si="8"/>
+        <v>149</v>
       </c>
       <c r="D24" s="1">
         <f>INT(D23*1.075)</f>
         <v>6652</v>
       </c>
       <c r="E24" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>30479</v>
       </c>
-      <c r="F24" s="31"/>
+      <c r="F24" s="28"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -1779,22 +1779,22 @@
         <v>23</v>
       </c>
       <c r="B25" s="1">
-        <f t="shared" si="0"/>
-        <v>294</v>
+        <f t="shared" si="7"/>
+        <v>298</v>
       </c>
       <c r="C25" s="1">
-        <f t="shared" si="1"/>
-        <v>150</v>
+        <f t="shared" si="8"/>
+        <v>154</v>
       </c>
       <c r="D25" s="1">
-        <f t="shared" ref="D25:D52" si="8">INT(D24*1.075)</f>
+        <f t="shared" ref="D25:D52" si="10">INT(D24*1.075)</f>
         <v>7150</v>
       </c>
       <c r="E25" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>37629</v>
       </c>
-      <c r="F25" s="31"/>
+      <c r="F25" s="28"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -1802,22 +1802,22 @@
         <v>24</v>
       </c>
       <c r="B26" s="1">
-        <f t="shared" si="0"/>
-        <v>301</v>
+        <f t="shared" si="7"/>
+        <v>306</v>
       </c>
       <c r="C26" s="1">
-        <f t="shared" si="1"/>
-        <v>154</v>
+        <f t="shared" si="8"/>
+        <v>159</v>
       </c>
       <c r="D26" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>7686</v>
       </c>
       <c r="E26" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>45315</v>
       </c>
-      <c r="F26" s="31"/>
+      <c r="F26" s="28"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -1825,22 +1825,22 @@
         <v>25</v>
       </c>
       <c r="B27" s="1">
-        <f t="shared" si="0"/>
-        <v>308</v>
+        <f t="shared" si="7"/>
+        <v>314</v>
       </c>
       <c r="C27" s="1">
-        <f t="shared" si="1"/>
-        <v>158</v>
+        <f t="shared" si="8"/>
+        <v>164</v>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>8262</v>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>53577</v>
       </c>
-      <c r="F27" s="31"/>
+      <c r="F27" s="28"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -1848,22 +1848,22 @@
         <v>26</v>
       </c>
       <c r="B28" s="1">
-        <f t="shared" si="0"/>
-        <v>315</v>
+        <f t="shared" si="7"/>
+        <v>322</v>
       </c>
       <c r="C28" s="1">
-        <f t="shared" si="1"/>
-        <v>162</v>
+        <f t="shared" si="8"/>
+        <v>169</v>
       </c>
       <c r="D28" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>8881</v>
       </c>
       <c r="E28" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>62458</v>
       </c>
-      <c r="F28" s="31"/>
+      <c r="F28" s="28"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -1871,22 +1871,22 @@
         <v>27</v>
       </c>
       <c r="B29" s="1">
-        <f t="shared" si="0"/>
-        <v>322</v>
+        <f t="shared" si="7"/>
+        <v>330</v>
       </c>
       <c r="C29" s="1">
-        <f t="shared" si="1"/>
-        <v>166</v>
+        <f t="shared" si="8"/>
+        <v>174</v>
       </c>
       <c r="D29" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>9547</v>
       </c>
       <c r="E29" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>72005</v>
       </c>
-      <c r="F29" s="31"/>
+      <c r="F29" s="28"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -1894,22 +1894,22 @@
         <v>28</v>
       </c>
       <c r="B30" s="1">
-        <f t="shared" si="0"/>
-        <v>329</v>
+        <f t="shared" si="7"/>
+        <v>338</v>
       </c>
       <c r="C30" s="1">
-        <f t="shared" si="1"/>
-        <v>170</v>
+        <f t="shared" si="8"/>
+        <v>179</v>
       </c>
       <c r="D30" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>10263</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>82268</v>
       </c>
-      <c r="F30" s="31"/>
+      <c r="F30" s="28"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -1917,22 +1917,22 @@
         <v>29</v>
       </c>
       <c r="B31" s="1">
-        <f t="shared" si="0"/>
-        <v>336</v>
+        <f t="shared" si="7"/>
+        <v>346</v>
       </c>
       <c r="C31" s="1">
-        <f t="shared" si="1"/>
-        <v>174</v>
+        <f t="shared" si="8"/>
+        <v>184</v>
       </c>
       <c r="D31" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11032</v>
       </c>
       <c r="E31" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>93300</v>
       </c>
-      <c r="F31" s="31"/>
+      <c r="F31" s="28"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -1940,22 +1940,22 @@
         <v>30</v>
       </c>
       <c r="B32" s="1">
-        <f t="shared" si="0"/>
-        <v>343</v>
+        <f t="shared" si="7"/>
+        <v>354</v>
       </c>
       <c r="C32" s="1">
-        <f t="shared" si="1"/>
-        <v>178</v>
+        <f t="shared" si="8"/>
+        <v>189</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>11859</v>
       </c>
       <c r="E32" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>105159</v>
       </c>
-      <c r="F32" s="31"/>
+      <c r="F32" s="28"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -1963,22 +1963,22 @@
         <v>31</v>
       </c>
       <c r="B33" s="1">
-        <f t="shared" si="0"/>
-        <v>350</v>
+        <f t="shared" si="7"/>
+        <v>362</v>
       </c>
       <c r="C33" s="1">
-        <f t="shared" si="1"/>
-        <v>182</v>
+        <f t="shared" si="8"/>
+        <v>194</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>12748</v>
       </c>
       <c r="E33" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>117907</v>
       </c>
-      <c r="F33" s="31"/>
+      <c r="F33" s="28"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -1986,22 +1986,22 @@
         <v>32</v>
       </c>
       <c r="B34" s="1">
-        <f t="shared" si="0"/>
-        <v>357</v>
+        <f t="shared" si="7"/>
+        <v>370</v>
       </c>
       <c r="C34" s="1">
-        <f t="shared" si="1"/>
-        <v>186</v>
+        <f t="shared" si="8"/>
+        <v>199</v>
       </c>
       <c r="D34" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>13704</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>131611</v>
       </c>
-      <c r="F34" s="31"/>
+      <c r="F34" s="28"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -2009,22 +2009,22 @@
         <v>33</v>
       </c>
       <c r="B35" s="1">
-        <f t="shared" si="0"/>
-        <v>364</v>
+        <f t="shared" si="7"/>
+        <v>378</v>
       </c>
       <c r="C35" s="1">
-        <f t="shared" si="1"/>
-        <v>190</v>
+        <f t="shared" si="8"/>
+        <v>204</v>
       </c>
       <c r="D35" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>14731</v>
       </c>
       <c r="E35" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>146342</v>
       </c>
-      <c r="F35" s="31"/>
+      <c r="F35" s="28"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -2032,22 +2032,22 @@
         <v>34</v>
       </c>
       <c r="B36" s="1">
-        <f t="shared" si="0"/>
-        <v>371</v>
+        <f t="shared" si="7"/>
+        <v>386</v>
       </c>
       <c r="C36" s="1">
-        <f t="shared" si="1"/>
-        <v>194</v>
+        <f t="shared" si="8"/>
+        <v>209</v>
       </c>
       <c r="D36" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>15835</v>
       </c>
       <c r="E36" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>162177</v>
       </c>
-      <c r="F36" s="31"/>
+      <c r="F36" s="28"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -2055,22 +2055,22 @@
         <v>35</v>
       </c>
       <c r="B37" s="1">
-        <f t="shared" si="0"/>
-        <v>378</v>
+        <f t="shared" si="7"/>
+        <v>394</v>
       </c>
       <c r="C37" s="1">
-        <f t="shared" si="1"/>
-        <v>198</v>
+        <f t="shared" si="8"/>
+        <v>214</v>
       </c>
       <c r="D37" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>17022</v>
       </c>
       <c r="E37" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>179199</v>
       </c>
-      <c r="F37" s="31"/>
+      <c r="F37" s="28"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -2078,22 +2078,22 @@
         <v>36</v>
       </c>
       <c r="B38" s="1">
-        <f t="shared" si="0"/>
-        <v>385</v>
+        <f t="shared" si="7"/>
+        <v>402</v>
       </c>
       <c r="C38" s="1">
-        <f t="shared" si="1"/>
-        <v>202</v>
+        <f t="shared" si="8"/>
+        <v>219</v>
       </c>
       <c r="D38" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>18298</v>
       </c>
       <c r="E38" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>197497</v>
       </c>
-      <c r="F38" s="31"/>
+      <c r="F38" s="28"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
@@ -2101,22 +2101,22 @@
         <v>37</v>
       </c>
       <c r="B39" s="1">
-        <f t="shared" si="0"/>
-        <v>392</v>
+        <f t="shared" si="7"/>
+        <v>410</v>
       </c>
       <c r="C39" s="1">
-        <f t="shared" si="1"/>
-        <v>206</v>
+        <f t="shared" si="8"/>
+        <v>224</v>
       </c>
       <c r="D39" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>19670</v>
       </c>
       <c r="E39" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>217167</v>
       </c>
-      <c r="F39" s="31"/>
+      <c r="F39" s="28"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
@@ -2124,22 +2124,22 @@
         <v>38</v>
       </c>
       <c r="B40" s="1">
-        <f t="shared" si="0"/>
-        <v>399</v>
+        <f t="shared" si="7"/>
+        <v>418</v>
       </c>
       <c r="C40" s="1">
-        <f t="shared" si="1"/>
-        <v>210</v>
+        <f t="shared" si="8"/>
+        <v>229</v>
       </c>
       <c r="D40" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>21145</v>
       </c>
       <c r="E40" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>238312</v>
       </c>
-      <c r="F40" s="31"/>
+      <c r="F40" s="28"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
@@ -2147,22 +2147,22 @@
         <v>39</v>
       </c>
       <c r="B41" s="1">
-        <f t="shared" si="0"/>
-        <v>406</v>
+        <f t="shared" si="7"/>
+        <v>426</v>
       </c>
       <c r="C41" s="1">
-        <f t="shared" si="1"/>
-        <v>214</v>
+        <f t="shared" si="8"/>
+        <v>234</v>
       </c>
       <c r="D41" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>22730</v>
       </c>
       <c r="E41" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>261042</v>
       </c>
-      <c r="F41" s="31"/>
+      <c r="F41" s="28"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
@@ -2170,22 +2170,22 @@
         <v>40</v>
       </c>
       <c r="B42" s="1">
-        <f t="shared" si="0"/>
-        <v>413</v>
+        <f t="shared" si="7"/>
+        <v>434</v>
       </c>
       <c r="C42" s="1">
-        <f t="shared" si="1"/>
-        <v>218</v>
+        <f>(C41+5)</f>
+        <v>239</v>
       </c>
       <c r="D42" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>24434</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>285476</v>
       </c>
-      <c r="F42" s="31"/>
+      <c r="F42" s="28"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
@@ -2193,22 +2193,22 @@
         <v>41</v>
       </c>
       <c r="B43" s="1">
-        <f t="shared" si="0"/>
-        <v>420</v>
+        <f t="shared" si="7"/>
+        <v>442</v>
       </c>
       <c r="C43" s="1">
-        <f t="shared" si="1"/>
-        <v>222</v>
+        <f t="shared" si="8"/>
+        <v>244</v>
       </c>
       <c r="D43" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>26266</v>
       </c>
       <c r="E43" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>311742</v>
       </c>
-      <c r="F43" s="31"/>
+      <c r="F43" s="28"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
@@ -2216,438 +2216,438 @@
         <v>42</v>
       </c>
       <c r="B44" s="1">
-        <f t="shared" si="0"/>
-        <v>427</v>
+        <f t="shared" si="7"/>
+        <v>450</v>
       </c>
       <c r="C44" s="1">
-        <f t="shared" si="1"/>
-        <v>226</v>
+        <f t="shared" si="8"/>
+        <v>249</v>
       </c>
       <c r="D44" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>28235</v>
       </c>
       <c r="E44" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>339977</v>
       </c>
-      <c r="F44" s="31"/>
+      <c r="F44" s="28"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <f t="shared" ref="A45:A62" si="9">A44+1</f>
+        <f t="shared" ref="A45:A62" si="11">A44+1</f>
         <v>43</v>
       </c>
       <c r="B45" s="1">
-        <f t="shared" si="0"/>
-        <v>434</v>
+        <f t="shared" si="7"/>
+        <v>458</v>
       </c>
       <c r="C45" s="1">
-        <f t="shared" si="1"/>
-        <v>230</v>
+        <f t="shared" si="8"/>
+        <v>254</v>
       </c>
       <c r="D45" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>30352</v>
       </c>
       <c r="E45" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>370329</v>
       </c>
-      <c r="F45" s="31"/>
+      <c r="F45" s="28"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>44</v>
       </c>
       <c r="B46" s="1">
-        <f t="shared" si="0"/>
-        <v>441</v>
+        <f t="shared" si="7"/>
+        <v>466</v>
       </c>
       <c r="C46" s="1">
-        <f t="shared" si="1"/>
-        <v>234</v>
+        <f t="shared" si="8"/>
+        <v>259</v>
       </c>
       <c r="D46" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>32628</v>
       </c>
       <c r="E46" s="1">
-        <f t="shared" ref="E46:E88" si="10">D46+E45</f>
+        <f t="shared" ref="E46:E88" si="12">D46+E45</f>
         <v>402957</v>
       </c>
-      <c r="F46" s="32" t="s">
+      <c r="F46" s="29" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>45</v>
       </c>
       <c r="B47" s="1">
-        <f t="shared" si="0"/>
-        <v>448</v>
+        <f t="shared" si="7"/>
+        <v>474</v>
       </c>
       <c r="C47" s="1">
-        <f t="shared" si="1"/>
-        <v>238</v>
+        <f t="shared" si="8"/>
+        <v>264</v>
       </c>
       <c r="D47" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>35075</v>
       </c>
       <c r="E47" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>438032</v>
       </c>
-      <c r="F47" s="32"/>
+      <c r="F47" s="29"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>46</v>
       </c>
       <c r="B48" s="1">
-        <f t="shared" si="0"/>
-        <v>455</v>
+        <f t="shared" si="7"/>
+        <v>482</v>
       </c>
       <c r="C48" s="1">
-        <f t="shared" si="1"/>
-        <v>242</v>
+        <f t="shared" si="8"/>
+        <v>269</v>
       </c>
       <c r="D48" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>37705</v>
       </c>
       <c r="E48" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>475737</v>
       </c>
-      <c r="F48" s="32"/>
+      <c r="F48" s="29"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>47</v>
       </c>
       <c r="B49" s="1">
-        <f t="shared" si="0"/>
-        <v>462</v>
+        <f t="shared" si="7"/>
+        <v>490</v>
       </c>
       <c r="C49" s="1">
-        <f t="shared" si="1"/>
-        <v>246</v>
+        <f t="shared" si="8"/>
+        <v>274</v>
       </c>
       <c r="D49" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>40532</v>
       </c>
       <c r="E49" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>516269</v>
       </c>
-      <c r="F49" s="32"/>
+      <c r="F49" s="29"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>48</v>
       </c>
       <c r="B50" s="1">
-        <f t="shared" si="0"/>
-        <v>469</v>
+        <f t="shared" si="7"/>
+        <v>498</v>
       </c>
       <c r="C50" s="1">
-        <f t="shared" si="1"/>
-        <v>250</v>
+        <f t="shared" si="8"/>
+        <v>279</v>
       </c>
       <c r="D50" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>43571</v>
       </c>
       <c r="E50" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>559840</v>
       </c>
-      <c r="F50" s="32"/>
+      <c r="F50" s="29"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>49</v>
       </c>
       <c r="B51" s="1">
-        <f t="shared" si="0"/>
-        <v>476</v>
+        <f t="shared" si="7"/>
+        <v>506</v>
       </c>
       <c r="C51" s="1">
-        <f t="shared" si="1"/>
-        <v>254</v>
+        <f t="shared" si="8"/>
+        <v>284</v>
       </c>
       <c r="D51" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>46838</v>
       </c>
       <c r="E51" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>606678</v>
       </c>
-      <c r="F51" s="32"/>
+      <c r="F51" s="29"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>50</v>
       </c>
       <c r="B52" s="1">
-        <f t="shared" si="0"/>
-        <v>483</v>
+        <f>(B51+11)</f>
+        <v>517</v>
       </c>
       <c r="C52" s="1">
-        <f t="shared" si="1"/>
-        <v>258</v>
+        <f>(C51+7)</f>
+        <v>291</v>
       </c>
       <c r="D52" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>50350</v>
       </c>
       <c r="E52" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>657028</v>
       </c>
-      <c r="F52" s="32"/>
+      <c r="F52" s="29"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>51</v>
       </c>
       <c r="B53" s="1">
-        <f t="shared" si="0"/>
-        <v>490</v>
+        <f t="shared" ref="B53:B101" si="13">(B52+11)</f>
+        <v>528</v>
       </c>
       <c r="C53" s="1">
-        <f t="shared" si="1"/>
-        <v>262</v>
+        <f t="shared" ref="C53:C101" si="14">(C52+7)</f>
+        <v>298</v>
       </c>
       <c r="D53" s="1">
         <f>INT(D52*1.03)</f>
         <v>51860</v>
       </c>
       <c r="E53" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>708888</v>
       </c>
-      <c r="F53" s="32"/>
+      <c r="F53" s="29"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>52</v>
       </c>
       <c r="B54" s="1">
-        <f t="shared" si="0"/>
-        <v>497</v>
+        <f t="shared" si="13"/>
+        <v>539</v>
       </c>
       <c r="C54" s="1">
-        <f t="shared" si="1"/>
-        <v>266</v>
+        <f t="shared" si="14"/>
+        <v>305</v>
       </c>
       <c r="D54" s="1">
-        <f t="shared" ref="D54:D102" si="11">INT(D53*1.03)</f>
+        <f t="shared" ref="D54:D101" si="15">INT(D53*1.03)</f>
         <v>53415</v>
       </c>
       <c r="E54" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>762303</v>
       </c>
-      <c r="F54" s="32"/>
+      <c r="F54" s="29"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>53</v>
       </c>
       <c r="B55" s="1">
-        <f t="shared" si="0"/>
-        <v>504</v>
+        <f t="shared" si="13"/>
+        <v>550</v>
       </c>
       <c r="C55" s="1">
-        <f t="shared" si="1"/>
-        <v>270</v>
+        <f t="shared" si="14"/>
+        <v>312</v>
       </c>
       <c r="D55" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>55017</v>
       </c>
       <c r="E55" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>817320</v>
       </c>
-      <c r="F55" s="32"/>
+      <c r="F55" s="29"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>54</v>
       </c>
       <c r="B56" s="1">
-        <f t="shared" si="0"/>
-        <v>511</v>
+        <f t="shared" si="13"/>
+        <v>561</v>
       </c>
       <c r="C56" s="1">
-        <f t="shared" si="1"/>
-        <v>274</v>
+        <f t="shared" si="14"/>
+        <v>319</v>
       </c>
       <c r="D56" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>56667</v>
       </c>
       <c r="E56" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>873987</v>
       </c>
-      <c r="F56" s="32"/>
+      <c r="F56" s="29"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>55</v>
       </c>
       <c r="B57" s="1">
-        <f t="shared" si="0"/>
-        <v>518</v>
+        <f t="shared" si="13"/>
+        <v>572</v>
       </c>
       <c r="C57" s="1">
-        <f t="shared" si="1"/>
-        <v>278</v>
+        <f t="shared" si="14"/>
+        <v>326</v>
       </c>
       <c r="D57" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>58367</v>
       </c>
       <c r="E57" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>932354</v>
       </c>
-      <c r="F57" s="32"/>
+      <c r="F57" s="29"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>56</v>
       </c>
       <c r="B58" s="1">
-        <f t="shared" si="0"/>
-        <v>525</v>
+        <f t="shared" si="13"/>
+        <v>583</v>
       </c>
       <c r="C58" s="1">
-        <f t="shared" si="1"/>
-        <v>282</v>
+        <f t="shared" si="14"/>
+        <v>333</v>
       </c>
       <c r="D58" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>60118</v>
       </c>
       <c r="E58" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>992472</v>
       </c>
-      <c r="F58" s="32"/>
+      <c r="F58" s="29"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>57</v>
       </c>
       <c r="B59" s="1">
-        <f t="shared" si="0"/>
-        <v>532</v>
+        <f t="shared" si="13"/>
+        <v>594</v>
       </c>
       <c r="C59" s="1">
-        <f t="shared" si="1"/>
-        <v>286</v>
+        <f t="shared" si="14"/>
+        <v>340</v>
       </c>
       <c r="D59" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>61921</v>
       </c>
       <c r="E59" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1054393</v>
       </c>
-      <c r="F59" s="32"/>
+      <c r="F59" s="29"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>58</v>
       </c>
       <c r="B60" s="1">
-        <f t="shared" si="0"/>
-        <v>539</v>
+        <f t="shared" si="13"/>
+        <v>605</v>
       </c>
       <c r="C60" s="1">
-        <f t="shared" si="1"/>
-        <v>290</v>
+        <f t="shared" si="14"/>
+        <v>347</v>
       </c>
       <c r="D60" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>63778</v>
       </c>
       <c r="E60" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1118171</v>
       </c>
-      <c r="F60" s="32"/>
+      <c r="F60" s="29"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>59</v>
       </c>
       <c r="B61" s="1">
-        <f t="shared" si="0"/>
-        <v>546</v>
+        <f t="shared" si="13"/>
+        <v>616</v>
       </c>
       <c r="C61" s="1">
-        <f t="shared" si="1"/>
-        <v>294</v>
+        <f t="shared" si="14"/>
+        <v>354</v>
       </c>
       <c r="D61" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>65691</v>
       </c>
       <c r="E61" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1183862</v>
       </c>
-      <c r="F61" s="32"/>
+      <c r="F61" s="29"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>60</v>
       </c>
       <c r="B62" s="1">
-        <f t="shared" si="0"/>
-        <v>553</v>
+        <f t="shared" si="13"/>
+        <v>627</v>
       </c>
       <c r="C62" s="1">
-        <f t="shared" si="1"/>
-        <v>298</v>
+        <f t="shared" si="14"/>
+        <v>361</v>
       </c>
       <c r="D62" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>67661</v>
       </c>
       <c r="E62" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1251523</v>
       </c>
-      <c r="F62" s="32"/>
+      <c r="F62" s="29"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
@@ -2655,22 +2655,22 @@
         <v>61</v>
       </c>
       <c r="B63" s="1">
-        <f t="shared" si="0"/>
-        <v>560</v>
+        <f t="shared" si="13"/>
+        <v>638</v>
       </c>
       <c r="C63" s="1">
-        <f t="shared" si="1"/>
-        <v>302</v>
+        <f t="shared" si="14"/>
+        <v>368</v>
       </c>
       <c r="D63" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>69690</v>
       </c>
       <c r="E63" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1321213</v>
       </c>
-      <c r="F63" s="31" t="s">
+      <c r="F63" s="28" t="s">
         <v>204</v>
       </c>
     </row>
@@ -2680,505 +2680,505 @@
         <v>62</v>
       </c>
       <c r="B64" s="1">
-        <f t="shared" si="0"/>
-        <v>567</v>
+        <f t="shared" si="13"/>
+        <v>649</v>
       </c>
       <c r="C64" s="1">
-        <f t="shared" si="1"/>
-        <v>306</v>
+        <f t="shared" si="14"/>
+        <v>375</v>
       </c>
       <c r="D64" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>71780</v>
       </c>
       <c r="E64" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1392993</v>
       </c>
-      <c r="F64" s="31"/>
+      <c r="F64" s="28"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <f t="shared" ref="A65:A85" si="12">A64+1</f>
+        <f t="shared" ref="A65:A85" si="16">A64+1</f>
         <v>63</v>
       </c>
       <c r="B65" s="1">
-        <f t="shared" si="0"/>
-        <v>574</v>
+        <f t="shared" si="13"/>
+        <v>660</v>
       </c>
       <c r="C65" s="1">
-        <f t="shared" si="1"/>
-        <v>310</v>
+        <f t="shared" si="14"/>
+        <v>382</v>
       </c>
       <c r="D65" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>73933</v>
       </c>
       <c r="E65" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1466926</v>
       </c>
-      <c r="F65" s="31"/>
+      <c r="F65" s="28"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
+        <f t="shared" si="16"/>
+        <v>64</v>
+      </c>
+      <c r="B66" s="1">
+        <f t="shared" si="13"/>
+        <v>671</v>
+      </c>
+      <c r="C66" s="1">
+        <f t="shared" si="14"/>
+        <v>389</v>
+      </c>
+      <c r="D66" s="1">
+        <f t="shared" si="15"/>
+        <v>76150</v>
+      </c>
+      <c r="E66" s="1">
         <f t="shared" si="12"/>
-        <v>64</v>
-      </c>
-      <c r="B66" s="1">
-        <f t="shared" si="0"/>
-        <v>581</v>
-      </c>
-      <c r="C66" s="1">
-        <f t="shared" si="1"/>
-        <v>314</v>
-      </c>
-      <c r="D66" s="1">
-        <f t="shared" si="11"/>
-        <v>76150</v>
-      </c>
-      <c r="E66" s="1">
-        <f t="shared" si="10"/>
         <v>1543076</v>
       </c>
-      <c r="F66" s="31"/>
+      <c r="F66" s="28"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
+        <f t="shared" si="16"/>
+        <v>65</v>
+      </c>
+      <c r="B67" s="1">
+        <f t="shared" si="13"/>
+        <v>682</v>
+      </c>
+      <c r="C67" s="1">
+        <f t="shared" si="14"/>
+        <v>396</v>
+      </c>
+      <c r="D67" s="1">
+        <f t="shared" si="15"/>
+        <v>78434</v>
+      </c>
+      <c r="E67" s="1">
         <f t="shared" si="12"/>
-        <v>65</v>
-      </c>
-      <c r="B67" s="1">
-        <f t="shared" si="0"/>
-        <v>588</v>
-      </c>
-      <c r="C67" s="1">
-        <f t="shared" si="1"/>
-        <v>318</v>
-      </c>
-      <c r="D67" s="1">
-        <f t="shared" si="11"/>
-        <v>78434</v>
-      </c>
-      <c r="E67" s="1">
-        <f t="shared" si="10"/>
         <v>1621510</v>
       </c>
-      <c r="F67" s="31"/>
+      <c r="F67" s="28"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
+        <f t="shared" si="16"/>
+        <v>66</v>
+      </c>
+      <c r="B68" s="1">
+        <f t="shared" si="13"/>
+        <v>693</v>
+      </c>
+      <c r="C68" s="1">
+        <f t="shared" si="14"/>
+        <v>403</v>
+      </c>
+      <c r="D68" s="1">
+        <f t="shared" si="15"/>
+        <v>80787</v>
+      </c>
+      <c r="E68" s="1">
         <f t="shared" si="12"/>
-        <v>66</v>
-      </c>
-      <c r="B68" s="1">
-        <f t="shared" si="0"/>
-        <v>595</v>
-      </c>
-      <c r="C68" s="1">
-        <f t="shared" si="1"/>
-        <v>322</v>
-      </c>
-      <c r="D68" s="1">
-        <f t="shared" si="11"/>
-        <v>80787</v>
-      </c>
-      <c r="E68" s="1">
-        <f t="shared" si="10"/>
         <v>1702297</v>
       </c>
-      <c r="F68" s="31"/>
+      <c r="F68" s="28"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
+        <f t="shared" si="16"/>
+        <v>67</v>
+      </c>
+      <c r="B69" s="1">
+        <f t="shared" si="13"/>
+        <v>704</v>
+      </c>
+      <c r="C69" s="1">
+        <f t="shared" si="14"/>
+        <v>410</v>
+      </c>
+      <c r="D69" s="1">
+        <f t="shared" si="15"/>
+        <v>83210</v>
+      </c>
+      <c r="E69" s="1">
         <f t="shared" si="12"/>
-        <v>67</v>
-      </c>
-      <c r="B69" s="1">
-        <f t="shared" ref="B69:B102" si="13">(B68+7)</f>
-        <v>602</v>
-      </c>
-      <c r="C69" s="1">
-        <f t="shared" ref="C69:C102" si="14">(C68+4)</f>
-        <v>326</v>
-      </c>
-      <c r="D69" s="1">
-        <f t="shared" si="11"/>
-        <v>83210</v>
-      </c>
-      <c r="E69" s="1">
-        <f t="shared" si="10"/>
         <v>1785507</v>
       </c>
-      <c r="F69" s="31"/>
+      <c r="F69" s="28"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>68</v>
       </c>
       <c r="B70" s="1">
         <f t="shared" si="13"/>
-        <v>609</v>
+        <v>715</v>
       </c>
       <c r="C70" s="1">
         <f t="shared" si="14"/>
-        <v>330</v>
+        <v>417</v>
       </c>
       <c r="D70" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>85706</v>
       </c>
       <c r="E70" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1871213</v>
       </c>
-      <c r="F70" s="31"/>
+      <c r="F70" s="28"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>69</v>
       </c>
       <c r="B71" s="1">
         <f t="shared" si="13"/>
-        <v>616</v>
+        <v>726</v>
       </c>
       <c r="C71" s="1">
         <f t="shared" si="14"/>
-        <v>334</v>
+        <v>424</v>
       </c>
       <c r="D71" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>88277</v>
       </c>
       <c r="E71" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>1959490</v>
       </c>
-      <c r="F71" s="31"/>
+      <c r="F71" s="28"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>70</v>
       </c>
       <c r="B72" s="1">
         <f t="shared" si="13"/>
-        <v>623</v>
+        <v>737</v>
       </c>
       <c r="C72" s="1">
         <f t="shared" si="14"/>
-        <v>338</v>
+        <v>431</v>
       </c>
       <c r="D72" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>90925</v>
       </c>
       <c r="E72" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2050415</v>
       </c>
-      <c r="F72" s="31"/>
+      <c r="F72" s="28"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>71</v>
       </c>
       <c r="B73" s="1">
         <f t="shared" si="13"/>
-        <v>630</v>
+        <v>748</v>
       </c>
       <c r="C73" s="1">
         <f t="shared" si="14"/>
-        <v>342</v>
+        <v>438</v>
       </c>
       <c r="D73" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>93652</v>
       </c>
       <c r="E73" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2144067</v>
       </c>
-      <c r="F73" s="31"/>
+      <c r="F73" s="28"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>72</v>
       </c>
       <c r="B74" s="1">
         <f t="shared" si="13"/>
-        <v>637</v>
+        <v>759</v>
       </c>
       <c r="C74" s="1">
         <f t="shared" si="14"/>
-        <v>346</v>
+        <v>445</v>
       </c>
       <c r="D74" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>96461</v>
       </c>
       <c r="E74" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2240528</v>
       </c>
-      <c r="F74" s="31"/>
+      <c r="F74" s="28"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>73</v>
       </c>
       <c r="B75" s="1">
         <f t="shared" si="13"/>
-        <v>644</v>
+        <v>770</v>
       </c>
       <c r="C75" s="1">
         <f t="shared" si="14"/>
-        <v>350</v>
+        <v>452</v>
       </c>
       <c r="D75" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>99354</v>
       </c>
       <c r="E75" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2339882</v>
       </c>
-      <c r="F75" s="31"/>
+      <c r="F75" s="28"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>74</v>
       </c>
       <c r="B76" s="1">
         <f t="shared" si="13"/>
-        <v>651</v>
+        <v>781</v>
       </c>
       <c r="C76" s="1">
         <f t="shared" si="14"/>
-        <v>354</v>
+        <v>459</v>
       </c>
       <c r="D76" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>102334</v>
       </c>
       <c r="E76" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2442216</v>
       </c>
-      <c r="F76" s="31"/>
+      <c r="F76" s="28"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>75</v>
       </c>
       <c r="B77" s="1">
         <f t="shared" si="13"/>
-        <v>658</v>
+        <v>792</v>
       </c>
       <c r="C77" s="1">
         <f t="shared" si="14"/>
-        <v>358</v>
+        <v>466</v>
       </c>
       <c r="D77" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>105404</v>
       </c>
       <c r="E77" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2547620</v>
       </c>
-      <c r="F77" s="31"/>
+      <c r="F77" s="28"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>76</v>
       </c>
       <c r="B78" s="1">
         <f t="shared" si="13"/>
-        <v>665</v>
+        <v>803</v>
       </c>
       <c r="C78" s="1">
         <f t="shared" si="14"/>
-        <v>362</v>
+        <v>473</v>
       </c>
       <c r="D78" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>108566</v>
       </c>
       <c r="E78" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2656186</v>
       </c>
-      <c r="F78" s="31"/>
+      <c r="F78" s="28"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>77</v>
       </c>
       <c r="B79" s="1">
         <f t="shared" si="13"/>
-        <v>672</v>
+        <v>814</v>
       </c>
       <c r="C79" s="1">
         <f t="shared" si="14"/>
-        <v>366</v>
+        <v>480</v>
       </c>
       <c r="D79" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>111822</v>
       </c>
       <c r="E79" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2768008</v>
       </c>
-      <c r="F79" s="31"/>
+      <c r="F79" s="28"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>78</v>
       </c>
       <c r="B80" s="1">
         <f t="shared" si="13"/>
-        <v>679</v>
+        <v>825</v>
       </c>
       <c r="C80" s="1">
         <f t="shared" si="14"/>
-        <v>370</v>
+        <v>487</v>
       </c>
       <c r="D80" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>115176</v>
       </c>
       <c r="E80" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>2883184</v>
       </c>
-      <c r="F80" s="31"/>
+      <c r="F80" s="28"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>79</v>
       </c>
       <c r="B81" s="1">
         <f t="shared" si="13"/>
-        <v>686</v>
+        <v>836</v>
       </c>
       <c r="C81" s="1">
         <f t="shared" si="14"/>
-        <v>374</v>
+        <v>494</v>
       </c>
       <c r="D81" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>118631</v>
       </c>
       <c r="E81" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3001815</v>
       </c>
-      <c r="F81" s="31"/>
+      <c r="F81" s="28"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>80</v>
       </c>
       <c r="B82" s="1">
         <f t="shared" si="13"/>
-        <v>693</v>
+        <v>847</v>
       </c>
       <c r="C82" s="1">
         <f t="shared" si="14"/>
-        <v>378</v>
+        <v>501</v>
       </c>
       <c r="D82" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>122189</v>
       </c>
       <c r="E82" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3124004</v>
       </c>
-      <c r="F82" s="31"/>
+      <c r="F82" s="28"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>81</v>
       </c>
       <c r="B83" s="1">
         <f t="shared" si="13"/>
-        <v>700</v>
+        <v>858</v>
       </c>
       <c r="C83" s="1">
         <f t="shared" si="14"/>
-        <v>382</v>
+        <v>508</v>
       </c>
       <c r="D83" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>125854</v>
       </c>
       <c r="E83" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3249858</v>
       </c>
-      <c r="F83" s="31"/>
+      <c r="F83" s="28"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>82</v>
       </c>
       <c r="B84" s="1">
         <f t="shared" si="13"/>
-        <v>707</v>
+        <v>869</v>
       </c>
       <c r="C84" s="1">
         <f t="shared" si="14"/>
-        <v>386</v>
+        <v>515</v>
       </c>
       <c r="D84" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>129629</v>
       </c>
       <c r="E84" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3379487</v>
       </c>
-      <c r="F84" s="31"/>
+      <c r="F84" s="28"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="16"/>
         <v>83</v>
       </c>
       <c r="B85" s="1">
         <f t="shared" si="13"/>
-        <v>714</v>
+        <v>880</v>
       </c>
       <c r="C85" s="1">
         <f t="shared" si="14"/>
-        <v>390</v>
+        <v>522</v>
       </c>
       <c r="D85" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>133517</v>
       </c>
       <c r="E85" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3513004</v>
       </c>
-      <c r="F85" s="31"/>
+      <c r="F85" s="28"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
@@ -3187,21 +3187,21 @@
       </c>
       <c r="B86" s="1">
         <f t="shared" si="13"/>
-        <v>721</v>
+        <v>891</v>
       </c>
       <c r="C86" s="1">
         <f t="shared" si="14"/>
-        <v>394</v>
+        <v>529</v>
       </c>
       <c r="D86" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>137522</v>
       </c>
       <c r="E86" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3650526</v>
       </c>
-      <c r="F86" s="31"/>
+      <c r="F86" s="28"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
@@ -3210,365 +3210,343 @@
       </c>
       <c r="B87" s="1">
         <f t="shared" si="13"/>
-        <v>728</v>
+        <v>902</v>
       </c>
       <c r="C87" s="1">
         <f t="shared" si="14"/>
-        <v>398</v>
+        <v>536</v>
       </c>
       <c r="D87" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>141647</v>
       </c>
       <c r="E87" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3792173</v>
       </c>
-      <c r="F87" s="31"/>
+      <c r="F87" s="28"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <f t="shared" ref="A88:A102" si="15">A87+1</f>
+        <f t="shared" ref="A88:A101" si="17">A87+1</f>
         <v>86</v>
       </c>
       <c r="B88" s="1">
         <f t="shared" si="13"/>
-        <v>735</v>
+        <v>913</v>
       </c>
       <c r="C88" s="1">
         <f t="shared" si="14"/>
-        <v>402</v>
+        <v>543</v>
       </c>
       <c r="D88" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>145896</v>
       </c>
       <c r="E88" s="1">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>3938069</v>
       </c>
-      <c r="F88" s="31"/>
+      <c r="F88" s="28"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>87</v>
       </c>
       <c r="B89" s="1">
         <f t="shared" si="13"/>
-        <v>742</v>
+        <v>924</v>
       </c>
       <c r="C89" s="1">
         <f t="shared" si="14"/>
-        <v>406</v>
+        <v>550</v>
       </c>
       <c r="D89" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>150272</v>
       </c>
       <c r="E89" s="1">
-        <f t="shared" ref="E89:E102" si="16">D89+E88</f>
+        <f t="shared" ref="E89:E101" si="18">D89+E88</f>
         <v>4088341</v>
       </c>
-      <c r="F89" s="31"/>
+      <c r="F89" s="28"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>88</v>
       </c>
       <c r="B90" s="1">
         <f t="shared" si="13"/>
-        <v>749</v>
+        <v>935</v>
       </c>
       <c r="C90" s="1">
         <f t="shared" si="14"/>
-        <v>410</v>
+        <v>557</v>
       </c>
       <c r="D90" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>154780</v>
       </c>
       <c r="E90" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4243121</v>
       </c>
-      <c r="F90" s="31"/>
+      <c r="F90" s="28"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>89</v>
       </c>
       <c r="B91" s="1">
         <f t="shared" si="13"/>
-        <v>756</v>
+        <v>946</v>
       </c>
       <c r="C91" s="1">
         <f t="shared" si="14"/>
-        <v>414</v>
+        <v>564</v>
       </c>
       <c r="D91" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>159423</v>
       </c>
       <c r="E91" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4402544</v>
       </c>
-      <c r="F91" s="31"/>
+      <c r="F91" s="28"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>90</v>
       </c>
       <c r="B92" s="1">
         <f t="shared" si="13"/>
-        <v>763</v>
+        <v>957</v>
       </c>
       <c r="C92" s="1">
         <f t="shared" si="14"/>
-        <v>418</v>
+        <v>571</v>
       </c>
       <c r="D92" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>164205</v>
       </c>
       <c r="E92" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4566749</v>
       </c>
-      <c r="F92" s="31"/>
+      <c r="F92" s="28"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>91</v>
       </c>
       <c r="B93" s="1">
         <f t="shared" si="13"/>
-        <v>770</v>
+        <v>968</v>
       </c>
       <c r="C93" s="1">
         <f t="shared" si="14"/>
-        <v>422</v>
+        <v>578</v>
       </c>
       <c r="D93" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>169131</v>
       </c>
       <c r="E93" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4735880</v>
       </c>
-      <c r="F93" s="31"/>
+      <c r="F93" s="28"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>92</v>
       </c>
       <c r="B94" s="1">
         <f t="shared" si="13"/>
-        <v>777</v>
+        <v>979</v>
       </c>
       <c r="C94" s="1">
         <f t="shared" si="14"/>
-        <v>426</v>
+        <v>585</v>
       </c>
       <c r="D94" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>174204</v>
       </c>
       <c r="E94" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4910084</v>
       </c>
-      <c r="F94" s="31"/>
+      <c r="F94" s="28"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>93</v>
       </c>
       <c r="B95" s="1">
         <f t="shared" si="13"/>
-        <v>784</v>
+        <v>990</v>
       </c>
       <c r="C95" s="1">
         <f t="shared" si="14"/>
-        <v>430</v>
+        <v>592</v>
       </c>
       <c r="D95" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>179430</v>
       </c>
       <c r="E95" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>5089514</v>
       </c>
-      <c r="F95" s="31"/>
+      <c r="F95" s="28"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>94</v>
       </c>
       <c r="B96" s="1">
         <f t="shared" si="13"/>
-        <v>791</v>
+        <v>1001</v>
       </c>
       <c r="C96" s="1">
         <f t="shared" si="14"/>
-        <v>434</v>
+        <v>599</v>
       </c>
       <c r="D96" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>184812</v>
       </c>
       <c r="E96" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>5274326</v>
       </c>
-      <c r="F96" s="31"/>
+      <c r="F96" s="28"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>95</v>
       </c>
       <c r="B97" s="1">
         <f t="shared" si="13"/>
-        <v>798</v>
+        <v>1012</v>
       </c>
       <c r="C97" s="1">
         <f t="shared" si="14"/>
-        <v>438</v>
+        <v>606</v>
       </c>
       <c r="D97" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>190356</v>
       </c>
       <c r="E97" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>5464682</v>
       </c>
-      <c r="F97" s="31"/>
+      <c r="F97" s="28"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>96</v>
       </c>
       <c r="B98" s="1">
         <f t="shared" si="13"/>
-        <v>805</v>
+        <v>1023</v>
       </c>
       <c r="C98" s="1">
         <f t="shared" si="14"/>
-        <v>442</v>
+        <v>613</v>
       </c>
       <c r="D98" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>196066</v>
       </c>
       <c r="E98" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>5660748</v>
       </c>
-      <c r="F98" s="31"/>
+      <c r="F98" s="28"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>97</v>
       </c>
       <c r="B99" s="1">
         <f t="shared" si="13"/>
-        <v>812</v>
+        <v>1034</v>
       </c>
       <c r="C99" s="1">
         <f t="shared" si="14"/>
-        <v>446</v>
+        <v>620</v>
       </c>
       <c r="D99" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>201947</v>
       </c>
       <c r="E99" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>5862695</v>
       </c>
-      <c r="F99" s="31"/>
+      <c r="F99" s="28"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>98</v>
       </c>
       <c r="B100" s="1">
         <f t="shared" si="13"/>
-        <v>819</v>
+        <v>1045</v>
       </c>
       <c r="C100" s="1">
         <f t="shared" si="14"/>
-        <v>450</v>
+        <v>627</v>
       </c>
       <c r="D100" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>208005</v>
       </c>
       <c r="E100" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>6070700</v>
       </c>
-      <c r="F100" s="31"/>
+      <c r="F100" s="28"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>99</v>
       </c>
       <c r="B101" s="1">
         <f t="shared" si="13"/>
-        <v>826</v>
+        <v>1056</v>
       </c>
       <c r="C101" s="1">
         <f t="shared" si="14"/>
-        <v>454</v>
+        <v>634</v>
       </c>
       <c r="D101" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="15"/>
         <v>214245</v>
       </c>
       <c r="E101" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>6284945</v>
       </c>
-      <c r="F101" s="31"/>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" s="1">
-        <f t="shared" si="15"/>
-        <v>100</v>
-      </c>
-      <c r="B102" s="1">
-        <f t="shared" si="13"/>
-        <v>833</v>
-      </c>
-      <c r="C102" s="1">
-        <f t="shared" si="14"/>
-        <v>458</v>
-      </c>
-      <c r="D102" s="1">
-        <f t="shared" si="11"/>
-        <v>220672</v>
-      </c>
-      <c r="E102" s="1">
-        <f t="shared" si="16"/>
-        <v>6505617</v>
-      </c>
+      <c r="F101" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3607,24 +3585,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="24" x14ac:dyDescent="0.4">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="27"/>
+      <c r="B1" s="30"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="29"/>
+      <c r="B3" s="32"/>
       <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="29"/>
+      <c r="F3" s="32"/>
       <c r="G3" s="17" t="s">
         <v>8</v>
       </c>
@@ -3640,10 +3618,10 @@
       <c r="K3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="28" t="s">
+      <c r="M3" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="29"/>
+      <c r="N3" s="32"/>
       <c r="O3" s="17" t="s">
         <v>8</v>
       </c>
@@ -3653,10 +3631,10 @@
       <c r="Q3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S3" s="28" t="s">
+      <c r="S3" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="29"/>
+      <c r="T3" s="32"/>
       <c r="U3" s="17" t="s">
         <v>8</v>
       </c>

</xml_diff>